<commit_message>
docs(account): Idempotency-Key 헤더·계좌 동시성 정합성 NFR 반영 (#5)
</commit_message>
<xml_diff>
--- a/docs/smart-spec.xlsx
+++ b/docs/smart-spec.xlsx
@@ -13,7 +13,7 @@
     <sheet name="트래픽 추정" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'요구사항'!$A$1:$G$70</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'요구사항'!$A$1:$G$71</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'API 목록'!$A$30:$H$47</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'API 상세'!$A$1:$G$163</definedName>
   </definedNames>
@@ -573,7 +573,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G70"/>
+  <dimension ref="A1:G71"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -2991,8 +2991,45 @@
       </c>
       <c r="G70" s="3" t="inlineStr"/>
     </row>
+    <row r="71">
+      <c r="A71" s="2" t="inlineStr">
+        <is>
+          <t>NFR-043</t>
+        </is>
+      </c>
+      <c r="B71" s="2" t="inlineStr">
+        <is>
+          <t>비기능</t>
+        </is>
+      </c>
+      <c r="C71" s="2" t="inlineStr">
+        <is>
+          <t>테스트</t>
+        </is>
+      </c>
+      <c r="D71" s="2" t="inlineStr">
+        <is>
+          <t>계좌 동시성 정합성</t>
+        </is>
+      </c>
+      <c r="E71" s="2" t="inlineStr">
+        <is>
+          <t>동시 계좌 개설(같은/다른 Idempotency-Key), 동시 대표 계좌 변경 후 확인: 대표 계좌 항상 1개, 멱등키 재사용 시 신규 계좌 미생성. 실제 PostgreSQL(Testcontainers)로 검증(목·가짜 DB 사용 안 함)</t>
+        </is>
+      </c>
+      <c r="F71" s="2" t="inlineStr">
+        <is>
+          <t>MVP</t>
+        </is>
+      </c>
+      <c r="G71" s="2" t="inlineStr">
+        <is>
+          <t>E-03, E-05</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:G70"/>
+  <autoFilter ref="A1:G71"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -3654,7 +3691,7 @@
       </c>
       <c r="H33" s="2" t="inlineStr">
         <is>
-          <t>첫 계좌면 대표</t>
+          <t>첫 계좌면 대표. Idempotency-Key 헤더 필수 — 같은 키 재요청 시 새 계좌를 만들지 않고 기존 계좌를 반환</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(account): 가상계좌 개설·대표 계좌 (#5) (#6)
* feat(account): 계좌 테이블 마이그레이션 (#5)

* feat(account): Account 엔티티·리포지토리 (#5)

* feat(account): 회원 행 잠금 조회 추가 (#5)

* feat(account): 계좌 개설 API — 멱등키·회원 행 잠금 (#5)

* feat(account): 대표 계좌 변경 API — 회원 행 잠금 공유 (#5)

* test(account): 계좌 개설·대표 변경 통합 테스트 — 동시성 3종 포함 (#5)

* docs(account): Idempotency-Key 헤더·계좌 동시성 정합성 NFR 반영 (#5)

* fix(account): 코덱스 리뷰 반영 — 응답 필드 누락, 명세 멱등키 헤더 누락 (#5)
</commit_message>
<xml_diff>
--- a/docs/smart-spec.xlsx
+++ b/docs/smart-spec.xlsx
@@ -13,9 +13,9 @@
     <sheet name="트래픽 추정" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'요구사항'!$A$1:$G$70</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'요구사항'!$A$1:$G$71</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'API 목록'!$A$30:$H$47</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'API 상세'!$A$1:$G$163</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'API 상세'!$A$1:$G$164</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -573,7 +573,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G70"/>
+  <dimension ref="A1:G71"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -2991,8 +2991,45 @@
       </c>
       <c r="G70" s="3" t="inlineStr"/>
     </row>
+    <row r="71">
+      <c r="A71" s="2" t="inlineStr">
+        <is>
+          <t>NFR-043</t>
+        </is>
+      </c>
+      <c r="B71" s="2" t="inlineStr">
+        <is>
+          <t>비기능</t>
+        </is>
+      </c>
+      <c r="C71" s="2" t="inlineStr">
+        <is>
+          <t>테스트</t>
+        </is>
+      </c>
+      <c r="D71" s="2" t="inlineStr">
+        <is>
+          <t>계좌 동시성 정합성</t>
+        </is>
+      </c>
+      <c r="E71" s="2" t="inlineStr">
+        <is>
+          <t>동시 계좌 개설(같은/다른 Idempotency-Key), 동시 대표 계좌 변경 후 확인: 대표 계좌 항상 1개, 멱등키 재사용 시 신규 계좌 미생성. 실제 PostgreSQL(Testcontainers)로 검증(목·가짜 DB 사용 안 함)</t>
+        </is>
+      </c>
+      <c r="F71" s="2" t="inlineStr">
+        <is>
+          <t>MVP</t>
+        </is>
+      </c>
+      <c r="G71" s="2" t="inlineStr">
+        <is>
+          <t>E-03, E-05</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:G70"/>
+  <autoFilter ref="A1:G71"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -3654,7 +3691,7 @@
       </c>
       <c r="H33" s="2" t="inlineStr">
         <is>
-          <t>첫 계좌면 대표</t>
+          <t>첫 계좌면 대표. Idempotency-Key 헤더 필수 — 같은 키 재요청 시 새 계좌를 만들지 않고 기존 계좌를 반환</t>
         </is>
       </c>
     </row>
@@ -4264,7 +4301,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G163"/>
+  <dimension ref="A1:G164"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -4667,17 +4704,17 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>응답</t>
+          <t>요청</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>data.accountId</t>
+          <t>Header Idempotency-Key</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>Long</t>
+          <t>String</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
@@ -4687,12 +4724,12 @@
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>계좌 ID</t>
+          <t>재시도 판별용 클라이언트 생성 키(UUID)</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>3f2504e0-4f89-4...</t>
         </is>
       </c>
     </row>
@@ -4709,12 +4746,12 @@
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>data.accountNumber</t>
+          <t>data.accountId</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>String</t>
+          <t>Long</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
@@ -4724,12 +4761,12 @@
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>12자리 자동 발급</t>
+          <t>계좌 ID</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>123456789012</t>
+          <t>10</t>
         </is>
       </c>
     </row>
@@ -4746,12 +4783,12 @@
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>data.balance</t>
+          <t>data.accountNumber</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>Long</t>
+          <t>String</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
@@ -4761,12 +4798,12 @@
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>잔액(원)</t>
+          <t>12자리 자동 발급</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>123456789012</t>
         </is>
       </c>
     </row>
@@ -4783,12 +4820,12 @@
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>data.primary</t>
+          <t>data.balance</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>Boolean</t>
+          <t>Long</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
@@ -4798,12 +4835,12 @@
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>대표 계좌 여부(첫 계좌면 true)</t>
+          <t>잔액(원)</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>true</t>
+          <t>0</t>
         </is>
       </c>
     </row>
@@ -4815,59 +4852,59 @@
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>에러</t>
+          <t>응답</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>AUTH_INVALID</t>
-        </is>
-      </c>
-      <c r="D16" s="2" t="inlineStr"/>
-      <c r="E16" s="2" t="inlineStr"/>
+          <t>data.primary</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>Boolean</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>JWT 없음·만료·위조, 로그인 실패</t>
-        </is>
-      </c>
-      <c r="G16" s="2" t="inlineStr"/>
+          <t>대표 계좌 여부(첫 계좌면 true)</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>E-04</t>
+          <t>E-03</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>요청</t>
+          <t>에러</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>Header Authorization</t>
-        </is>
-      </c>
-      <c r="D17" s="2" t="inlineStr">
-        <is>
-          <t>String</t>
-        </is>
-      </c>
-      <c r="E17" s="2" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+          <t>AUTH_INVALID</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr"/>
+      <c r="E17" s="2" t="inlineStr"/>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>Bearer {JWT}</t>
-        </is>
-      </c>
-      <c r="G17" s="2" t="inlineStr">
-        <is>
-          <t>Bearer eyJ...</t>
-        </is>
-      </c>
+          <t>JWT 없음·만료·위조, 로그인 실패</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -4877,17 +4914,17 @@
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>응답</t>
+          <t>요청</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>data.accounts[].accountId</t>
+          <t>Header Authorization</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>Long</t>
+          <t>String</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
@@ -4897,12 +4934,12 @@
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>계좌 ID</t>
+          <t>Bearer {JWT}</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>Bearer eyJ...</t>
         </is>
       </c>
     </row>
@@ -4919,12 +4956,12 @@
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>data.accounts[].accountNumber</t>
+          <t>data.accounts[].accountId</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>String</t>
+          <t>Long</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
@@ -4934,12 +4971,12 @@
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>계좌번호</t>
+          <t>계좌 ID</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>123456789012</t>
+          <t>10</t>
         </is>
       </c>
     </row>
@@ -4956,12 +4993,12 @@
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>data.accounts[].balance</t>
+          <t>data.accounts[].accountNumber</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>Long</t>
+          <t>String</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
@@ -4971,12 +5008,12 @@
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>잔액(원)</t>
+          <t>계좌번호</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>150000</t>
+          <t>123456789012</t>
         </is>
       </c>
     </row>
@@ -4993,12 +5030,12 @@
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>data.accounts[].primary</t>
+          <t>data.accounts[].balance</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>Boolean</t>
+          <t>Long</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr">
@@ -5008,12 +5045,12 @@
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>대표 계좌 여부</t>
+          <t>잔액(원)</t>
         </is>
       </c>
       <c r="G21" s="2" t="inlineStr">
         <is>
-          <t>true</t>
+          <t>150000</t>
         </is>
       </c>
     </row>
@@ -5025,59 +5062,59 @@
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>에러</t>
+          <t>응답</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>AUTH_INVALID</t>
-        </is>
-      </c>
-      <c r="D22" s="2" t="inlineStr"/>
-      <c r="E22" s="2" t="inlineStr"/>
+          <t>data.accounts[].primary</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>Boolean</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>JWT 없음·만료·위조, 로그인 실패</t>
-        </is>
-      </c>
-      <c r="G22" s="2" t="inlineStr"/>
+          <t>대표 계좌 여부</t>
+        </is>
+      </c>
+      <c r="G22" s="2" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>E-05</t>
+          <t>E-04</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>요청</t>
+          <t>에러</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>Header Authorization</t>
-        </is>
-      </c>
-      <c r="D23" s="2" t="inlineStr">
-        <is>
-          <t>String</t>
-        </is>
-      </c>
-      <c r="E23" s="2" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+          <t>AUTH_INVALID</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr"/>
+      <c r="E23" s="2" t="inlineStr"/>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>Bearer {JWT}</t>
-        </is>
-      </c>
-      <c r="G23" s="2" t="inlineStr">
-        <is>
-          <t>Bearer eyJ...</t>
-        </is>
-      </c>
+          <t>JWT 없음·만료·위조, 로그인 실패</t>
+        </is>
+      </c>
+      <c r="G23" s="2" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -5092,12 +5129,12 @@
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>Path accountId</t>
+          <t>Header Authorization</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>Long</t>
+          <t>String</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
@@ -5107,12 +5144,12 @@
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>대표로 바꿀 계좌 ID</t>
+          <t>Bearer {JWT}</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>Bearer eyJ...</t>
         </is>
       </c>
     </row>
@@ -5124,12 +5161,12 @@
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>응답</t>
+          <t>요청</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>data.accountId</t>
+          <t>Path accountId</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
@@ -5144,7 +5181,7 @@
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>계좌 ID</t>
+          <t>대표로 바꿀 계좌 ID</t>
         </is>
       </c>
       <c r="G25" s="2" t="inlineStr">
@@ -5166,12 +5203,12 @@
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>data.primary</t>
+          <t>data.accountId</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>Boolean</t>
+          <t>Long</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
@@ -5181,12 +5218,12 @@
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>true</t>
+          <t>계좌 ID</t>
         </is>
       </c>
       <c r="G26" s="2" t="inlineStr">
         <is>
-          <t>true</t>
+          <t>11</t>
         </is>
       </c>
     </row>
@@ -5198,22 +5235,34 @@
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>에러</t>
+          <t>응답</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>AUTH_INVALID</t>
-        </is>
-      </c>
-      <c r="D27" s="2" t="inlineStr"/>
-      <c r="E27" s="2" t="inlineStr"/>
+          <t>data.primary</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>Boolean</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>JWT 없음·만료·위조, 로그인 실패</t>
-        </is>
-      </c>
-      <c r="G27" s="2" t="inlineStr"/>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="G27" s="2" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -5228,14 +5277,14 @@
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>ACCOUNT_NOT_FOUND</t>
+          <t>AUTH_INVALID</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr"/>
       <c r="E28" s="2" t="inlineStr"/>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>계좌 없음</t>
+          <t>JWT 없음·만료·위조, 로그인 실패</t>
         </is>
       </c>
       <c r="G28" s="2" t="inlineStr"/>
@@ -5253,14 +5302,14 @@
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>ACCOUNT_NOT_OWNED</t>
+          <t>ACCOUNT_NOT_FOUND</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr"/>
       <c r="E29" s="2" t="inlineStr"/>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>내 계좌가 아님</t>
+          <t>계좌 없음</t>
         </is>
       </c>
       <c r="G29" s="2" t="inlineStr"/>
@@ -5268,39 +5317,27 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>E-06</t>
+          <t>E-05</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>요청</t>
+          <t>에러</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>Header Authorization</t>
-        </is>
-      </c>
-      <c r="D30" s="2" t="inlineStr">
-        <is>
-          <t>String</t>
-        </is>
-      </c>
-      <c r="E30" s="2" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+          <t>ACCOUNT_NOT_OWNED</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="inlineStr"/>
+      <c r="E30" s="2" t="inlineStr"/>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>Bearer {JWT}</t>
-        </is>
-      </c>
-      <c r="G30" s="2" t="inlineStr">
-        <is>
-          <t>Bearer eyJ...</t>
-        </is>
-      </c>
+          <t>내 계좌가 아님</t>
+        </is>
+      </c>
+      <c r="G30" s="2" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -5315,12 +5352,12 @@
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>Path accountId</t>
+          <t>Header Authorization</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>Long</t>
+          <t>String</t>
         </is>
       </c>
       <c r="E31" s="2" t="inlineStr">
@@ -5330,12 +5367,12 @@
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>충전할 계좌 ID</t>
+          <t>Bearer {JWT}</t>
         </is>
       </c>
       <c r="G31" s="2" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>Bearer eyJ...</t>
         </is>
       </c>
     </row>
@@ -5352,7 +5389,7 @@
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>amount</t>
+          <t>Path accountId</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
@@ -5367,12 +5404,12 @@
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>충전 금액(원)</t>
+          <t>충전할 계좌 ID</t>
         </is>
       </c>
       <c r="G32" s="2" t="inlineStr">
         <is>
-          <t>100000</t>
+          <t>10</t>
         </is>
       </c>
     </row>
@@ -5384,12 +5421,12 @@
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>응답</t>
+          <t>요청</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>data.accountId</t>
+          <t>amount</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
@@ -5404,12 +5441,12 @@
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
-          <t>계좌 ID</t>
+          <t>충전 금액(원)</t>
         </is>
       </c>
       <c r="G33" s="2" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>100000</t>
         </is>
       </c>
     </row>
@@ -5426,7 +5463,7 @@
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>data.balance</t>
+          <t>data.accountId</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
@@ -5441,12 +5478,12 @@
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>충전 후 잔액(원)</t>
+          <t>계좌 ID</t>
         </is>
       </c>
       <c r="G34" s="2" t="inlineStr">
         <is>
-          <t>100000</t>
+          <t>10</t>
         </is>
       </c>
     </row>
@@ -5458,22 +5495,34 @@
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>에러</t>
+          <t>응답</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>AUTH_INVALID</t>
-        </is>
-      </c>
-      <c r="D35" s="2" t="inlineStr"/>
-      <c r="E35" s="2" t="inlineStr"/>
+          <t>data.balance</t>
+        </is>
+      </c>
+      <c r="D35" s="2" t="inlineStr">
+        <is>
+          <t>Long</t>
+        </is>
+      </c>
+      <c r="E35" s="2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
-          <t>JWT 없음·만료·위조, 로그인 실패</t>
-        </is>
-      </c>
-      <c r="G35" s="2" t="inlineStr"/>
+          <t>충전 후 잔액(원)</t>
+        </is>
+      </c>
+      <c r="G35" s="2" t="inlineStr">
+        <is>
+          <t>100000</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -5488,14 +5537,14 @@
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>ACCOUNT_NOT_FOUND</t>
+          <t>AUTH_INVALID</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr"/>
       <c r="E36" s="2" t="inlineStr"/>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>계좌 없음</t>
+          <t>JWT 없음·만료·위조, 로그인 실패</t>
         </is>
       </c>
       <c r="G36" s="2" t="inlineStr"/>
@@ -5513,14 +5562,14 @@
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>ACCOUNT_NOT_OWNED</t>
+          <t>ACCOUNT_NOT_FOUND</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr"/>
       <c r="E37" s="2" t="inlineStr"/>
       <c r="F37" s="2" t="inlineStr">
         <is>
-          <t>내 계좌가 아님</t>
+          <t>계좌 없음</t>
         </is>
       </c>
       <c r="G37" s="2" t="inlineStr"/>
@@ -5528,39 +5577,27 @@
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>E-07</t>
+          <t>E-06</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>요청</t>
+          <t>에러</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>Header Authorization</t>
-        </is>
-      </c>
-      <c r="D38" s="2" t="inlineStr">
-        <is>
-          <t>String</t>
-        </is>
-      </c>
-      <c r="E38" s="2" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+          <t>ACCOUNT_NOT_OWNED</t>
+        </is>
+      </c>
+      <c r="D38" s="2" t="inlineStr"/>
+      <c r="E38" s="2" t="inlineStr"/>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>Bearer {JWT}</t>
-        </is>
-      </c>
-      <c r="G38" s="2" t="inlineStr">
-        <is>
-          <t>Bearer eyJ...</t>
-        </is>
-      </c>
+          <t>내 계좌가 아님</t>
+        </is>
+      </c>
+      <c r="G38" s="2" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -5575,7 +5612,7 @@
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t>alias</t>
+          <t>Header Authorization</t>
         </is>
       </c>
       <c r="D39" s="2" t="inlineStr">
@@ -5590,12 +5627,12 @@
       </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
-          <t>별칭</t>
+          <t>Bearer {JWT}</t>
         </is>
       </c>
       <c r="G39" s="2" t="inlineStr">
         <is>
-          <t>엄마</t>
+          <t>Bearer eyJ...</t>
         </is>
       </c>
     </row>
@@ -5612,7 +5649,7 @@
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>accountNumber</t>
+          <t>alias</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
@@ -5627,12 +5664,12 @@
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>상대 계좌번호</t>
+          <t>별칭</t>
         </is>
       </c>
       <c r="G40" s="2" t="inlineStr">
         <is>
-          <t>123456789012</t>
+          <t>엄마</t>
         </is>
       </c>
     </row>
@@ -5644,17 +5681,17 @@
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>응답</t>
+          <t>요청</t>
         </is>
       </c>
       <c r="C41" s="2" t="inlineStr">
         <is>
-          <t>data.aliasId</t>
+          <t>accountNumber</t>
         </is>
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
-          <t>Long</t>
+          <t>String</t>
         </is>
       </c>
       <c r="E41" s="2" t="inlineStr">
@@ -5664,12 +5701,12 @@
       </c>
       <c r="F41" s="2" t="inlineStr">
         <is>
-          <t>별칭 ID</t>
+          <t>상대 계좌번호</t>
         </is>
       </c>
       <c r="G41" s="2" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>123456789012</t>
         </is>
       </c>
     </row>
@@ -5686,12 +5723,12 @@
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>data.alias</t>
+          <t>data.aliasId</t>
         </is>
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>String</t>
+          <t>Long</t>
         </is>
       </c>
       <c r="E42" s="2" t="inlineStr">
@@ -5701,12 +5738,12 @@
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
-          <t>별칭</t>
+          <t>별칭 ID</t>
         </is>
       </c>
       <c r="G42" s="2" t="inlineStr">
         <is>
-          <t>엄마</t>
+          <t>3</t>
         </is>
       </c>
     </row>
@@ -5723,7 +5760,7 @@
       </c>
       <c r="C43" s="2" t="inlineStr">
         <is>
-          <t>data.accountNumber</t>
+          <t>data.alias</t>
         </is>
       </c>
       <c r="D43" s="2" t="inlineStr">
@@ -5738,12 +5775,12 @@
       </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
-          <t>계좌번호</t>
+          <t>별칭</t>
         </is>
       </c>
       <c r="G43" s="2" t="inlineStr">
         <is>
-          <t>123456789012</t>
+          <t>엄마</t>
         </is>
       </c>
     </row>
@@ -5760,7 +5797,7 @@
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>data.ownerName</t>
+          <t>data.accountNumber</t>
         </is>
       </c>
       <c r="D44" s="2" t="inlineStr">
@@ -5775,12 +5812,12 @@
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
-          <t>예금주 이름</t>
+          <t>계좌번호</t>
         </is>
       </c>
       <c r="G44" s="2" t="inlineStr">
         <is>
-          <t>김영희</t>
+          <t>123456789012</t>
         </is>
       </c>
     </row>
@@ -5792,22 +5829,34 @@
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>에러</t>
+          <t>응답</t>
         </is>
       </c>
       <c r="C45" s="2" t="inlineStr">
         <is>
-          <t>AUTH_INVALID</t>
-        </is>
-      </c>
-      <c r="D45" s="2" t="inlineStr"/>
-      <c r="E45" s="2" t="inlineStr"/>
+          <t>data.ownerName</t>
+        </is>
+      </c>
+      <c r="D45" s="2" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="E45" s="2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="F45" s="2" t="inlineStr">
         <is>
-          <t>JWT 없음·만료·위조, 로그인 실패</t>
-        </is>
-      </c>
-      <c r="G45" s="2" t="inlineStr"/>
+          <t>예금주 이름</t>
+        </is>
+      </c>
+      <c r="G45" s="2" t="inlineStr">
+        <is>
+          <t>김영희</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
@@ -5822,14 +5871,14 @@
       </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t>ACCOUNT_NOT_FOUND</t>
+          <t>AUTH_INVALID</t>
         </is>
       </c>
       <c r="D46" s="2" t="inlineStr"/>
       <c r="E46" s="2" t="inlineStr"/>
       <c r="F46" s="2" t="inlineStr">
         <is>
-          <t>계좌 없음</t>
+          <t>JWT 없음·만료·위조, 로그인 실패</t>
         </is>
       </c>
       <c r="G46" s="2" t="inlineStr"/>
@@ -5837,39 +5886,27 @@
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>E-08</t>
+          <t>E-07</t>
         </is>
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
-          <t>요청</t>
+          <t>에러</t>
         </is>
       </c>
       <c r="C47" s="2" t="inlineStr">
         <is>
-          <t>Header Authorization</t>
-        </is>
-      </c>
-      <c r="D47" s="2" t="inlineStr">
-        <is>
-          <t>String</t>
-        </is>
-      </c>
-      <c r="E47" s="2" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+          <t>ACCOUNT_NOT_FOUND</t>
+        </is>
+      </c>
+      <c r="D47" s="2" t="inlineStr"/>
+      <c r="E47" s="2" t="inlineStr"/>
       <c r="F47" s="2" t="inlineStr">
         <is>
-          <t>Bearer {JWT}</t>
-        </is>
-      </c>
-      <c r="G47" s="2" t="inlineStr">
-        <is>
-          <t>Bearer eyJ...</t>
-        </is>
-      </c>
+          <t>계좌 없음</t>
+        </is>
+      </c>
+      <c r="G47" s="2" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
@@ -5879,17 +5916,17 @@
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>응답</t>
+          <t>요청</t>
         </is>
       </c>
       <c r="C48" s="2" t="inlineStr">
         <is>
-          <t>data.aliases[].aliasId</t>
+          <t>Header Authorization</t>
         </is>
       </c>
       <c r="D48" s="2" t="inlineStr">
         <is>
-          <t>Long</t>
+          <t>String</t>
         </is>
       </c>
       <c r="E48" s="2" t="inlineStr">
@@ -5899,12 +5936,12 @@
       </c>
       <c r="F48" s="2" t="inlineStr">
         <is>
-          <t>별칭 ID</t>
+          <t>Bearer {JWT}</t>
         </is>
       </c>
       <c r="G48" s="2" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>Bearer eyJ...</t>
         </is>
       </c>
     </row>
@@ -5921,12 +5958,12 @@
       </c>
       <c r="C49" s="2" t="inlineStr">
         <is>
-          <t>data.aliases[].alias</t>
+          <t>data.aliases[].aliasId</t>
         </is>
       </c>
       <c r="D49" s="2" t="inlineStr">
         <is>
-          <t>String</t>
+          <t>Long</t>
         </is>
       </c>
       <c r="E49" s="2" t="inlineStr">
@@ -5936,12 +5973,12 @@
       </c>
       <c r="F49" s="2" t="inlineStr">
         <is>
-          <t>별칭</t>
+          <t>별칭 ID</t>
         </is>
       </c>
       <c r="G49" s="2" t="inlineStr">
         <is>
-          <t>엄마</t>
+          <t>3</t>
         </is>
       </c>
     </row>
@@ -5958,7 +5995,7 @@
       </c>
       <c r="C50" s="2" t="inlineStr">
         <is>
-          <t>data.aliases[].accountNumber</t>
+          <t>data.aliases[].alias</t>
         </is>
       </c>
       <c r="D50" s="2" t="inlineStr">
@@ -5973,12 +6010,12 @@
       </c>
       <c r="F50" s="2" t="inlineStr">
         <is>
-          <t>계좌번호</t>
+          <t>별칭</t>
         </is>
       </c>
       <c r="G50" s="2" t="inlineStr">
         <is>
-          <t>123456789012</t>
+          <t>엄마</t>
         </is>
       </c>
     </row>
@@ -5995,7 +6032,7 @@
       </c>
       <c r="C51" s="2" t="inlineStr">
         <is>
-          <t>data.aliases[].ownerName</t>
+          <t>data.aliases[].accountNumber</t>
         </is>
       </c>
       <c r="D51" s="2" t="inlineStr">
@@ -6010,12 +6047,12 @@
       </c>
       <c r="F51" s="2" t="inlineStr">
         <is>
-          <t>예금주 이름</t>
+          <t>계좌번호</t>
         </is>
       </c>
       <c r="G51" s="2" t="inlineStr">
         <is>
-          <t>김영희</t>
+          <t>123456789012</t>
         </is>
       </c>
     </row>
@@ -6027,59 +6064,59 @@
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>에러</t>
+          <t>응답</t>
         </is>
       </c>
       <c r="C52" s="2" t="inlineStr">
         <is>
-          <t>AUTH_INVALID</t>
-        </is>
-      </c>
-      <c r="D52" s="2" t="inlineStr"/>
-      <c r="E52" s="2" t="inlineStr"/>
+          <t>data.aliases[].ownerName</t>
+        </is>
+      </c>
+      <c r="D52" s="2" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="E52" s="2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="F52" s="2" t="inlineStr">
         <is>
-          <t>JWT 없음·만료·위조, 로그인 실패</t>
-        </is>
-      </c>
-      <c r="G52" s="2" t="inlineStr"/>
+          <t>예금주 이름</t>
+        </is>
+      </c>
+      <c r="G52" s="2" t="inlineStr">
+        <is>
+          <t>김영희</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
         <is>
-          <t>E-09</t>
+          <t>E-08</t>
         </is>
       </c>
       <c r="B53" s="2" t="inlineStr">
         <is>
-          <t>요청</t>
+          <t>에러</t>
         </is>
       </c>
       <c r="C53" s="2" t="inlineStr">
         <is>
-          <t>Header Authorization</t>
-        </is>
-      </c>
-      <c r="D53" s="2" t="inlineStr">
-        <is>
-          <t>String</t>
-        </is>
-      </c>
-      <c r="E53" s="2" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+          <t>AUTH_INVALID</t>
+        </is>
+      </c>
+      <c r="D53" s="2" t="inlineStr"/>
+      <c r="E53" s="2" t="inlineStr"/>
       <c r="F53" s="2" t="inlineStr">
         <is>
-          <t>Bearer {JWT}</t>
-        </is>
-      </c>
-      <c r="G53" s="2" t="inlineStr">
-        <is>
-          <t>Bearer eyJ...</t>
-        </is>
-      </c>
+          <t>JWT 없음·만료·위조, 로그인 실패</t>
+        </is>
+      </c>
+      <c r="G53" s="2" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
@@ -6094,27 +6131,27 @@
       </c>
       <c r="C54" s="2" t="inlineStr">
         <is>
-          <t>Query cursor</t>
+          <t>Header Authorization</t>
         </is>
       </c>
       <c r="D54" s="2" t="inlineStr">
         <is>
-          <t>Long</t>
+          <t>String</t>
         </is>
       </c>
       <c r="E54" s="2" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="F54" s="2" t="inlineStr">
         <is>
-          <t>이전 응답의 nextCursor. 없으면 최신부터</t>
+          <t>Bearer {JWT}</t>
         </is>
       </c>
       <c r="G54" s="2" t="inlineStr">
         <is>
-          <t>1025</t>
+          <t>Bearer eyJ...</t>
         </is>
       </c>
     </row>
@@ -6131,12 +6168,12 @@
       </c>
       <c r="C55" s="2" t="inlineStr">
         <is>
-          <t>Query size</t>
+          <t>Query cursor</t>
         </is>
       </c>
       <c r="D55" s="2" t="inlineStr">
         <is>
-          <t>Integer</t>
+          <t>Long</t>
         </is>
       </c>
       <c r="E55" s="2" t="inlineStr">
@@ -6146,12 +6183,12 @@
       </c>
       <c r="F55" s="2" t="inlineStr">
         <is>
-          <t>묶음 크기(기본 20)</t>
+          <t>이전 응답의 nextCursor. 없으면 최신부터</t>
         </is>
       </c>
       <c r="G55" s="2" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>1025</t>
         </is>
       </c>
     </row>
@@ -6163,32 +6200,32 @@
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
-          <t>응답</t>
+          <t>요청</t>
         </is>
       </c>
       <c r="C56" s="2" t="inlineStr">
         <is>
-          <t>data.items[].transferId</t>
+          <t>Query size</t>
         </is>
       </c>
       <c r="D56" s="2" t="inlineStr">
         <is>
-          <t>Long</t>
+          <t>Integer</t>
         </is>
       </c>
       <c r="E56" s="2" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="F56" s="2" t="inlineStr">
         <is>
-          <t>송금 ID</t>
+          <t>묶음 크기(기본 20)</t>
         </is>
       </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>1024</t>
+          <t>20</t>
         </is>
       </c>
     </row>
@@ -6205,12 +6242,12 @@
       </c>
       <c r="C57" s="2" t="inlineStr">
         <is>
-          <t>data.items[].direction</t>
+          <t>data.items[].transferId</t>
         </is>
       </c>
       <c r="D57" s="2" t="inlineStr">
         <is>
-          <t>String</t>
+          <t>Long</t>
         </is>
       </c>
       <c r="E57" s="2" t="inlineStr">
@@ -6220,12 +6257,12 @@
       </c>
       <c r="F57" s="2" t="inlineStr">
         <is>
-          <t>SENT / RECEIVED</t>
+          <t>송금 ID</t>
         </is>
       </c>
       <c r="G57" s="2" t="inlineStr">
         <is>
-          <t>SENT</t>
+          <t>1024</t>
         </is>
       </c>
     </row>
@@ -6242,7 +6279,7 @@
       </c>
       <c r="C58" s="2" t="inlineStr">
         <is>
-          <t>data.items[].counterpartName</t>
+          <t>data.items[].direction</t>
         </is>
       </c>
       <c r="D58" s="2" t="inlineStr">
@@ -6257,12 +6294,12 @@
       </c>
       <c r="F58" s="2" t="inlineStr">
         <is>
-          <t>상대 이름</t>
+          <t>SENT / RECEIVED</t>
         </is>
       </c>
       <c r="G58" s="2" t="inlineStr">
         <is>
-          <t>김영희</t>
+          <t>SENT</t>
         </is>
       </c>
     </row>
@@ -6279,7 +6316,7 @@
       </c>
       <c r="C59" s="2" t="inlineStr">
         <is>
-          <t>data.items[].counterpartAccountNumber</t>
+          <t>data.items[].counterpartName</t>
         </is>
       </c>
       <c r="D59" s="2" t="inlineStr">
@@ -6294,12 +6331,12 @@
       </c>
       <c r="F59" s="2" t="inlineStr">
         <is>
-          <t>상대 계좌</t>
+          <t>상대 이름</t>
         </is>
       </c>
       <c r="G59" s="2" t="inlineStr">
         <is>
-          <t>123456789012</t>
+          <t>김영희</t>
         </is>
       </c>
     </row>
@@ -6316,12 +6353,12 @@
       </c>
       <c r="C60" s="2" t="inlineStr">
         <is>
-          <t>data.items[].amount</t>
+          <t>data.items[].counterpartAccountNumber</t>
         </is>
       </c>
       <c r="D60" s="2" t="inlineStr">
         <is>
-          <t>Long</t>
+          <t>String</t>
         </is>
       </c>
       <c r="E60" s="2" t="inlineStr">
@@ -6331,12 +6368,12 @@
       </c>
       <c r="F60" s="2" t="inlineStr">
         <is>
-          <t>금액(원)</t>
+          <t>상대 계좌</t>
         </is>
       </c>
       <c r="G60" s="2" t="inlineStr">
         <is>
-          <t>10000</t>
+          <t>123456789012</t>
         </is>
       </c>
     </row>
@@ -6353,12 +6390,12 @@
       </c>
       <c r="C61" s="2" t="inlineStr">
         <is>
-          <t>data.items[].createdAt</t>
+          <t>data.items[].amount</t>
         </is>
       </c>
       <c r="D61" s="2" t="inlineStr">
         <is>
-          <t>String</t>
+          <t>Long</t>
         </is>
       </c>
       <c r="E61" s="2" t="inlineStr">
@@ -6368,12 +6405,12 @@
       </c>
       <c r="F61" s="2" t="inlineStr">
         <is>
-          <t>시각(ISO-8601)</t>
+          <t>금액(원)</t>
         </is>
       </c>
       <c r="G61" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T10:01:00+09:00</t>
+          <t>10000</t>
         </is>
       </c>
     </row>
@@ -6390,27 +6427,27 @@
       </c>
       <c r="C62" s="2" t="inlineStr">
         <is>
-          <t>data.nextCursor</t>
+          <t>data.items[].createdAt</t>
         </is>
       </c>
       <c r="D62" s="2" t="inlineStr">
         <is>
-          <t>Long</t>
+          <t>String</t>
         </is>
       </c>
       <c r="E62" s="2" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="F62" s="2" t="inlineStr">
         <is>
-          <t>다음 요청의 cursor(마지막 transferId). 없으면 null</t>
+          <t>시각(ISO-8601)</t>
         </is>
       </c>
       <c r="G62" s="2" t="inlineStr">
         <is>
-          <t>1005</t>
+          <t>2026-09-27T10:01:00+09:00</t>
         </is>
       </c>
     </row>
@@ -6427,27 +6464,27 @@
       </c>
       <c r="C63" s="2" t="inlineStr">
         <is>
-          <t>data.hasNext</t>
+          <t>data.nextCursor</t>
         </is>
       </c>
       <c r="D63" s="2" t="inlineStr">
         <is>
-          <t>Boolean</t>
+          <t>Long</t>
         </is>
       </c>
       <c r="E63" s="2" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="F63" s="2" t="inlineStr">
         <is>
-          <t>다음 묶음 존재 여부</t>
+          <t>다음 요청의 cursor(마지막 transferId). 없으면 null</t>
         </is>
       </c>
       <c r="G63" s="2" t="inlineStr">
         <is>
-          <t>true</t>
+          <t>1005</t>
         </is>
       </c>
     </row>
@@ -6459,59 +6496,59 @@
       </c>
       <c r="B64" s="2" t="inlineStr">
         <is>
-          <t>에러</t>
+          <t>응답</t>
         </is>
       </c>
       <c r="C64" s="2" t="inlineStr">
         <is>
-          <t>AUTH_INVALID</t>
-        </is>
-      </c>
-      <c r="D64" s="2" t="inlineStr"/>
-      <c r="E64" s="2" t="inlineStr"/>
+          <t>data.hasNext</t>
+        </is>
+      </c>
+      <c r="D64" s="2" t="inlineStr">
+        <is>
+          <t>Boolean</t>
+        </is>
+      </c>
+      <c r="E64" s="2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="F64" s="2" t="inlineStr">
         <is>
-          <t>JWT 없음·만료·위조, 로그인 실패</t>
-        </is>
-      </c>
-      <c r="G64" s="2" t="inlineStr"/>
+          <t>다음 묶음 존재 여부</t>
+        </is>
+      </c>
+      <c r="G64" s="2" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
         <is>
-          <t>E-10</t>
+          <t>E-09</t>
         </is>
       </c>
       <c r="B65" s="2" t="inlineStr">
         <is>
-          <t>요청</t>
+          <t>에러</t>
         </is>
       </c>
       <c r="C65" s="2" t="inlineStr">
         <is>
-          <t>Header Authorization</t>
-        </is>
-      </c>
-      <c r="D65" s="2" t="inlineStr">
-        <is>
-          <t>String</t>
-        </is>
-      </c>
-      <c r="E65" s="2" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+          <t>AUTH_INVALID</t>
+        </is>
+      </c>
+      <c r="D65" s="2" t="inlineStr"/>
+      <c r="E65" s="2" t="inlineStr"/>
       <c r="F65" s="2" t="inlineStr">
         <is>
-          <t>Bearer {JWT}</t>
-        </is>
-      </c>
-      <c r="G65" s="2" t="inlineStr">
-        <is>
-          <t>Bearer eyJ...</t>
-        </is>
-      </c>
+          <t>JWT 없음·만료·위조, 로그인 실패</t>
+        </is>
+      </c>
+      <c r="G65" s="2" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
@@ -6521,12 +6558,12 @@
       </c>
       <c r="B66" s="2" t="inlineStr">
         <is>
-          <t>응답</t>
+          <t>요청</t>
         </is>
       </c>
       <c r="C66" s="2" t="inlineStr">
         <is>
-          <t>data.threadId</t>
+          <t>Header Authorization</t>
         </is>
       </c>
       <c r="D66" s="2" t="inlineStr">
@@ -6541,12 +6578,12 @@
       </c>
       <c r="F66" s="2" t="inlineStr">
         <is>
-          <t>Spring이 발급, 사용자와 묶어 저장</t>
+          <t>Bearer {JWT}</t>
         </is>
       </c>
       <c r="G66" s="2" t="inlineStr">
         <is>
-          <t>th_5b21...</t>
+          <t>Bearer eyJ...</t>
         </is>
       </c>
     </row>
@@ -6558,59 +6595,59 @@
       </c>
       <c r="B67" s="2" t="inlineStr">
         <is>
-          <t>에러</t>
+          <t>응답</t>
         </is>
       </c>
       <c r="C67" s="2" t="inlineStr">
         <is>
-          <t>AUTH_INVALID</t>
-        </is>
-      </c>
-      <c r="D67" s="2" t="inlineStr"/>
-      <c r="E67" s="2" t="inlineStr"/>
+          <t>data.threadId</t>
+        </is>
+      </c>
+      <c r="D67" s="2" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="E67" s="2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="F67" s="2" t="inlineStr">
         <is>
-          <t>JWT 없음·만료·위조, 로그인 실패</t>
-        </is>
-      </c>
-      <c r="G67" s="2" t="inlineStr"/>
+          <t>Spring이 발급, 사용자와 묶어 저장</t>
+        </is>
+      </c>
+      <c r="G67" s="2" t="inlineStr">
+        <is>
+          <t>th_5b21...</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>E-11</t>
+          <t>E-10</t>
         </is>
       </c>
       <c r="B68" s="2" t="inlineStr">
         <is>
-          <t>요청</t>
+          <t>에러</t>
         </is>
       </c>
       <c r="C68" s="2" t="inlineStr">
         <is>
-          <t>Header Authorization</t>
-        </is>
-      </c>
-      <c r="D68" s="2" t="inlineStr">
-        <is>
-          <t>String</t>
-        </is>
-      </c>
-      <c r="E68" s="2" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+          <t>AUTH_INVALID</t>
+        </is>
+      </c>
+      <c r="D68" s="2" t="inlineStr"/>
+      <c r="E68" s="2" t="inlineStr"/>
       <c r="F68" s="2" t="inlineStr">
         <is>
-          <t>Bearer {JWT}</t>
-        </is>
-      </c>
-      <c r="G68" s="2" t="inlineStr">
-        <is>
-          <t>Bearer eyJ...</t>
-        </is>
-      </c>
+          <t>JWT 없음·만료·위조, 로그인 실패</t>
+        </is>
+      </c>
+      <c r="G68" s="2" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
@@ -6625,7 +6662,7 @@
       </c>
       <c r="C69" s="2" t="inlineStr">
         <is>
-          <t>Path threadId</t>
+          <t>Header Authorization</t>
         </is>
       </c>
       <c r="D69" s="2" t="inlineStr">
@@ -6640,12 +6677,12 @@
       </c>
       <c r="F69" s="2" t="inlineStr">
         <is>
-          <t>대화 ID</t>
+          <t>Bearer {JWT}</t>
         </is>
       </c>
       <c r="G69" s="2" t="inlineStr">
         <is>
-          <t>th_5b21...</t>
+          <t>Bearer eyJ...</t>
         </is>
       </c>
     </row>
@@ -6662,7 +6699,7 @@
       </c>
       <c r="C70" s="2" t="inlineStr">
         <is>
-          <t>message</t>
+          <t>Path threadId</t>
         </is>
       </c>
       <c r="D70" s="2" t="inlineStr">
@@ -6677,12 +6714,12 @@
       </c>
       <c r="F70" s="2" t="inlineStr">
         <is>
-          <t>사용자 메시지</t>
+          <t>대화 ID</t>
         </is>
       </c>
       <c r="G70" s="2" t="inlineStr">
         <is>
-          <t>엄마한테 1만원 보내줘</t>
+          <t>th_5b21...</t>
         </is>
       </c>
     </row>
@@ -6694,12 +6731,12 @@
       </c>
       <c r="B71" s="2" t="inlineStr">
         <is>
-          <t>응답</t>
+          <t>요청</t>
         </is>
       </c>
       <c r="C71" s="2" t="inlineStr">
         <is>
-          <t>data.reply</t>
+          <t>message</t>
         </is>
       </c>
       <c r="D71" s="2" t="inlineStr">
@@ -6714,12 +6751,12 @@
       </c>
       <c r="F71" s="2" t="inlineStr">
         <is>
-          <t>요약 답변. 가드에 걸리면 고정 문장</t>
+          <t>사용자 메시지</t>
         </is>
       </c>
       <c r="G71" s="2" t="inlineStr">
         <is>
-          <t>삼성전자 2분기 영업이익은 ...</t>
+          <t>엄마한테 1만원 보내줘</t>
         </is>
       </c>
     </row>
@@ -6736,7 +6773,7 @@
       </c>
       <c r="C72" s="2" t="inlineStr">
         <is>
-          <t>data.guard</t>
+          <t>data.reply</t>
         </is>
       </c>
       <c r="D72" s="2" t="inlineStr">
@@ -6751,12 +6788,12 @@
       </c>
       <c r="F72" s="2" t="inlineStr">
         <is>
-          <t>판정 코드: PASS / INJECTION / NUMBER_UNVERIFIED / ADVICE / PROMPT_LEAK</t>
+          <t>요약 답변. 가드에 걸리면 고정 문장</t>
         </is>
       </c>
       <c r="G72" s="2" t="inlineStr">
         <is>
-          <t>PASS</t>
+          <t>삼성전자 2분기 영업이익은 ...</t>
         </is>
       </c>
     </row>
@@ -6773,7 +6810,7 @@
       </c>
       <c r="C73" s="2" t="inlineStr">
         <is>
-          <t>data.transferCard.requestId</t>
+          <t>data.guard</t>
         </is>
       </c>
       <c r="D73" s="2" t="inlineStr">
@@ -6783,17 +6820,17 @@
       </c>
       <c r="E73" s="2" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="F73" s="2" t="inlineStr">
         <is>
-          <t>송금 요청ID(1회용)</t>
+          <t>판정 코드: PASS / INJECTION / NUMBER_UNVERIFIED / ADVICE / PROMPT_LEAK</t>
         </is>
       </c>
       <c r="G73" s="2" t="inlineStr">
         <is>
-          <t>tr_7f3a...</t>
+          <t>PASS</t>
         </is>
       </c>
     </row>
@@ -6810,7 +6847,7 @@
       </c>
       <c r="C74" s="2" t="inlineStr">
         <is>
-          <t>data.transferCard.recipientName</t>
+          <t>data.transferCard.requestId</t>
         </is>
       </c>
       <c r="D74" s="2" t="inlineStr">
@@ -6825,12 +6862,12 @@
       </c>
       <c r="F74" s="2" t="inlineStr">
         <is>
-          <t>수취인 이름</t>
+          <t>송금 요청ID(1회용)</t>
         </is>
       </c>
       <c r="G74" s="2" t="inlineStr">
         <is>
-          <t>김영희</t>
+          <t>tr_7f3a...</t>
         </is>
       </c>
     </row>
@@ -6847,7 +6884,7 @@
       </c>
       <c r="C75" s="2" t="inlineStr">
         <is>
-          <t>data.transferCard.recipientAccountNumber</t>
+          <t>data.transferCard.recipientName</t>
         </is>
       </c>
       <c r="D75" s="2" t="inlineStr">
@@ -6862,12 +6899,12 @@
       </c>
       <c r="F75" s="2" t="inlineStr">
         <is>
-          <t>수취인 계좌</t>
+          <t>수취인 이름</t>
         </is>
       </c>
       <c r="G75" s="2" t="inlineStr">
         <is>
-          <t>123456789012</t>
+          <t>김영희</t>
         </is>
       </c>
     </row>
@@ -6884,7 +6921,7 @@
       </c>
       <c r="C76" s="2" t="inlineStr">
         <is>
-          <t>data.transferCard.fromAccountNumber</t>
+          <t>data.transferCard.recipientAccountNumber</t>
         </is>
       </c>
       <c r="D76" s="2" t="inlineStr">
@@ -6899,12 +6936,12 @@
       </c>
       <c r="F76" s="2" t="inlineStr">
         <is>
-          <t>출금 계좌(대표 계좌)</t>
+          <t>수취인 계좌</t>
         </is>
       </c>
       <c r="G76" s="2" t="inlineStr">
         <is>
-          <t>987654321098</t>
+          <t>123456789012</t>
         </is>
       </c>
     </row>
@@ -6921,12 +6958,12 @@
       </c>
       <c r="C77" s="2" t="inlineStr">
         <is>
-          <t>data.transferCard.amount</t>
+          <t>data.transferCard.fromAccountNumber</t>
         </is>
       </c>
       <c r="D77" s="2" t="inlineStr">
         <is>
-          <t>Long</t>
+          <t>String</t>
         </is>
       </c>
       <c r="E77" s="2" t="inlineStr">
@@ -6936,12 +6973,12 @@
       </c>
       <c r="F77" s="2" t="inlineStr">
         <is>
-          <t>금액(원)</t>
+          <t>출금 계좌(대표 계좌)</t>
         </is>
       </c>
       <c r="G77" s="2" t="inlineStr">
         <is>
-          <t>10000</t>
+          <t>987654321098</t>
         </is>
       </c>
     </row>
@@ -6958,12 +6995,12 @@
       </c>
       <c r="C78" s="2" t="inlineStr">
         <is>
-          <t>data.transferCard.expiresAt</t>
+          <t>data.transferCard.amount</t>
         </is>
       </c>
       <c r="D78" s="2" t="inlineStr">
         <is>
-          <t>String</t>
+          <t>Long</t>
         </is>
       </c>
       <c r="E78" s="2" t="inlineStr">
@@ -6973,12 +7010,12 @@
       </c>
       <c r="F78" s="2" t="inlineStr">
         <is>
-          <t>만료 시각(생성 + 5분, ISO-8601)</t>
+          <t>금액(원)</t>
         </is>
       </c>
       <c r="G78" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T10:05:00+09:00</t>
+          <t>10000</t>
         </is>
       </c>
     </row>
@@ -6995,12 +7032,12 @@
       </c>
       <c r="C79" s="2" t="inlineStr">
         <is>
-          <t>data.table.columns</t>
+          <t>data.transferCard.expiresAt</t>
         </is>
       </c>
       <c r="D79" s="2" t="inlineStr">
         <is>
-          <t>String[]</t>
+          <t>String</t>
         </is>
       </c>
       <c r="E79" s="2" t="inlineStr">
@@ -7010,12 +7047,12 @@
       </c>
       <c r="F79" s="2" t="inlineStr">
         <is>
-          <t>표 머리글</t>
+          <t>만료 시각(생성 + 5분, ISO-8601)</t>
         </is>
       </c>
       <c r="G79" s="2" t="inlineStr">
         <is>
-          <t>["항목","삼성전자","SK하이닉스"]</t>
+          <t>2026-09-27T10:05:00+09:00</t>
         </is>
       </c>
     </row>
@@ -7032,12 +7069,12 @@
       </c>
       <c r="C80" s="2" t="inlineStr">
         <is>
-          <t>data.table.rows</t>
+          <t>data.table.columns</t>
         </is>
       </c>
       <c r="D80" s="2" t="inlineStr">
         <is>
-          <t>String[][]</t>
+          <t>String[]</t>
         </is>
       </c>
       <c r="E80" s="2" t="inlineStr">
@@ -7047,12 +7084,12 @@
       </c>
       <c r="F80" s="2" t="inlineStr">
         <is>
-          <t>표 행</t>
+          <t>표 머리글</t>
         </is>
       </c>
       <c r="G80" s="2" t="inlineStr">
         <is>
-          <t>[["영업이익","...","..."]]</t>
+          <t>["항목","삼성전자","SK하이닉스"]</t>
         </is>
       </c>
     </row>
@@ -7069,12 +7106,12 @@
       </c>
       <c r="C81" s="2" t="inlineStr">
         <is>
-          <t>data.table.note</t>
+          <t>data.table.rows</t>
         </is>
       </c>
       <c r="D81" s="2" t="inlineStr">
         <is>
-          <t>String</t>
+          <t>String[][]</t>
         </is>
       </c>
       <c r="E81" s="2" t="inlineStr">
@@ -7084,12 +7121,12 @@
       </c>
       <c r="F81" s="2" t="inlineStr">
         <is>
-          <t>재무제표 기준(연결/별도)·미공시 표시</t>
+          <t>표 행</t>
         </is>
       </c>
       <c r="G81" s="2" t="inlineStr">
         <is>
-          <t>연결 기준</t>
+          <t>[["영업이익","...","..."]]</t>
         </is>
       </c>
     </row>
@@ -7106,7 +7143,7 @@
       </c>
       <c r="C82" s="2" t="inlineStr">
         <is>
-          <t>data.detailId</t>
+          <t>data.table.note</t>
         </is>
       </c>
       <c r="D82" s="2" t="inlineStr">
@@ -7121,12 +7158,12 @@
       </c>
       <c r="F82" s="2" t="inlineStr">
         <is>
-          <t>상세 보기 ID(분석 답변일 때)</t>
+          <t>재무제표 기준(연결/별도)·미공시 표시</t>
         </is>
       </c>
       <c r="G82" s="2" t="inlineStr">
         <is>
-          <t>dt_91c2...</t>
+          <t>연결 기준</t>
         </is>
       </c>
     </row>
@@ -7138,22 +7175,34 @@
       </c>
       <c r="B83" s="2" t="inlineStr">
         <is>
-          <t>에러</t>
+          <t>응답</t>
         </is>
       </c>
       <c r="C83" s="2" t="inlineStr">
         <is>
-          <t>AUTH_INVALID</t>
-        </is>
-      </c>
-      <c r="D83" s="2" t="inlineStr"/>
-      <c r="E83" s="2" t="inlineStr"/>
+          <t>data.detailId</t>
+        </is>
+      </c>
+      <c r="D83" s="2" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="E83" s="2" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="F83" s="2" t="inlineStr">
         <is>
-          <t>JWT 없음·만료·위조, 로그인 실패</t>
-        </is>
-      </c>
-      <c r="G83" s="2" t="inlineStr"/>
+          <t>상세 보기 ID(분석 답변일 때)</t>
+        </is>
+      </c>
+      <c r="G83" s="2" t="inlineStr">
+        <is>
+          <t>dt_91c2...</t>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
@@ -7168,14 +7217,14 @@
       </c>
       <c r="C84" s="2" t="inlineStr">
         <is>
-          <t>THREAD_NOT_FOUND</t>
+          <t>AUTH_INVALID</t>
         </is>
       </c>
       <c r="D84" s="2" t="inlineStr"/>
       <c r="E84" s="2" t="inlineStr"/>
       <c r="F84" s="2" t="inlineStr">
         <is>
-          <t>대화 없음(또는 남의 대화)</t>
+          <t>JWT 없음·만료·위조, 로그인 실패</t>
         </is>
       </c>
       <c r="G84" s="2" t="inlineStr"/>
@@ -7193,14 +7242,14 @@
       </c>
       <c r="C85" s="2" t="inlineStr">
         <is>
-          <t>RATE_LIMITED</t>
+          <t>THREAD_NOT_FOUND</t>
         </is>
       </c>
       <c r="D85" s="2" t="inlineStr"/>
       <c r="E85" s="2" t="inlineStr"/>
       <c r="F85" s="2" t="inlineStr">
         <is>
-          <t>사용자별 채팅 호출 제한 초과</t>
+          <t>대화 없음(또는 남의 대화)</t>
         </is>
       </c>
       <c r="G85" s="2" t="inlineStr"/>
@@ -7218,14 +7267,14 @@
       </c>
       <c r="C86" s="2" t="inlineStr">
         <is>
-          <t>AI_SERVER_UNAVAILABLE</t>
+          <t>RATE_LIMITED</t>
         </is>
       </c>
       <c r="D86" s="2" t="inlineStr"/>
       <c r="E86" s="2" t="inlineStr"/>
       <c r="F86" s="2" t="inlineStr">
         <is>
-          <t>FastAPI 장애·지연 — 채팅만 실패, 송금·계좌는 정상(장애 격리)</t>
+          <t>사용자별 채팅 호출 제한 초과</t>
         </is>
       </c>
       <c r="G86" s="2" t="inlineStr"/>
@@ -7233,39 +7282,27 @@
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
         <is>
-          <t>E-12</t>
+          <t>E-11</t>
         </is>
       </c>
       <c r="B87" s="2" t="inlineStr">
         <is>
-          <t>요청</t>
+          <t>에러</t>
         </is>
       </c>
       <c r="C87" s="2" t="inlineStr">
         <is>
-          <t>Header Authorization</t>
-        </is>
-      </c>
-      <c r="D87" s="2" t="inlineStr">
-        <is>
-          <t>String</t>
-        </is>
-      </c>
-      <c r="E87" s="2" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+          <t>AI_SERVER_UNAVAILABLE</t>
+        </is>
+      </c>
+      <c r="D87" s="2" t="inlineStr"/>
+      <c r="E87" s="2" t="inlineStr"/>
       <c r="F87" s="2" t="inlineStr">
         <is>
-          <t>Bearer {JWT}</t>
-        </is>
-      </c>
-      <c r="G87" s="2" t="inlineStr">
-        <is>
-          <t>Bearer eyJ...</t>
-        </is>
-      </c>
+          <t>FastAPI 장애·지연 — 채팅만 실패, 송금·계좌는 정상(장애 격리)</t>
+        </is>
+      </c>
+      <c r="G87" s="2" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -7280,7 +7317,7 @@
       </c>
       <c r="C88" s="2" t="inlineStr">
         <is>
-          <t>Path requestId</t>
+          <t>Header Authorization</t>
         </is>
       </c>
       <c r="D88" s="2" t="inlineStr">
@@ -7295,12 +7332,12 @@
       </c>
       <c r="F88" s="2" t="inlineStr">
         <is>
-          <t>확인 카드의 요청ID</t>
+          <t>Bearer {JWT}</t>
         </is>
       </c>
       <c r="G88" s="2" t="inlineStr">
         <is>
-          <t>tr_7f3a...</t>
+          <t>Bearer eyJ...</t>
         </is>
       </c>
     </row>
@@ -7312,17 +7349,17 @@
       </c>
       <c r="B89" s="2" t="inlineStr">
         <is>
-          <t>응답</t>
+          <t>요청</t>
         </is>
       </c>
       <c r="C89" s="2" t="inlineStr">
         <is>
-          <t>data.transferId</t>
+          <t>Path requestId</t>
         </is>
       </c>
       <c r="D89" s="2" t="inlineStr">
         <is>
-          <t>Long</t>
+          <t>String</t>
         </is>
       </c>
       <c r="E89" s="2" t="inlineStr">
@@ -7332,12 +7369,12 @@
       </c>
       <c r="F89" s="2" t="inlineStr">
         <is>
-          <t>송금 ID</t>
+          <t>확인 카드의 요청ID</t>
         </is>
       </c>
       <c r="G89" s="2" t="inlineStr">
         <is>
-          <t>1026</t>
+          <t>tr_7f3a...</t>
         </is>
       </c>
     </row>
@@ -7354,12 +7391,12 @@
       </c>
       <c r="C90" s="2" t="inlineStr">
         <is>
-          <t>data.recipientName</t>
+          <t>data.transferId</t>
         </is>
       </c>
       <c r="D90" s="2" t="inlineStr">
         <is>
-          <t>String</t>
+          <t>Long</t>
         </is>
       </c>
       <c r="E90" s="2" t="inlineStr">
@@ -7369,12 +7406,12 @@
       </c>
       <c r="F90" s="2" t="inlineStr">
         <is>
-          <t>수취인 이름</t>
+          <t>송금 ID</t>
         </is>
       </c>
       <c r="G90" s="2" t="inlineStr">
         <is>
-          <t>김영희</t>
+          <t>1026</t>
         </is>
       </c>
     </row>
@@ -7391,12 +7428,12 @@
       </c>
       <c r="C91" s="2" t="inlineStr">
         <is>
-          <t>data.amount</t>
+          <t>data.recipientName</t>
         </is>
       </c>
       <c r="D91" s="2" t="inlineStr">
         <is>
-          <t>Long</t>
+          <t>String</t>
         </is>
       </c>
       <c r="E91" s="2" t="inlineStr">
@@ -7406,12 +7443,12 @@
       </c>
       <c r="F91" s="2" t="inlineStr">
         <is>
-          <t>금액(원)</t>
+          <t>수취인 이름</t>
         </is>
       </c>
       <c r="G91" s="2" t="inlineStr">
         <is>
-          <t>10000</t>
+          <t>김영희</t>
         </is>
       </c>
     </row>
@@ -7428,12 +7465,12 @@
       </c>
       <c r="C92" s="2" t="inlineStr">
         <is>
-          <t>data.fromAccountNumber</t>
+          <t>data.amount</t>
         </is>
       </c>
       <c r="D92" s="2" t="inlineStr">
         <is>
-          <t>String</t>
+          <t>Long</t>
         </is>
       </c>
       <c r="E92" s="2" t="inlineStr">
@@ -7443,12 +7480,12 @@
       </c>
       <c r="F92" s="2" t="inlineStr">
         <is>
-          <t>출금 계좌</t>
+          <t>금액(원)</t>
         </is>
       </c>
       <c r="G92" s="2" t="inlineStr">
         <is>
-          <t>987654321098</t>
+          <t>10000</t>
         </is>
       </c>
     </row>
@@ -7465,12 +7502,12 @@
       </c>
       <c r="C93" s="2" t="inlineStr">
         <is>
-          <t>data.balanceAfter</t>
+          <t>data.fromAccountNumber</t>
         </is>
       </c>
       <c r="D93" s="2" t="inlineStr">
         <is>
-          <t>Long</t>
+          <t>String</t>
         </is>
       </c>
       <c r="E93" s="2" t="inlineStr">
@@ -7480,12 +7517,12 @@
       </c>
       <c r="F93" s="2" t="inlineStr">
         <is>
-          <t>송금 후 잔액(원)</t>
+          <t>출금 계좌</t>
         </is>
       </c>
       <c r="G93" s="2" t="inlineStr">
         <is>
-          <t>140000</t>
+          <t>987654321098</t>
         </is>
       </c>
     </row>
@@ -7497,22 +7534,34 @@
       </c>
       <c r="B94" s="2" t="inlineStr">
         <is>
-          <t>에러</t>
+          <t>응답</t>
         </is>
       </c>
       <c r="C94" s="2" t="inlineStr">
         <is>
-          <t>AUTH_INVALID</t>
-        </is>
-      </c>
-      <c r="D94" s="2" t="inlineStr"/>
-      <c r="E94" s="2" t="inlineStr"/>
+          <t>data.balanceAfter</t>
+        </is>
+      </c>
+      <c r="D94" s="2" t="inlineStr">
+        <is>
+          <t>Long</t>
+        </is>
+      </c>
+      <c r="E94" s="2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="F94" s="2" t="inlineStr">
         <is>
-          <t>JWT 없음·만료·위조, 로그인 실패</t>
-        </is>
-      </c>
-      <c r="G94" s="2" t="inlineStr"/>
+          <t>송금 후 잔액(원)</t>
+        </is>
+      </c>
+      <c r="G94" s="2" t="inlineStr">
+        <is>
+          <t>140000</t>
+        </is>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
@@ -7527,14 +7576,14 @@
       </c>
       <c r="C95" s="2" t="inlineStr">
         <is>
-          <t>TRANSFER_REQUEST_NOT_FOUND</t>
+          <t>AUTH_INVALID</t>
         </is>
       </c>
       <c r="D95" s="2" t="inlineStr"/>
       <c r="E95" s="2" t="inlineStr"/>
       <c r="F95" s="2" t="inlineStr">
         <is>
-          <t>송금 요청 없음(또는 남의 요청)</t>
+          <t>JWT 없음·만료·위조, 로그인 실패</t>
         </is>
       </c>
       <c r="G95" s="2" t="inlineStr"/>
@@ -7552,14 +7601,14 @@
       </c>
       <c r="C96" s="2" t="inlineStr">
         <is>
-          <t>TRANSFER_REQUEST_EXPIRED</t>
+          <t>TRANSFER_REQUEST_NOT_FOUND</t>
         </is>
       </c>
       <c r="D96" s="2" t="inlineStr"/>
       <c r="E96" s="2" t="inlineStr"/>
       <c r="F96" s="2" t="inlineStr">
         <is>
-          <t>송금 요청 5분 만료</t>
+          <t>송금 요청 없음(또는 남의 요청)</t>
         </is>
       </c>
       <c r="G96" s="2" t="inlineStr"/>
@@ -7577,14 +7626,14 @@
       </c>
       <c r="C97" s="2" t="inlineStr">
         <is>
-          <t>TRANSFER_REQUEST_ALREADY_USED</t>
+          <t>TRANSFER_REQUEST_EXPIRED</t>
         </is>
       </c>
       <c r="D97" s="2" t="inlineStr"/>
       <c r="E97" s="2" t="inlineStr"/>
       <c r="F97" s="2" t="inlineStr">
         <is>
-          <t>이미 확정된 송금 요청</t>
+          <t>송금 요청 5분 만료</t>
         </is>
       </c>
       <c r="G97" s="2" t="inlineStr"/>
@@ -7602,14 +7651,14 @@
       </c>
       <c r="C98" s="2" t="inlineStr">
         <is>
-          <t>ACCOUNT_NOT_OWNED</t>
+          <t>TRANSFER_REQUEST_ALREADY_USED</t>
         </is>
       </c>
       <c r="D98" s="2" t="inlineStr"/>
       <c r="E98" s="2" t="inlineStr"/>
       <c r="F98" s="2" t="inlineStr">
         <is>
-          <t>내 계좌가 아님</t>
+          <t>이미 확정된 송금 요청</t>
         </is>
       </c>
       <c r="G98" s="2" t="inlineStr"/>
@@ -7627,14 +7676,14 @@
       </c>
       <c r="C99" s="2" t="inlineStr">
         <is>
-          <t>INSUFFICIENT_BALANCE</t>
+          <t>ACCOUNT_NOT_OWNED</t>
         </is>
       </c>
       <c r="D99" s="2" t="inlineStr"/>
       <c r="E99" s="2" t="inlineStr"/>
       <c r="F99" s="2" t="inlineStr">
         <is>
-          <t>잔액 부족</t>
+          <t>내 계좌가 아님</t>
         </is>
       </c>
       <c r="G99" s="2" t="inlineStr"/>
@@ -7642,39 +7691,27 @@
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
         <is>
-          <t>E-13</t>
+          <t>E-12</t>
         </is>
       </c>
       <c r="B100" s="2" t="inlineStr">
         <is>
-          <t>요청</t>
+          <t>에러</t>
         </is>
       </c>
       <c r="C100" s="2" t="inlineStr">
         <is>
-          <t>Header Authorization</t>
-        </is>
-      </c>
-      <c r="D100" s="2" t="inlineStr">
-        <is>
-          <t>String</t>
-        </is>
-      </c>
-      <c r="E100" s="2" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+          <t>INSUFFICIENT_BALANCE</t>
+        </is>
+      </c>
+      <c r="D100" s="2" t="inlineStr"/>
+      <c r="E100" s="2" t="inlineStr"/>
       <c r="F100" s="2" t="inlineStr">
         <is>
-          <t>Bearer {JWT}</t>
-        </is>
-      </c>
-      <c r="G100" s="2" t="inlineStr">
-        <is>
-          <t>Bearer eyJ...</t>
-        </is>
-      </c>
+          <t>잔액 부족</t>
+        </is>
+      </c>
+      <c r="G100" s="2" t="inlineStr"/>
     </row>
     <row r="101">
       <c r="A101" s="2" t="inlineStr">
@@ -7689,7 +7726,7 @@
       </c>
       <c r="C101" s="2" t="inlineStr">
         <is>
-          <t>Path detailId</t>
+          <t>Header Authorization</t>
         </is>
       </c>
       <c r="D101" s="2" t="inlineStr">
@@ -7704,12 +7741,12 @@
       </c>
       <c r="F101" s="2" t="inlineStr">
         <is>
-          <t>답변의 detailId</t>
+          <t>Bearer {JWT}</t>
         </is>
       </c>
       <c r="G101" s="2" t="inlineStr">
         <is>
-          <t>dt_91c2...</t>
+          <t>Bearer eyJ...</t>
         </is>
       </c>
     </row>
@@ -7721,12 +7758,12 @@
       </c>
       <c r="B102" s="2" t="inlineStr">
         <is>
-          <t>응답</t>
+          <t>요청</t>
         </is>
       </c>
       <c r="C102" s="2" t="inlineStr">
         <is>
-          <t>data.detailId</t>
+          <t>Path detailId</t>
         </is>
       </c>
       <c r="D102" s="2" t="inlineStr">
@@ -7741,7 +7778,7 @@
       </c>
       <c r="F102" s="2" t="inlineStr">
         <is>
-          <t>상세 보기 ID</t>
+          <t>답변의 detailId</t>
         </is>
       </c>
       <c r="G102" s="2" t="inlineStr">
@@ -7763,7 +7800,7 @@
       </c>
       <c r="C103" s="2" t="inlineStr">
         <is>
-          <t>data.report</t>
+          <t>data.detailId</t>
         </is>
       </c>
       <c r="D103" s="2" t="inlineStr">
@@ -7778,12 +7815,12 @@
       </c>
       <c r="F103" s="2" t="inlineStr">
         <is>
-          <t>상세 보고서 본문(클릭할 때 생성)</t>
+          <t>상세 보기 ID</t>
         </is>
       </c>
       <c r="G103" s="2" t="inlineStr">
         <is>
-          <t>...</t>
+          <t>dt_91c2...</t>
         </is>
       </c>
     </row>
@@ -7800,27 +7837,27 @@
       </c>
       <c r="C104" s="2" t="inlineStr">
         <is>
-          <t>data.table.columns</t>
+          <t>data.report</t>
         </is>
       </c>
       <c r="D104" s="2" t="inlineStr">
         <is>
-          <t>String[]</t>
+          <t>String</t>
         </is>
       </c>
       <c r="E104" s="2" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="F104" s="2" t="inlineStr">
         <is>
-          <t>표 머리글</t>
+          <t>상세 보고서 본문(클릭할 때 생성)</t>
         </is>
       </c>
       <c r="G104" s="2" t="inlineStr">
         <is>
-          <t>["항목", ...]</t>
+          <t>...</t>
         </is>
       </c>
     </row>
@@ -7837,12 +7874,12 @@
       </c>
       <c r="C105" s="2" t="inlineStr">
         <is>
-          <t>data.table.rows</t>
+          <t>data.table.columns</t>
         </is>
       </c>
       <c r="D105" s="2" t="inlineStr">
         <is>
-          <t>String[][]</t>
+          <t>String[]</t>
         </is>
       </c>
       <c r="E105" s="2" t="inlineStr">
@@ -7852,12 +7889,12 @@
       </c>
       <c r="F105" s="2" t="inlineStr">
         <is>
-          <t>표 행</t>
+          <t>표 머리글</t>
         </is>
       </c>
       <c r="G105" s="2" t="inlineStr">
         <is>
-          <t>[[...]]</t>
+          <t>["항목", ...]</t>
         </is>
       </c>
     </row>
@@ -7874,12 +7911,12 @@
       </c>
       <c r="C106" s="2" t="inlineStr">
         <is>
-          <t>data.table.note</t>
+          <t>data.table.rows</t>
         </is>
       </c>
       <c r="D106" s="2" t="inlineStr">
         <is>
-          <t>String</t>
+          <t>String[][]</t>
         </is>
       </c>
       <c r="E106" s="2" t="inlineStr">
@@ -7889,12 +7926,12 @@
       </c>
       <c r="F106" s="2" t="inlineStr">
         <is>
-          <t>재무제표 기준·미공시 표시</t>
+          <t>표 행</t>
         </is>
       </c>
       <c r="G106" s="2" t="inlineStr">
         <is>
-          <t>연결 기준</t>
+          <t>[[...]]</t>
         </is>
       </c>
     </row>
@@ -7906,22 +7943,34 @@
       </c>
       <c r="B107" s="2" t="inlineStr">
         <is>
-          <t>에러</t>
+          <t>응답</t>
         </is>
       </c>
       <c r="C107" s="2" t="inlineStr">
         <is>
-          <t>AUTH_INVALID</t>
-        </is>
-      </c>
-      <c r="D107" s="2" t="inlineStr"/>
-      <c r="E107" s="2" t="inlineStr"/>
+          <t>data.table.note</t>
+        </is>
+      </c>
+      <c r="D107" s="2" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="E107" s="2" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="F107" s="2" t="inlineStr">
         <is>
-          <t>JWT 없음·만료·위조, 로그인 실패</t>
-        </is>
-      </c>
-      <c r="G107" s="2" t="inlineStr"/>
+          <t>재무제표 기준·미공시 표시</t>
+        </is>
+      </c>
+      <c r="G107" s="2" t="inlineStr">
+        <is>
+          <t>연결 기준</t>
+        </is>
+      </c>
     </row>
     <row r="108">
       <c r="A108" s="2" t="inlineStr">
@@ -7936,14 +7985,14 @@
       </c>
       <c r="C108" s="2" t="inlineStr">
         <is>
-          <t>DETAIL_NOT_FOUND</t>
+          <t>AUTH_INVALID</t>
         </is>
       </c>
       <c r="D108" s="2" t="inlineStr"/>
       <c r="E108" s="2" t="inlineStr"/>
       <c r="F108" s="2" t="inlineStr">
         <is>
-          <t>상세 보기 대상 없음(또는 남의 것)</t>
+          <t>JWT 없음·만료·위조, 로그인 실패</t>
         </is>
       </c>
       <c r="G108" s="2" t="inlineStr"/>
@@ -7961,14 +8010,14 @@
       </c>
       <c r="C109" s="2" t="inlineStr">
         <is>
-          <t>AI_SERVER_UNAVAILABLE</t>
+          <t>DETAIL_NOT_FOUND</t>
         </is>
       </c>
       <c r="D109" s="2" t="inlineStr"/>
       <c r="E109" s="2" t="inlineStr"/>
       <c r="F109" s="2" t="inlineStr">
         <is>
-          <t>FastAPI 장애·지연 — 채팅만 실패, 송금·계좌는 정상(장애 격리)</t>
+          <t>상세 보기 대상 없음(또는 남의 것)</t>
         </is>
       </c>
       <c r="G109" s="2" t="inlineStr"/>
@@ -7976,39 +8025,27 @@
     <row r="110">
       <c r="A110" s="2" t="inlineStr">
         <is>
-          <t>I-01</t>
+          <t>E-13</t>
         </is>
       </c>
       <c r="B110" s="2" t="inlineStr">
         <is>
-          <t>요청</t>
+          <t>에러</t>
         </is>
       </c>
       <c r="C110" s="2" t="inlineStr">
         <is>
-          <t>Header Authorization</t>
-        </is>
-      </c>
-      <c r="D110" s="2" t="inlineStr">
-        <is>
-          <t>String</t>
-        </is>
-      </c>
-      <c r="E110" s="2" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+          <t>AI_SERVER_UNAVAILABLE</t>
+        </is>
+      </c>
+      <c r="D110" s="2" t="inlineStr"/>
+      <c r="E110" s="2" t="inlineStr"/>
       <c r="F110" s="2" t="inlineStr">
         <is>
-          <t>Bearer {JWT}</t>
-        </is>
-      </c>
-      <c r="G110" s="2" t="inlineStr">
-        <is>
-          <t>Bearer eyJ...</t>
-        </is>
-      </c>
+          <t>FastAPI 장애·지연 — 채팅만 실패, 송금·계좌는 정상(장애 격리)</t>
+        </is>
+      </c>
+      <c r="G110" s="2" t="inlineStr"/>
     </row>
     <row r="111">
       <c r="A111" s="2" t="inlineStr">
@@ -8023,7 +8060,7 @@
       </c>
       <c r="C111" s="2" t="inlineStr">
         <is>
-          <t>threadId</t>
+          <t>Header Authorization</t>
         </is>
       </c>
       <c r="D111" s="2" t="inlineStr">
@@ -8038,12 +8075,12 @@
       </c>
       <c r="F111" s="2" t="inlineStr">
         <is>
-          <t>대화 ID(체크포인터 키)</t>
+          <t>Bearer {JWT}</t>
         </is>
       </c>
       <c r="G111" s="2" t="inlineStr">
         <is>
-          <t>th_5b21...</t>
+          <t>Bearer eyJ...</t>
         </is>
       </c>
     </row>
@@ -8060,7 +8097,7 @@
       </c>
       <c r="C112" s="2" t="inlineStr">
         <is>
-          <t>message</t>
+          <t>threadId</t>
         </is>
       </c>
       <c r="D112" s="2" t="inlineStr">
@@ -8075,12 +8112,12 @@
       </c>
       <c r="F112" s="2" t="inlineStr">
         <is>
-          <t>사용자 메시지</t>
+          <t>대화 ID(체크포인터 키)</t>
         </is>
       </c>
       <c r="G112" s="2" t="inlineStr">
         <is>
-          <t>엄마한테 1만원 보내줘</t>
+          <t>th_5b21...</t>
         </is>
       </c>
     </row>
@@ -8092,12 +8129,12 @@
       </c>
       <c r="B113" s="2" t="inlineStr">
         <is>
-          <t>응답</t>
+          <t>요청</t>
         </is>
       </c>
       <c r="C113" s="2" t="inlineStr">
         <is>
-          <t>data.reply</t>
+          <t>message</t>
         </is>
       </c>
       <c r="D113" s="2" t="inlineStr">
@@ -8112,12 +8149,12 @@
       </c>
       <c r="F113" s="2" t="inlineStr">
         <is>
-          <t>요약 답변. 가드에 걸리면 고정 문장</t>
+          <t>사용자 메시지</t>
         </is>
       </c>
       <c r="G113" s="2" t="inlineStr">
         <is>
-          <t>삼성전자 2분기 영업이익은 ...</t>
+          <t>엄마한테 1만원 보내줘</t>
         </is>
       </c>
     </row>
@@ -8134,7 +8171,7 @@
       </c>
       <c r="C114" s="2" t="inlineStr">
         <is>
-          <t>data.guard</t>
+          <t>data.reply</t>
         </is>
       </c>
       <c r="D114" s="2" t="inlineStr">
@@ -8149,12 +8186,12 @@
       </c>
       <c r="F114" s="2" t="inlineStr">
         <is>
-          <t>판정 코드: PASS / INJECTION / NUMBER_UNVERIFIED / ADVICE / PROMPT_LEAK</t>
+          <t>요약 답변. 가드에 걸리면 고정 문장</t>
         </is>
       </c>
       <c r="G114" s="2" t="inlineStr">
         <is>
-          <t>PASS</t>
+          <t>삼성전자 2분기 영업이익은 ...</t>
         </is>
       </c>
     </row>
@@ -8171,7 +8208,7 @@
       </c>
       <c r="C115" s="2" t="inlineStr">
         <is>
-          <t>data.transferCard.requestId</t>
+          <t>data.guard</t>
         </is>
       </c>
       <c r="D115" s="2" t="inlineStr">
@@ -8181,17 +8218,17 @@
       </c>
       <c r="E115" s="2" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="F115" s="2" t="inlineStr">
         <is>
-          <t>송금 요청ID(1회용)</t>
+          <t>판정 코드: PASS / INJECTION / NUMBER_UNVERIFIED / ADVICE / PROMPT_LEAK</t>
         </is>
       </c>
       <c r="G115" s="2" t="inlineStr">
         <is>
-          <t>tr_7f3a...</t>
+          <t>PASS</t>
         </is>
       </c>
     </row>
@@ -8208,7 +8245,7 @@
       </c>
       <c r="C116" s="2" t="inlineStr">
         <is>
-          <t>data.transferCard.recipientName</t>
+          <t>data.transferCard.requestId</t>
         </is>
       </c>
       <c r="D116" s="2" t="inlineStr">
@@ -8223,12 +8260,12 @@
       </c>
       <c r="F116" s="2" t="inlineStr">
         <is>
-          <t>수취인 이름</t>
+          <t>송금 요청ID(1회용)</t>
         </is>
       </c>
       <c r="G116" s="2" t="inlineStr">
         <is>
-          <t>김영희</t>
+          <t>tr_7f3a...</t>
         </is>
       </c>
     </row>
@@ -8245,7 +8282,7 @@
       </c>
       <c r="C117" s="2" t="inlineStr">
         <is>
-          <t>data.transferCard.recipientAccountNumber</t>
+          <t>data.transferCard.recipientName</t>
         </is>
       </c>
       <c r="D117" s="2" t="inlineStr">
@@ -8260,12 +8297,12 @@
       </c>
       <c r="F117" s="2" t="inlineStr">
         <is>
-          <t>수취인 계좌</t>
+          <t>수취인 이름</t>
         </is>
       </c>
       <c r="G117" s="2" t="inlineStr">
         <is>
-          <t>123456789012</t>
+          <t>김영희</t>
         </is>
       </c>
     </row>
@@ -8282,7 +8319,7 @@
       </c>
       <c r="C118" s="2" t="inlineStr">
         <is>
-          <t>data.transferCard.fromAccountNumber</t>
+          <t>data.transferCard.recipientAccountNumber</t>
         </is>
       </c>
       <c r="D118" s="2" t="inlineStr">
@@ -8297,12 +8334,12 @@
       </c>
       <c r="F118" s="2" t="inlineStr">
         <is>
-          <t>출금 계좌(대표 계좌)</t>
+          <t>수취인 계좌</t>
         </is>
       </c>
       <c r="G118" s="2" t="inlineStr">
         <is>
-          <t>987654321098</t>
+          <t>123456789012</t>
         </is>
       </c>
     </row>
@@ -8319,12 +8356,12 @@
       </c>
       <c r="C119" s="2" t="inlineStr">
         <is>
-          <t>data.transferCard.amount</t>
+          <t>data.transferCard.fromAccountNumber</t>
         </is>
       </c>
       <c r="D119" s="2" t="inlineStr">
         <is>
-          <t>Long</t>
+          <t>String</t>
         </is>
       </c>
       <c r="E119" s="2" t="inlineStr">
@@ -8334,12 +8371,12 @@
       </c>
       <c r="F119" s="2" t="inlineStr">
         <is>
-          <t>금액(원)</t>
+          <t>출금 계좌(대표 계좌)</t>
         </is>
       </c>
       <c r="G119" s="2" t="inlineStr">
         <is>
-          <t>10000</t>
+          <t>987654321098</t>
         </is>
       </c>
     </row>
@@ -8356,12 +8393,12 @@
       </c>
       <c r="C120" s="2" t="inlineStr">
         <is>
-          <t>data.transferCard.expiresAt</t>
+          <t>data.transferCard.amount</t>
         </is>
       </c>
       <c r="D120" s="2" t="inlineStr">
         <is>
-          <t>String</t>
+          <t>Long</t>
         </is>
       </c>
       <c r="E120" s="2" t="inlineStr">
@@ -8371,12 +8408,12 @@
       </c>
       <c r="F120" s="2" t="inlineStr">
         <is>
-          <t>만료 시각(생성 + 5분, ISO-8601)</t>
+          <t>금액(원)</t>
         </is>
       </c>
       <c r="G120" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T10:05:00+09:00</t>
+          <t>10000</t>
         </is>
       </c>
     </row>
@@ -8393,12 +8430,12 @@
       </c>
       <c r="C121" s="2" t="inlineStr">
         <is>
-          <t>data.table.columns</t>
+          <t>data.transferCard.expiresAt</t>
         </is>
       </c>
       <c r="D121" s="2" t="inlineStr">
         <is>
-          <t>String[]</t>
+          <t>String</t>
         </is>
       </c>
       <c r="E121" s="2" t="inlineStr">
@@ -8408,12 +8445,12 @@
       </c>
       <c r="F121" s="2" t="inlineStr">
         <is>
-          <t>표 머리글</t>
+          <t>만료 시각(생성 + 5분, ISO-8601)</t>
         </is>
       </c>
       <c r="G121" s="2" t="inlineStr">
         <is>
-          <t>["항목","삼성전자","SK하이닉스"]</t>
+          <t>2026-09-27T10:05:00+09:00</t>
         </is>
       </c>
     </row>
@@ -8430,12 +8467,12 @@
       </c>
       <c r="C122" s="2" t="inlineStr">
         <is>
-          <t>data.table.rows</t>
+          <t>data.table.columns</t>
         </is>
       </c>
       <c r="D122" s="2" t="inlineStr">
         <is>
-          <t>String[][]</t>
+          <t>String[]</t>
         </is>
       </c>
       <c r="E122" s="2" t="inlineStr">
@@ -8445,12 +8482,12 @@
       </c>
       <c r="F122" s="2" t="inlineStr">
         <is>
-          <t>표 행</t>
+          <t>표 머리글</t>
         </is>
       </c>
       <c r="G122" s="2" t="inlineStr">
         <is>
-          <t>[["영업이익","...","..."]]</t>
+          <t>["항목","삼성전자","SK하이닉스"]</t>
         </is>
       </c>
     </row>
@@ -8467,12 +8504,12 @@
       </c>
       <c r="C123" s="2" t="inlineStr">
         <is>
-          <t>data.table.note</t>
+          <t>data.table.rows</t>
         </is>
       </c>
       <c r="D123" s="2" t="inlineStr">
         <is>
-          <t>String</t>
+          <t>String[][]</t>
         </is>
       </c>
       <c r="E123" s="2" t="inlineStr">
@@ -8482,12 +8519,12 @@
       </c>
       <c r="F123" s="2" t="inlineStr">
         <is>
-          <t>재무제표 기준(연결/별도)·미공시 표시</t>
+          <t>표 행</t>
         </is>
       </c>
       <c r="G123" s="2" t="inlineStr">
         <is>
-          <t>연결 기준</t>
+          <t>[["영업이익","...","..."]]</t>
         </is>
       </c>
     </row>
@@ -8504,7 +8541,7 @@
       </c>
       <c r="C124" s="2" t="inlineStr">
         <is>
-          <t>data.detailId</t>
+          <t>data.table.note</t>
         </is>
       </c>
       <c r="D124" s="2" t="inlineStr">
@@ -8519,12 +8556,12 @@
       </c>
       <c r="F124" s="2" t="inlineStr">
         <is>
-          <t>상세 보기 ID(분석 답변일 때)</t>
+          <t>재무제표 기준(연결/별도)·미공시 표시</t>
         </is>
       </c>
       <c r="G124" s="2" t="inlineStr">
         <is>
-          <t>dt_91c2...</t>
+          <t>연결 기준</t>
         </is>
       </c>
     </row>
@@ -8536,59 +8573,59 @@
       </c>
       <c r="B125" s="2" t="inlineStr">
         <is>
-          <t>에러</t>
+          <t>응답</t>
         </is>
       </c>
       <c r="C125" s="2" t="inlineStr">
         <is>
-          <t>AUTH_INVALID</t>
-        </is>
-      </c>
-      <c r="D125" s="2" t="inlineStr"/>
-      <c r="E125" s="2" t="inlineStr"/>
+          <t>data.detailId</t>
+        </is>
+      </c>
+      <c r="D125" s="2" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="E125" s="2" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="F125" s="2" t="inlineStr">
         <is>
-          <t>JWT 없음·만료·위조, 로그인 실패</t>
-        </is>
-      </c>
-      <c r="G125" s="2" t="inlineStr"/>
+          <t>상세 보기 ID(분석 답변일 때)</t>
+        </is>
+      </c>
+      <c r="G125" s="2" t="inlineStr">
+        <is>
+          <t>dt_91c2...</t>
+        </is>
+      </c>
     </row>
     <row r="126">
       <c r="A126" s="2" t="inlineStr">
         <is>
-          <t>I-02</t>
+          <t>I-01</t>
         </is>
       </c>
       <c r="B126" s="2" t="inlineStr">
         <is>
-          <t>요청</t>
+          <t>에러</t>
         </is>
       </c>
       <c r="C126" s="2" t="inlineStr">
         <is>
-          <t>Header Authorization</t>
-        </is>
-      </c>
-      <c r="D126" s="2" t="inlineStr">
-        <is>
-          <t>String</t>
-        </is>
-      </c>
-      <c r="E126" s="2" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+          <t>AUTH_INVALID</t>
+        </is>
+      </c>
+      <c r="D126" s="2" t="inlineStr"/>
+      <c r="E126" s="2" t="inlineStr"/>
       <c r="F126" s="2" t="inlineStr">
         <is>
-          <t>Bearer {JWT}</t>
-        </is>
-      </c>
-      <c r="G126" s="2" t="inlineStr">
-        <is>
-          <t>Bearer eyJ...</t>
-        </is>
-      </c>
+          <t>JWT 없음·만료·위조, 로그인 실패</t>
+        </is>
+      </c>
+      <c r="G126" s="2" t="inlineStr"/>
     </row>
     <row r="127">
       <c r="A127" s="2" t="inlineStr">
@@ -8603,7 +8640,7 @@
       </c>
       <c r="C127" s="2" t="inlineStr">
         <is>
-          <t>Path detailId</t>
+          <t>Header Authorization</t>
         </is>
       </c>
       <c r="D127" s="2" t="inlineStr">
@@ -8618,12 +8655,12 @@
       </c>
       <c r="F127" s="2" t="inlineStr">
         <is>
-          <t>상세 보기 ID</t>
+          <t>Bearer {JWT}</t>
         </is>
       </c>
       <c r="G127" s="2" t="inlineStr">
         <is>
-          <t>dt_91c2...</t>
+          <t>Bearer eyJ...</t>
         </is>
       </c>
     </row>
@@ -8635,12 +8672,12 @@
       </c>
       <c r="B128" s="2" t="inlineStr">
         <is>
-          <t>응답</t>
+          <t>요청</t>
         </is>
       </c>
       <c r="C128" s="2" t="inlineStr">
         <is>
-          <t>data.report</t>
+          <t>Path detailId</t>
         </is>
       </c>
       <c r="D128" s="2" t="inlineStr">
@@ -8655,12 +8692,12 @@
       </c>
       <c r="F128" s="2" t="inlineStr">
         <is>
-          <t>상세 보고서 본문</t>
+          <t>상세 보기 ID</t>
         </is>
       </c>
       <c r="G128" s="2" t="inlineStr">
         <is>
-          <t>...</t>
+          <t>dt_91c2...</t>
         </is>
       </c>
     </row>
@@ -8677,27 +8714,27 @@
       </c>
       <c r="C129" s="2" t="inlineStr">
         <is>
-          <t>data.table.columns</t>
+          <t>data.report</t>
         </is>
       </c>
       <c r="D129" s="2" t="inlineStr">
         <is>
-          <t>String[]</t>
+          <t>String</t>
         </is>
       </c>
       <c r="E129" s="2" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="F129" s="2" t="inlineStr">
         <is>
-          <t>표 머리글</t>
+          <t>상세 보고서 본문</t>
         </is>
       </c>
       <c r="G129" s="2" t="inlineStr">
         <is>
-          <t>["항목", ...]</t>
+          <t>...</t>
         </is>
       </c>
     </row>
@@ -8714,12 +8751,12 @@
       </c>
       <c r="C130" s="2" t="inlineStr">
         <is>
-          <t>data.table.rows</t>
+          <t>data.table.columns</t>
         </is>
       </c>
       <c r="D130" s="2" t="inlineStr">
         <is>
-          <t>String[][]</t>
+          <t>String[]</t>
         </is>
       </c>
       <c r="E130" s="2" t="inlineStr">
@@ -8729,12 +8766,12 @@
       </c>
       <c r="F130" s="2" t="inlineStr">
         <is>
-          <t>표 행</t>
+          <t>표 머리글</t>
         </is>
       </c>
       <c r="G130" s="2" t="inlineStr">
         <is>
-          <t>[[...]]</t>
+          <t>["항목", ...]</t>
         </is>
       </c>
     </row>
@@ -8751,12 +8788,12 @@
       </c>
       <c r="C131" s="2" t="inlineStr">
         <is>
-          <t>data.table.note</t>
+          <t>data.table.rows</t>
         </is>
       </c>
       <c r="D131" s="2" t="inlineStr">
         <is>
-          <t>String</t>
+          <t>String[][]</t>
         </is>
       </c>
       <c r="E131" s="2" t="inlineStr">
@@ -8766,12 +8803,12 @@
       </c>
       <c r="F131" s="2" t="inlineStr">
         <is>
-          <t>재무제표 기준·미공시 표시</t>
+          <t>표 행</t>
         </is>
       </c>
       <c r="G131" s="2" t="inlineStr">
         <is>
-          <t>연결 기준</t>
+          <t>[[...]]</t>
         </is>
       </c>
     </row>
@@ -8783,22 +8820,34 @@
       </c>
       <c r="B132" s="2" t="inlineStr">
         <is>
-          <t>에러</t>
+          <t>응답</t>
         </is>
       </c>
       <c r="C132" s="2" t="inlineStr">
         <is>
-          <t>AUTH_INVALID</t>
-        </is>
-      </c>
-      <c r="D132" s="2" t="inlineStr"/>
-      <c r="E132" s="2" t="inlineStr"/>
+          <t>data.table.note</t>
+        </is>
+      </c>
+      <c r="D132" s="2" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="E132" s="2" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="F132" s="2" t="inlineStr">
         <is>
-          <t>JWT 없음·만료·위조, 로그인 실패</t>
-        </is>
-      </c>
-      <c r="G132" s="2" t="inlineStr"/>
+          <t>재무제표 기준·미공시 표시</t>
+        </is>
+      </c>
+      <c r="G132" s="2" t="inlineStr">
+        <is>
+          <t>연결 기준</t>
+        </is>
+      </c>
     </row>
     <row r="133">
       <c r="A133" s="2" t="inlineStr">
@@ -8813,14 +8862,14 @@
       </c>
       <c r="C133" s="2" t="inlineStr">
         <is>
-          <t>DETAIL_NOT_FOUND</t>
+          <t>AUTH_INVALID</t>
         </is>
       </c>
       <c r="D133" s="2" t="inlineStr"/>
       <c r="E133" s="2" t="inlineStr"/>
       <c r="F133" s="2" t="inlineStr">
         <is>
-          <t>상세 보기 대상 없음(또는 남의 것)</t>
+          <t>JWT 없음·만료·위조, 로그인 실패</t>
         </is>
       </c>
       <c r="G133" s="2" t="inlineStr"/>
@@ -8828,39 +8877,27 @@
     <row r="134">
       <c r="A134" s="2" t="inlineStr">
         <is>
-          <t>I-03</t>
+          <t>I-02</t>
         </is>
       </c>
       <c r="B134" s="2" t="inlineStr">
         <is>
-          <t>요청</t>
+          <t>에러</t>
         </is>
       </c>
       <c r="C134" s="2" t="inlineStr">
         <is>
-          <t>Header Authorization</t>
-        </is>
-      </c>
-      <c r="D134" s="2" t="inlineStr">
-        <is>
-          <t>String</t>
-        </is>
-      </c>
-      <c r="E134" s="2" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+          <t>DETAIL_NOT_FOUND</t>
+        </is>
+      </c>
+      <c r="D134" s="2" t="inlineStr"/>
+      <c r="E134" s="2" t="inlineStr"/>
       <c r="F134" s="2" t="inlineStr">
         <is>
-          <t>Bearer {JWT}</t>
-        </is>
-      </c>
-      <c r="G134" s="2" t="inlineStr">
-        <is>
-          <t>Bearer eyJ...</t>
-        </is>
-      </c>
+          <t>상세 보기 대상 없음(또는 남의 것)</t>
+        </is>
+      </c>
+      <c r="G134" s="2" t="inlineStr"/>
     </row>
     <row r="135">
       <c r="A135" s="2" t="inlineStr">
@@ -8875,7 +8912,7 @@
       </c>
       <c r="C135" s="2" t="inlineStr">
         <is>
-          <t>recipientAccountNumber</t>
+          <t>Header Authorization</t>
         </is>
       </c>
       <c r="D135" s="2" t="inlineStr">
@@ -8885,17 +8922,17 @@
       </c>
       <c r="E135" s="2" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="F135" s="2" t="inlineStr">
         <is>
-          <t>수취인 계좌번호(alias와 둘 중 하나)</t>
+          <t>Bearer {JWT}</t>
         </is>
       </c>
       <c r="G135" s="2" t="inlineStr">
         <is>
-          <t>123456789012</t>
+          <t>Bearer eyJ...</t>
         </is>
       </c>
     </row>
@@ -8912,7 +8949,7 @@
       </c>
       <c r="C136" s="2" t="inlineStr">
         <is>
-          <t>alias</t>
+          <t>recipientAccountNumber</t>
         </is>
       </c>
       <c r="D136" s="2" t="inlineStr">
@@ -8927,12 +8964,12 @@
       </c>
       <c r="F136" s="2" t="inlineStr">
         <is>
-          <t>별칭(recipientAccountNumber와 둘 중 하나)</t>
+          <t>수취인 계좌번호(alias와 둘 중 하나)</t>
         </is>
       </c>
       <c r="G136" s="2" t="inlineStr">
         <is>
-          <t>엄마</t>
+          <t>123456789012</t>
         </is>
       </c>
     </row>
@@ -8949,27 +8986,27 @@
       </c>
       <c r="C137" s="2" t="inlineStr">
         <is>
-          <t>amount</t>
+          <t>alias</t>
         </is>
       </c>
       <c r="D137" s="2" t="inlineStr">
         <is>
-          <t>Long</t>
+          <t>String</t>
         </is>
       </c>
       <c r="E137" s="2" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="F137" s="2" t="inlineStr">
         <is>
-          <t>금액(원)</t>
+          <t>별칭(recipientAccountNumber와 둘 중 하나)</t>
         </is>
       </c>
       <c r="G137" s="2" t="inlineStr">
         <is>
-          <t>10000</t>
+          <t>엄마</t>
         </is>
       </c>
     </row>
@@ -8981,17 +9018,17 @@
       </c>
       <c r="B138" s="2" t="inlineStr">
         <is>
-          <t>응답</t>
+          <t>요청</t>
         </is>
       </c>
       <c r="C138" s="2" t="inlineStr">
         <is>
-          <t>data.requestId</t>
+          <t>amount</t>
         </is>
       </c>
       <c r="D138" s="2" t="inlineStr">
         <is>
-          <t>String</t>
+          <t>Long</t>
         </is>
       </c>
       <c r="E138" s="2" t="inlineStr">
@@ -9001,12 +9038,12 @@
       </c>
       <c r="F138" s="2" t="inlineStr">
         <is>
-          <t>송금 요청ID(1회용)</t>
+          <t>금액(원)</t>
         </is>
       </c>
       <c r="G138" s="2" t="inlineStr">
         <is>
-          <t>tr_7f3a...</t>
+          <t>10000</t>
         </is>
       </c>
     </row>
@@ -9023,7 +9060,7 @@
       </c>
       <c r="C139" s="2" t="inlineStr">
         <is>
-          <t>data.recipientName</t>
+          <t>data.requestId</t>
         </is>
       </c>
       <c r="D139" s="2" t="inlineStr">
@@ -9038,12 +9075,12 @@
       </c>
       <c r="F139" s="2" t="inlineStr">
         <is>
-          <t>수취인 이름</t>
+          <t>송금 요청ID(1회용)</t>
         </is>
       </c>
       <c r="G139" s="2" t="inlineStr">
         <is>
-          <t>김영희</t>
+          <t>tr_7f3a...</t>
         </is>
       </c>
     </row>
@@ -9060,7 +9097,7 @@
       </c>
       <c r="C140" s="2" t="inlineStr">
         <is>
-          <t>data.recipientAccountNumber</t>
+          <t>data.recipientName</t>
         </is>
       </c>
       <c r="D140" s="2" t="inlineStr">
@@ -9075,12 +9112,12 @@
       </c>
       <c r="F140" s="2" t="inlineStr">
         <is>
-          <t>수취인 계좌</t>
+          <t>수취인 이름</t>
         </is>
       </c>
       <c r="G140" s="2" t="inlineStr">
         <is>
-          <t>123456789012</t>
+          <t>김영희</t>
         </is>
       </c>
     </row>
@@ -9097,7 +9134,7 @@
       </c>
       <c r="C141" s="2" t="inlineStr">
         <is>
-          <t>data.fromAccountNumber</t>
+          <t>data.recipientAccountNumber</t>
         </is>
       </c>
       <c r="D141" s="2" t="inlineStr">
@@ -9112,12 +9149,12 @@
       </c>
       <c r="F141" s="2" t="inlineStr">
         <is>
-          <t>출금 계좌(대표 계좌)</t>
+          <t>수취인 계좌</t>
         </is>
       </c>
       <c r="G141" s="2" t="inlineStr">
         <is>
-          <t>987654321098</t>
+          <t>123456789012</t>
         </is>
       </c>
     </row>
@@ -9134,12 +9171,12 @@
       </c>
       <c r="C142" s="2" t="inlineStr">
         <is>
-          <t>data.amount</t>
+          <t>data.fromAccountNumber</t>
         </is>
       </c>
       <c r="D142" s="2" t="inlineStr">
         <is>
-          <t>Long</t>
+          <t>String</t>
         </is>
       </c>
       <c r="E142" s="2" t="inlineStr">
@@ -9149,12 +9186,12 @@
       </c>
       <c r="F142" s="2" t="inlineStr">
         <is>
-          <t>금액(원)</t>
+          <t>출금 계좌(대표 계좌)</t>
         </is>
       </c>
       <c r="G142" s="2" t="inlineStr">
         <is>
-          <t>10000</t>
+          <t>987654321098</t>
         </is>
       </c>
     </row>
@@ -9171,12 +9208,12 @@
       </c>
       <c r="C143" s="2" t="inlineStr">
         <is>
-          <t>data.expiresAt</t>
+          <t>data.amount</t>
         </is>
       </c>
       <c r="D143" s="2" t="inlineStr">
         <is>
-          <t>String</t>
+          <t>Long</t>
         </is>
       </c>
       <c r="E143" s="2" t="inlineStr">
@@ -9186,12 +9223,12 @@
       </c>
       <c r="F143" s="2" t="inlineStr">
         <is>
-          <t>만료 시각(생성 + 5분, ISO-8601)</t>
+          <t>금액(원)</t>
         </is>
       </c>
       <c r="G143" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T10:05:00+09:00</t>
+          <t>10000</t>
         </is>
       </c>
     </row>
@@ -9203,22 +9240,34 @@
       </c>
       <c r="B144" s="2" t="inlineStr">
         <is>
-          <t>에러</t>
+          <t>응답</t>
         </is>
       </c>
       <c r="C144" s="2" t="inlineStr">
         <is>
-          <t>AUTH_INVALID</t>
-        </is>
-      </c>
-      <c r="D144" s="2" t="inlineStr"/>
-      <c r="E144" s="2" t="inlineStr"/>
+          <t>data.expiresAt</t>
+        </is>
+      </c>
+      <c r="D144" s="2" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="E144" s="2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="F144" s="2" t="inlineStr">
         <is>
-          <t>JWT 없음·만료·위조, 로그인 실패</t>
-        </is>
-      </c>
-      <c r="G144" s="2" t="inlineStr"/>
+          <t>만료 시각(생성 + 5분, ISO-8601)</t>
+        </is>
+      </c>
+      <c r="G144" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-27T10:05:00+09:00</t>
+        </is>
+      </c>
     </row>
     <row r="145">
       <c r="A145" s="2" t="inlineStr">
@@ -9233,14 +9282,14 @@
       </c>
       <c r="C145" s="2" t="inlineStr">
         <is>
-          <t>ALIAS_NOT_FOUND</t>
+          <t>AUTH_INVALID</t>
         </is>
       </c>
       <c r="D145" s="2" t="inlineStr"/>
       <c r="E145" s="2" t="inlineStr"/>
       <c r="F145" s="2" t="inlineStr">
         <is>
-          <t>등록되지 않은 별칭</t>
+          <t>JWT 없음·만료·위조, 로그인 실패</t>
         </is>
       </c>
       <c r="G145" s="2" t="inlineStr"/>
@@ -9258,14 +9307,14 @@
       </c>
       <c r="C146" s="2" t="inlineStr">
         <is>
-          <t>ACCOUNT_NOT_FOUND</t>
+          <t>ALIAS_NOT_FOUND</t>
         </is>
       </c>
       <c r="D146" s="2" t="inlineStr"/>
       <c r="E146" s="2" t="inlineStr"/>
       <c r="F146" s="2" t="inlineStr">
         <is>
-          <t>계좌 없음</t>
+          <t>등록되지 않은 별칭</t>
         </is>
       </c>
       <c r="G146" s="2" t="inlineStr"/>
@@ -9273,39 +9322,27 @@
     <row r="147">
       <c r="A147" s="2" t="inlineStr">
         <is>
-          <t>I-04</t>
+          <t>I-03</t>
         </is>
       </c>
       <c r="B147" s="2" t="inlineStr">
         <is>
-          <t>요청</t>
+          <t>에러</t>
         </is>
       </c>
       <c r="C147" s="2" t="inlineStr">
         <is>
-          <t>Header Authorization</t>
-        </is>
-      </c>
-      <c r="D147" s="2" t="inlineStr">
-        <is>
-          <t>String</t>
-        </is>
-      </c>
-      <c r="E147" s="2" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+          <t>ACCOUNT_NOT_FOUND</t>
+        </is>
+      </c>
+      <c r="D147" s="2" t="inlineStr"/>
+      <c r="E147" s="2" t="inlineStr"/>
       <c r="F147" s="2" t="inlineStr">
         <is>
-          <t>Bearer {JWT}</t>
-        </is>
-      </c>
-      <c r="G147" s="2" t="inlineStr">
-        <is>
-          <t>Bearer eyJ...</t>
-        </is>
-      </c>
+          <t>계좌 없음</t>
+        </is>
+      </c>
+      <c r="G147" s="2" t="inlineStr"/>
     </row>
     <row r="148">
       <c r="A148" s="2" t="inlineStr">
@@ -9320,7 +9357,7 @@
       </c>
       <c r="C148" s="2" t="inlineStr">
         <is>
-          <t>Query from</t>
+          <t>Header Authorization</t>
         </is>
       </c>
       <c r="D148" s="2" t="inlineStr">
@@ -9335,12 +9372,12 @@
       </c>
       <c r="F148" s="2" t="inlineStr">
         <is>
-          <t>시작일(yyyy-MM-dd)</t>
+          <t>Bearer {JWT}</t>
         </is>
       </c>
       <c r="G148" s="2" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>Bearer eyJ...</t>
         </is>
       </c>
     </row>
@@ -9357,7 +9394,7 @@
       </c>
       <c r="C149" s="2" t="inlineStr">
         <is>
-          <t>Query to</t>
+          <t>Query from</t>
         </is>
       </c>
       <c r="D149" s="2" t="inlineStr">
@@ -9372,12 +9409,12 @@
       </c>
       <c r="F149" s="2" t="inlineStr">
         <is>
-          <t>종료일(yyyy-MM-dd)</t>
+          <t>시작일(yyyy-MM-dd)</t>
         </is>
       </c>
       <c r="G149" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-09-01</t>
         </is>
       </c>
     </row>
@@ -9394,25 +9431,29 @@
       </c>
       <c r="C150" s="2" t="inlineStr">
         <is>
-          <t>Query cursor</t>
+          <t>Query to</t>
         </is>
       </c>
       <c r="D150" s="2" t="inlineStr">
         <is>
-          <t>Long</t>
+          <t>String</t>
         </is>
       </c>
       <c r="E150" s="2" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="F150" s="2" t="inlineStr">
         <is>
-          <t>E-09와 같은 커서 규칙</t>
-        </is>
-      </c>
-      <c r="G150" s="2" t="inlineStr"/>
+          <t>종료일(yyyy-MM-dd)</t>
+        </is>
+      </c>
+      <c r="G150" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
     </row>
     <row r="151">
       <c r="A151" s="2" t="inlineStr">
@@ -9427,12 +9468,12 @@
       </c>
       <c r="C151" s="2" t="inlineStr">
         <is>
-          <t>Query size</t>
+          <t>Query cursor</t>
         </is>
       </c>
       <c r="D151" s="2" t="inlineStr">
         <is>
-          <t>Integer</t>
+          <t>Long</t>
         </is>
       </c>
       <c r="E151" s="2" t="inlineStr">
@@ -9442,14 +9483,10 @@
       </c>
       <c r="F151" s="2" t="inlineStr">
         <is>
-          <t>기본 20</t>
-        </is>
-      </c>
-      <c r="G151" s="2" t="inlineStr">
-        <is>
-          <t>20</t>
-        </is>
-      </c>
+          <t>E-09와 같은 커서 규칙</t>
+        </is>
+      </c>
+      <c r="G151" s="2" t="inlineStr"/>
     </row>
     <row r="152">
       <c r="A152" s="2" t="inlineStr">
@@ -9459,32 +9496,32 @@
       </c>
       <c r="B152" s="2" t="inlineStr">
         <is>
-          <t>응답</t>
+          <t>요청</t>
         </is>
       </c>
       <c r="C152" s="2" t="inlineStr">
         <is>
-          <t>data.sentTotal</t>
+          <t>Query size</t>
         </is>
       </c>
       <c r="D152" s="2" t="inlineStr">
         <is>
-          <t>Long</t>
+          <t>Integer</t>
         </is>
       </c>
       <c r="E152" s="2" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="F152" s="2" t="inlineStr">
         <is>
-          <t>기간 내 보낸 합계(원, Spring 계산)</t>
+          <t>기본 20</t>
         </is>
       </c>
       <c r="G152" s="2" t="inlineStr">
         <is>
-          <t>230000</t>
+          <t>20</t>
         </is>
       </c>
     </row>
@@ -9501,7 +9538,7 @@
       </c>
       <c r="C153" s="2" t="inlineStr">
         <is>
-          <t>data.receivedTotal</t>
+          <t>data.sentTotal</t>
         </is>
       </c>
       <c r="D153" s="2" t="inlineStr">
@@ -9516,12 +9553,12 @@
       </c>
       <c r="F153" s="2" t="inlineStr">
         <is>
-          <t>기간 내 받은 합계(원, Spring 계산)</t>
+          <t>기간 내 보낸 합계(원, Spring 계산)</t>
         </is>
       </c>
       <c r="G153" s="2" t="inlineStr">
         <is>
-          <t>50000</t>
+          <t>230000</t>
         </is>
       </c>
     </row>
@@ -9538,12 +9575,12 @@
       </c>
       <c r="C154" s="2" t="inlineStr">
         <is>
-          <t>data.count</t>
+          <t>data.receivedTotal</t>
         </is>
       </c>
       <c r="D154" s="2" t="inlineStr">
         <is>
-          <t>Integer</t>
+          <t>Long</t>
         </is>
       </c>
       <c r="E154" s="2" t="inlineStr">
@@ -9553,12 +9590,12 @@
       </c>
       <c r="F154" s="2" t="inlineStr">
         <is>
-          <t>기간 내 건수</t>
+          <t>기간 내 받은 합계(원, Spring 계산)</t>
         </is>
       </c>
       <c r="G154" s="2" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>50000</t>
         </is>
       </c>
     </row>
@@ -9575,12 +9612,12 @@
       </c>
       <c r="C155" s="2" t="inlineStr">
         <is>
-          <t>data.items[].transferId</t>
+          <t>data.count</t>
         </is>
       </c>
       <c r="D155" s="2" t="inlineStr">
         <is>
-          <t>Long</t>
+          <t>Integer</t>
         </is>
       </c>
       <c r="E155" s="2" t="inlineStr">
@@ -9590,12 +9627,12 @@
       </c>
       <c r="F155" s="2" t="inlineStr">
         <is>
-          <t>송금 ID</t>
+          <t>기간 내 건수</t>
         </is>
       </c>
       <c r="G155" s="2" t="inlineStr">
         <is>
-          <t>1024</t>
+          <t>7</t>
         </is>
       </c>
     </row>
@@ -9612,12 +9649,12 @@
       </c>
       <c r="C156" s="2" t="inlineStr">
         <is>
-          <t>data.items[].direction</t>
+          <t>data.items[].transferId</t>
         </is>
       </c>
       <c r="D156" s="2" t="inlineStr">
         <is>
-          <t>String</t>
+          <t>Long</t>
         </is>
       </c>
       <c r="E156" s="2" t="inlineStr">
@@ -9627,12 +9664,12 @@
       </c>
       <c r="F156" s="2" t="inlineStr">
         <is>
-          <t>SENT / RECEIVED</t>
+          <t>송금 ID</t>
         </is>
       </c>
       <c r="G156" s="2" t="inlineStr">
         <is>
-          <t>SENT</t>
+          <t>1024</t>
         </is>
       </c>
     </row>
@@ -9649,7 +9686,7 @@
       </c>
       <c r="C157" s="2" t="inlineStr">
         <is>
-          <t>data.items[].counterpartName</t>
+          <t>data.items[].direction</t>
         </is>
       </c>
       <c r="D157" s="2" t="inlineStr">
@@ -9664,12 +9701,12 @@
       </c>
       <c r="F157" s="2" t="inlineStr">
         <is>
-          <t>상대 이름</t>
+          <t>SENT / RECEIVED</t>
         </is>
       </c>
       <c r="G157" s="2" t="inlineStr">
         <is>
-          <t>김영희</t>
+          <t>SENT</t>
         </is>
       </c>
     </row>
@@ -9686,7 +9723,7 @@
       </c>
       <c r="C158" s="2" t="inlineStr">
         <is>
-          <t>data.items[].counterpartAccountNumber</t>
+          <t>data.items[].counterpartName</t>
         </is>
       </c>
       <c r="D158" s="2" t="inlineStr">
@@ -9701,12 +9738,12 @@
       </c>
       <c r="F158" s="2" t="inlineStr">
         <is>
-          <t>상대 계좌</t>
+          <t>상대 이름</t>
         </is>
       </c>
       <c r="G158" s="2" t="inlineStr">
         <is>
-          <t>123456789012</t>
+          <t>김영희</t>
         </is>
       </c>
     </row>
@@ -9723,12 +9760,12 @@
       </c>
       <c r="C159" s="2" t="inlineStr">
         <is>
-          <t>data.items[].amount</t>
+          <t>data.items[].counterpartAccountNumber</t>
         </is>
       </c>
       <c r="D159" s="2" t="inlineStr">
         <is>
-          <t>Long</t>
+          <t>String</t>
         </is>
       </c>
       <c r="E159" s="2" t="inlineStr">
@@ -9738,12 +9775,12 @@
       </c>
       <c r="F159" s="2" t="inlineStr">
         <is>
-          <t>금액(원)</t>
+          <t>상대 계좌</t>
         </is>
       </c>
       <c r="G159" s="2" t="inlineStr">
         <is>
-          <t>10000</t>
+          <t>123456789012</t>
         </is>
       </c>
     </row>
@@ -9760,12 +9797,12 @@
       </c>
       <c r="C160" s="2" t="inlineStr">
         <is>
-          <t>data.items[].createdAt</t>
+          <t>data.items[].amount</t>
         </is>
       </c>
       <c r="D160" s="2" t="inlineStr">
         <is>
-          <t>String</t>
+          <t>Long</t>
         </is>
       </c>
       <c r="E160" s="2" t="inlineStr">
@@ -9775,12 +9812,12 @@
       </c>
       <c r="F160" s="2" t="inlineStr">
         <is>
-          <t>시각(ISO-8601)</t>
+          <t>금액(원)</t>
         </is>
       </c>
       <c r="G160" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T10:01:00+09:00</t>
+          <t>10000</t>
         </is>
       </c>
     </row>
@@ -9797,27 +9834,27 @@
       </c>
       <c r="C161" s="2" t="inlineStr">
         <is>
-          <t>data.nextCursor</t>
+          <t>data.items[].createdAt</t>
         </is>
       </c>
       <c r="D161" s="2" t="inlineStr">
         <is>
-          <t>Long</t>
+          <t>String</t>
         </is>
       </c>
       <c r="E161" s="2" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="F161" s="2" t="inlineStr">
         <is>
-          <t>다음 요청의 cursor(마지막 transferId). 없으면 null</t>
+          <t>시각(ISO-8601)</t>
         </is>
       </c>
       <c r="G161" s="2" t="inlineStr">
         <is>
-          <t>1005</t>
+          <t>2026-09-27T10:01:00+09:00</t>
         </is>
       </c>
     </row>
@@ -9834,27 +9871,27 @@
       </c>
       <c r="C162" s="2" t="inlineStr">
         <is>
-          <t>data.hasNext</t>
+          <t>data.nextCursor</t>
         </is>
       </c>
       <c r="D162" s="2" t="inlineStr">
         <is>
-          <t>Boolean</t>
+          <t>Long</t>
         </is>
       </c>
       <c r="E162" s="2" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="F162" s="2" t="inlineStr">
         <is>
-          <t>다음 묶음 존재 여부</t>
+          <t>다음 요청의 cursor(마지막 transferId). 없으면 null</t>
         </is>
       </c>
       <c r="G162" s="2" t="inlineStr">
         <is>
-          <t>true</t>
+          <t>1005</t>
         </is>
       </c>
     </row>
@@ -9866,25 +9903,62 @@
       </c>
       <c r="B163" s="2" t="inlineStr">
         <is>
+          <t>응답</t>
+        </is>
+      </c>
+      <c r="C163" s="2" t="inlineStr">
+        <is>
+          <t>data.hasNext</t>
+        </is>
+      </c>
+      <c r="D163" s="2" t="inlineStr">
+        <is>
+          <t>Boolean</t>
+        </is>
+      </c>
+      <c r="E163" s="2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="F163" s="2" t="inlineStr">
+        <is>
+          <t>다음 묶음 존재 여부</t>
+        </is>
+      </c>
+      <c r="G163" s="2" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" s="2" t="inlineStr">
+        <is>
+          <t>I-04</t>
+        </is>
+      </c>
+      <c r="B164" s="2" t="inlineStr">
+        <is>
           <t>에러</t>
         </is>
       </c>
-      <c r="C163" s="2" t="inlineStr">
+      <c r="C164" s="2" t="inlineStr">
         <is>
           <t>AUTH_INVALID</t>
         </is>
       </c>
-      <c r="D163" s="2" t="inlineStr"/>
-      <c r="E163" s="2" t="inlineStr"/>
-      <c r="F163" s="2" t="inlineStr">
+      <c r="D164" s="2" t="inlineStr"/>
+      <c r="E164" s="2" t="inlineStr"/>
+      <c r="F164" s="2" t="inlineStr">
         <is>
           <t>JWT 없음·만료·위조, 로그인 실패</t>
         </is>
       </c>
-      <c r="G163" s="2" t="inlineStr"/>
+      <c r="G164" s="2" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G163"/>
+  <autoFilter ref="A1:G164"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
feat(account): 계좌 충전 (#7) (#9)
* feat(account): 원자적 잔액 증가 쿼리 추가 (#7)

* feat(account): 계좌 충전 API (#7)

* test(account): 계좌 충전 통합 테스트 — 동시 충전 정합성 포함 (#7)

* fix(account): 충전 금액 0 이하 거부 — 리뷰 반영 (#7)
</commit_message>
<xml_diff>
--- a/docs/smart-spec.xlsx
+++ b/docs/smart-spec.xlsx
@@ -14,8 +14,8 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'요구사항'!$A$1:$G$71</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'API 목록'!$A$30:$H$47</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'API 상세'!$A$1:$G$164</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'API 목록'!$A$31:$H$48</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'API 상세'!$A$1:$G$165</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -3040,7 +3040,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H47"/>
+  <dimension ref="A1:H48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -3250,15 +3250,15 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>INSUFFICIENT_BALANCE</t>
+          <t>INVALID_AMOUNT</t>
         </is>
       </c>
       <c r="B14" s="2" t="n">
-        <v>409</v>
+        <v>400</v>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>잔액 부족</t>
+          <t>충전 금액이 0 이하</t>
         </is>
       </c>
       <c r="D14" s="9" t="n"/>
@@ -3270,15 +3270,15 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>ALIAS_NOT_FOUND</t>
+          <t>INSUFFICIENT_BALANCE</t>
         </is>
       </c>
       <c r="B15" s="2" t="n">
-        <v>404</v>
+        <v>409</v>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>등록되지 않은 별칭</t>
+          <t>잔액 부족</t>
         </is>
       </c>
       <c r="D15" s="9" t="n"/>
@@ -3290,7 +3290,7 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>TRANSFER_REQUEST_NOT_FOUND</t>
+          <t>ALIAS_NOT_FOUND</t>
         </is>
       </c>
       <c r="B16" s="2" t="n">
@@ -3298,7 +3298,7 @@
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>송금 요청 없음(또는 남의 요청)</t>
+          <t>등록되지 않은 별칭</t>
         </is>
       </c>
       <c r="D16" s="9" t="n"/>
@@ -3310,15 +3310,15 @@
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>TRANSFER_REQUEST_EXPIRED</t>
+          <t>TRANSFER_REQUEST_NOT_FOUND</t>
         </is>
       </c>
       <c r="B17" s="2" t="n">
-        <v>410</v>
+        <v>404</v>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>송금 요청 5분 만료</t>
+          <t>송금 요청 없음(또는 남의 요청)</t>
         </is>
       </c>
       <c r="D17" s="9" t="n"/>
@@ -3330,15 +3330,15 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>TRANSFER_REQUEST_ALREADY_USED</t>
+          <t>TRANSFER_REQUEST_EXPIRED</t>
         </is>
       </c>
       <c r="B18" s="2" t="n">
-        <v>409</v>
+        <v>410</v>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>이미 확정된 송금 요청</t>
+          <t>송금 요청 5분 만료</t>
         </is>
       </c>
       <c r="D18" s="9" t="n"/>
@@ -3350,15 +3350,15 @@
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>THREAD_NOT_FOUND</t>
+          <t>TRANSFER_REQUEST_ALREADY_USED</t>
         </is>
       </c>
       <c r="B19" s="2" t="n">
-        <v>404</v>
+        <v>409</v>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>대화 없음(또는 남의 대화)</t>
+          <t>이미 확정된 송금 요청</t>
         </is>
       </c>
       <c r="D19" s="9" t="n"/>
@@ -3370,7 +3370,7 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>DETAIL_NOT_FOUND</t>
+          <t>THREAD_NOT_FOUND</t>
         </is>
       </c>
       <c r="B20" s="2" t="n">
@@ -3378,7 +3378,7 @@
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>상세 보기 대상 없음(또는 남의 것)</t>
+          <t>대화 없음(또는 남의 대화)</t>
         </is>
       </c>
       <c r="D20" s="9" t="n"/>
@@ -3390,15 +3390,15 @@
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>AI_SERVER_UNAVAILABLE</t>
+          <t>DETAIL_NOT_FOUND</t>
         </is>
       </c>
       <c r="B21" s="2" t="n">
-        <v>503</v>
+        <v>404</v>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>FastAPI 장애·지연 — 채팅만 실패, 송금·계좌는 정상(장애 격리)</t>
+          <t>상세 보기 대상 없음(또는 남의 것)</t>
         </is>
       </c>
       <c r="D21" s="9" t="n"/>
@@ -3410,15 +3410,15 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>RATE_LIMITED</t>
+          <t>AI_SERVER_UNAVAILABLE</t>
         </is>
       </c>
       <c r="B22" s="2" t="n">
-        <v>429</v>
+        <v>503</v>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>사용자별 채팅 호출 제한 초과</t>
+          <t>FastAPI 장애·지연 — 채팅만 실패, 송금·계좌는 정상(장애 격리)</t>
         </is>
       </c>
       <c r="D22" s="9" t="n"/>
@@ -3428,17 +3428,19 @@
       <c r="H22" s="10" t="n"/>
     </row>
     <row r="23">
-      <c r="A23" s="8" t="inlineStr">
-        <is>
-          <t>guard 코드</t>
-        </is>
-      </c>
-      <c r="B23" s="8" t="inlineStr">
-        <is>
-          <t>설명</t>
-        </is>
-      </c>
-      <c r="C23" s="9" t="n"/>
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>RATE_LIMITED</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="n">
+        <v>429</v>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>사용자별 채팅 호출 제한 초과</t>
+        </is>
+      </c>
       <c r="D23" s="9" t="n"/>
       <c r="E23" s="9" t="n"/>
       <c r="F23" s="9" t="n"/>
@@ -3446,14 +3448,14 @@
       <c r="H23" s="10" t="n"/>
     </row>
     <row r="24">
-      <c r="A24" s="2" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="B24" s="2" t="inlineStr">
-        <is>
-          <t>통과</t>
+      <c r="A24" s="8" t="inlineStr">
+        <is>
+          <t>guard 코드</t>
+        </is>
+      </c>
+      <c r="B24" s="8" t="inlineStr">
+        <is>
+          <t>설명</t>
         </is>
       </c>
       <c r="C24" s="9" t="n"/>
@@ -3466,12 +3468,12 @@
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>INJECTION</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>입력 차단 — 프롬프트 인젝션 대표 유형. LLM 미호출, 고정 문장</t>
+          <t>통과</t>
         </is>
       </c>
       <c r="C25" s="9" t="n"/>
@@ -3484,12 +3486,12 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>NUMBER_UNVERIFIED</t>
+          <t>INJECTION</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>출력 교체 — 근거(재무 테이블)에 없는 숫자</t>
+          <t>입력 차단 — 프롬프트 인젝션 대표 유형. LLM 미호출, 고정 문장</t>
         </is>
       </c>
       <c r="C26" s="9" t="n"/>
@@ -3502,12 +3504,12 @@
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>ADVICE</t>
+          <t>NUMBER_UNVERIFIED</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>출력 교체 — 투자 권유 표현</t>
+          <t>출력 교체 — 근거(재무 테이블)에 없는 숫자</t>
         </is>
       </c>
       <c r="C27" s="9" t="n"/>
@@ -3520,12 +3522,12 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>PROMPT_LEAK</t>
+          <t>ADVICE</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>출력 교체 — 시스템 프롬프트 카나리 단어 노출</t>
+          <t>출력 교체 — 투자 권유 표현</t>
         </is>
       </c>
       <c r="C28" s="9" t="n"/>
@@ -3535,90 +3537,71 @@
       <c r="G28" s="9" t="n"/>
       <c r="H28" s="10" t="n"/>
     </row>
-    <row r="30">
-      <c r="A30" s="1" t="inlineStr">
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>PROMPT_LEAK</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>출력 교체 — 시스템 프롬프트 카나리 단어 노출</t>
+        </is>
+      </c>
+      <c r="C29" s="9" t="n"/>
+      <c r="D29" s="9" t="n"/>
+      <c r="E29" s="9" t="n"/>
+      <c r="F29" s="9" t="n"/>
+      <c r="G29" s="9" t="n"/>
+      <c r="H29" s="10" t="n"/>
+    </row>
+    <row r="30"/>
+    <row r="31">
+      <c r="A31" s="1" t="inlineStr">
         <is>
           <t>API ID</t>
         </is>
       </c>
-      <c r="B30" s="1" t="inlineStr">
+      <c r="B31" s="1" t="inlineStr">
         <is>
           <t>구분</t>
         </is>
       </c>
-      <c r="C30" s="1" t="inlineStr">
+      <c r="C31" s="1" t="inlineStr">
         <is>
           <t>Method</t>
         </is>
       </c>
-      <c r="D30" s="1" t="inlineStr">
+      <c r="D31" s="1" t="inlineStr">
         <is>
           <t>URL</t>
         </is>
       </c>
-      <c r="E30" s="1" t="inlineStr">
+      <c r="E31" s="1" t="inlineStr">
         <is>
           <t>설명</t>
         </is>
       </c>
-      <c r="F30" s="1" t="inlineStr">
+      <c r="F31" s="1" t="inlineStr">
         <is>
           <t>인증</t>
         </is>
       </c>
-      <c r="G30" s="1" t="inlineStr">
+      <c r="G31" s="1" t="inlineStr">
         <is>
           <t>요구사항 ID</t>
         </is>
       </c>
-      <c r="H30" s="1" t="inlineStr">
+      <c r="H31" s="1" t="inlineStr">
         <is>
           <t>비고</t>
         </is>
       </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="2" t="inlineStr">
-        <is>
-          <t>E-01</t>
-        </is>
-      </c>
-      <c r="B31" s="2" t="inlineStr">
-        <is>
-          <t>외부</t>
-        </is>
-      </c>
-      <c r="C31" s="2" t="inlineStr">
-        <is>
-          <t>POST</t>
-        </is>
-      </c>
-      <c r="D31" s="2" t="inlineStr">
-        <is>
-          <t>/api/v1/auth/signup</t>
-        </is>
-      </c>
-      <c r="E31" s="2" t="inlineStr">
-        <is>
-          <t>회원가입</t>
-        </is>
-      </c>
-      <c r="F31" s="2" t="inlineStr">
-        <is>
-          <t>없음</t>
-        </is>
-      </c>
-      <c r="G31" s="2" t="inlineStr">
-        <is>
-          <t>FR-001</t>
-        </is>
-      </c>
-      <c r="H31" s="2" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>E-02</t>
+          <t>E-01</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
@@ -3633,12 +3616,12 @@
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>/api/v1/auth/login</t>
+          <t>/api/v1/auth/signup</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>로그인</t>
+          <t>회원가입</t>
         </is>
       </c>
       <c r="F32" s="2" t="inlineStr">
@@ -3648,7 +3631,7 @@
       </c>
       <c r="G32" s="2" t="inlineStr">
         <is>
-          <t>FR-002</t>
+          <t>FR-001</t>
         </is>
       </c>
       <c r="H32" s="2" t="inlineStr"/>
@@ -3656,7 +3639,7 @@
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>E-03</t>
+          <t>E-02</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
@@ -3671,34 +3654,30 @@
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>/api/v1/accounts</t>
+          <t>/api/v1/auth/login</t>
         </is>
       </c>
       <c r="E33" s="2" t="inlineStr">
         <is>
-          <t>가상계좌 개설</t>
+          <t>로그인</t>
         </is>
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
-          <t>Bearer</t>
+          <t>없음</t>
         </is>
       </c>
       <c r="G33" s="2" t="inlineStr">
         <is>
-          <t>FR-003, FR-004</t>
-        </is>
-      </c>
-      <c r="H33" s="2" t="inlineStr">
-        <is>
-          <t>첫 계좌면 대표. Idempotency-Key 헤더 필수 — 같은 키 재요청 시 새 계좌를 만들지 않고 기존 계좌를 반환</t>
-        </is>
-      </c>
+          <t>FR-002</t>
+        </is>
+      </c>
+      <c r="H33" s="2" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>E-04</t>
+          <t>E-03</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
@@ -3708,7 +3687,7 @@
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>GET</t>
+          <t>POST</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
@@ -3718,7 +3697,7 @@
       </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>내 계좌·잔액 조회</t>
+          <t>가상계좌 개설</t>
         </is>
       </c>
       <c r="F34" s="2" t="inlineStr">
@@ -3728,15 +3707,19 @@
       </c>
       <c r="G34" s="2" t="inlineStr">
         <is>
-          <t>FR-006</t>
-        </is>
-      </c>
-      <c r="H34" s="2" t="inlineStr"/>
+          <t>FR-003, FR-004</t>
+        </is>
+      </c>
+      <c r="H34" s="2" t="inlineStr">
+        <is>
+          <t>첫 계좌면 대표. Idempotency-Key 헤더 필수 — 같은 키 재요청 시 새 계좌를 만들지 않고 기존 계좌를 반환</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>E-05</t>
+          <t>E-04</t>
         </is>
       </c>
       <c r="B35" s="2" t="inlineStr">
@@ -3746,17 +3729,17 @@
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>PATCH</t>
+          <t>GET</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>/api/v1/accounts/{accountId}/primary</t>
+          <t>/api/v1/accounts</t>
         </is>
       </c>
       <c r="E35" s="2" t="inlineStr">
         <is>
-          <t>대표 계좌 변경</t>
+          <t>내 계좌·잔액 조회</t>
         </is>
       </c>
       <c r="F35" s="2" t="inlineStr">
@@ -3766,7 +3749,7 @@
       </c>
       <c r="G35" s="2" t="inlineStr">
         <is>
-          <t>FR-004</t>
+          <t>FR-006</t>
         </is>
       </c>
       <c r="H35" s="2" t="inlineStr"/>
@@ -3774,7 +3757,7 @@
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>E-06</t>
+          <t>E-05</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
@@ -3784,17 +3767,17 @@
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>POST</t>
+          <t>PATCH</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>/api/v1/accounts/{accountId}/charge</t>
+          <t>/api/v1/accounts/{accountId}/primary</t>
         </is>
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t>충전</t>
+          <t>대표 계좌 변경</t>
         </is>
       </c>
       <c r="F36" s="2" t="inlineStr">
@@ -3804,7 +3787,7 @@
       </c>
       <c r="G36" s="2" t="inlineStr">
         <is>
-          <t>FR-005</t>
+          <t>FR-004</t>
         </is>
       </c>
       <c r="H36" s="2" t="inlineStr"/>
@@ -3812,7 +3795,7 @@
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>E-07</t>
+          <t>E-06</t>
         </is>
       </c>
       <c r="B37" s="2" t="inlineStr">
@@ -3827,12 +3810,12 @@
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>/api/v1/aliases</t>
+          <t>/api/v1/accounts/{accountId}/charge</t>
         </is>
       </c>
       <c r="E37" s="2" t="inlineStr">
         <is>
-          <t>별칭 등록</t>
+          <t>충전</t>
         </is>
       </c>
       <c r="F37" s="2" t="inlineStr">
@@ -3842,7 +3825,7 @@
       </c>
       <c r="G37" s="2" t="inlineStr">
         <is>
-          <t>FR-007</t>
+          <t>FR-005</t>
         </is>
       </c>
       <c r="H37" s="2" t="inlineStr"/>
@@ -3850,7 +3833,7 @@
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>E-08</t>
+          <t>E-07</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
@@ -3860,7 +3843,7 @@
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>GET</t>
+          <t>POST</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
@@ -3870,7 +3853,7 @@
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>별칭 목록</t>
+          <t>별칭 등록</t>
         </is>
       </c>
       <c r="F38" s="2" t="inlineStr">
@@ -3880,7 +3863,7 @@
       </c>
       <c r="G38" s="2" t="inlineStr">
         <is>
-          <t>FR-008</t>
+          <t>FR-007</t>
         </is>
       </c>
       <c r="H38" s="2" t="inlineStr"/>
@@ -3888,7 +3871,7 @@
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>E-09</t>
+          <t>E-08</t>
         </is>
       </c>
       <c r="B39" s="2" t="inlineStr">
@@ -3903,12 +3886,12 @@
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>/api/v1/transfers?cursor&amp;size</t>
+          <t>/api/v1/aliases</t>
         </is>
       </c>
       <c r="E39" s="2" t="inlineStr">
         <is>
-          <t>송금 내역 목록</t>
+          <t>별칭 목록</t>
         </is>
       </c>
       <c r="F39" s="2" t="inlineStr">
@@ -3918,19 +3901,15 @@
       </c>
       <c r="G39" s="2" t="inlineStr">
         <is>
-          <t>FR-011</t>
-        </is>
-      </c>
-      <c r="H39" s="2" t="inlineStr">
-        <is>
-          <t>최종 형태(커서). 개선 흐름: 전체 조회 → 오프셋 → 커서</t>
-        </is>
-      </c>
+          <t>FR-008</t>
+        </is>
+      </c>
+      <c r="H39" s="2" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>E-10</t>
+          <t>E-09</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
@@ -3940,17 +3919,17 @@
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>POST</t>
+          <t>GET</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>/api/v1/chat/threads</t>
+          <t>/api/v1/transfers?cursor&amp;size</t>
         </is>
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>새 대화</t>
+          <t>송금 내역 목록</t>
         </is>
       </c>
       <c r="F40" s="2" t="inlineStr">
@@ -3960,15 +3939,19 @@
       </c>
       <c r="G40" s="2" t="inlineStr">
         <is>
-          <t>FR-013</t>
-        </is>
-      </c>
-      <c r="H40" s="2" t="inlineStr"/>
+          <t>FR-011</t>
+        </is>
+      </c>
+      <c r="H40" s="2" t="inlineStr">
+        <is>
+          <t>최종 형태(커서). 개선 흐름: 전체 조회 → 오프셋 → 커서</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>E-11</t>
+          <t>E-10</t>
         </is>
       </c>
       <c r="B41" s="2" t="inlineStr">
@@ -3983,12 +3966,12 @@
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
-          <t>/api/v1/chat/threads/{threadId}/messages</t>
+          <t>/api/v1/chat/threads</t>
         </is>
       </c>
       <c r="E41" s="2" t="inlineStr">
         <is>
-          <t>채팅 메시지</t>
+          <t>새 대화</t>
         </is>
       </c>
       <c r="F41" s="2" t="inlineStr">
@@ -3998,19 +3981,15 @@
       </c>
       <c r="G41" s="2" t="inlineStr">
         <is>
-          <t>FR-014, FR-015, FR-009, FR-012, FR-017, FR-018, FR-019, NFR-003, NFR-019, NFR-024</t>
-        </is>
-      </c>
-      <c r="H41" s="2" t="inlineStr">
-        <is>
-          <t>Spring이 I-01 호출. 호출 제한 적용</t>
-        </is>
-      </c>
+          <t>FR-013</t>
+        </is>
+      </c>
+      <c r="H41" s="2" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>E-12</t>
+          <t>E-11</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
@@ -4025,12 +4004,12 @@
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>/api/v1/transfer-requests/{requestId}/confirm</t>
+          <t>/api/v1/chat/threads/{threadId}/messages</t>
         </is>
       </c>
       <c r="E42" s="2" t="inlineStr">
         <is>
-          <t>송금 확정([보내기])</t>
+          <t>채팅 메시지</t>
         </is>
       </c>
       <c r="F42" s="2" t="inlineStr">
@@ -4040,19 +4019,19 @@
       </c>
       <c r="G42" s="2" t="inlineStr">
         <is>
-          <t>FR-010, NFR-001, NFR-009, NFR-010</t>
+          <t>FR-014, FR-015, FR-009, FR-012, FR-017, FR-018, FR-019, NFR-003, NFR-019, NFR-024</t>
         </is>
       </c>
       <c r="H42" s="2" t="inlineStr">
         <is>
-          <t>AI 경로를 거치지 않음</t>
+          <t>Spring이 I-01 호출. 호출 제한 적용</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>E-13</t>
+          <t>E-12</t>
         </is>
       </c>
       <c r="B43" s="2" t="inlineStr">
@@ -4062,17 +4041,17 @@
       </c>
       <c r="C43" s="2" t="inlineStr">
         <is>
-          <t>GET</t>
+          <t>POST</t>
         </is>
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>/api/v1/chat/details/{detailId}</t>
+          <t>/api/v1/transfer-requests/{requestId}/confirm</t>
         </is>
       </c>
       <c r="E43" s="2" t="inlineStr">
         <is>
-          <t>상세 보기</t>
+          <t>송금 확정([보내기])</t>
         </is>
       </c>
       <c r="F43" s="2" t="inlineStr">
@@ -4082,61 +4061,61 @@
       </c>
       <c r="G43" s="2" t="inlineStr">
         <is>
-          <t>FR-016, FR-019</t>
+          <t>FR-010, NFR-001, NFR-009, NFR-010</t>
         </is>
       </c>
       <c r="H43" s="2" t="inlineStr">
         <is>
-          <t>Spring이 I-02 호출</t>
+          <t>AI 경로를 거치지 않음</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>I-01</t>
+          <t>E-13</t>
         </is>
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>내부 Spring→FastAPI</t>
+          <t>외부</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>POST</t>
+          <t>GET</t>
         </is>
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>/internal/chat</t>
+          <t>/api/v1/chat/details/{detailId}</t>
         </is>
       </c>
       <c r="E44" s="2" t="inlineStr">
         <is>
-          <t>채팅 처리(LangGraph 구동)</t>
+          <t>상세 보기</t>
         </is>
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
-          <t>Bearer(사용자 JWT 전달)</t>
+          <t>Bearer</t>
         </is>
       </c>
       <c r="G44" s="2" t="inlineStr">
         <is>
-          <t>FR-014, FR-015, NFR-005, NFR-006</t>
+          <t>FR-016, FR-019</t>
         </is>
       </c>
       <c r="H44" s="2" t="inlineStr">
         <is>
-          <t>FastAPI 쪽 API</t>
+          <t>Spring이 I-02 호출</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>I-02</t>
+          <t>I-01</t>
         </is>
       </c>
       <c r="B45" s="2" t="inlineStr">
@@ -4146,17 +4125,17 @@
       </c>
       <c r="C45" s="2" t="inlineStr">
         <is>
-          <t>GET</t>
+          <t>POST</t>
         </is>
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t>/internal/details/{detailId}</t>
+          <t>/internal/chat</t>
         </is>
       </c>
       <c r="E45" s="2" t="inlineStr">
         <is>
-          <t>상세 보고서 생성</t>
+          <t>채팅 처리(LangGraph 구동)</t>
         </is>
       </c>
       <c r="F45" s="2" t="inlineStr">
@@ -4166,7 +4145,7 @@
       </c>
       <c r="G45" s="2" t="inlineStr">
         <is>
-          <t>FR-016, NFR-005, NFR-006</t>
+          <t>FR-014, FR-015, NFR-005, NFR-006</t>
         </is>
       </c>
       <c r="H45" s="2" t="inlineStr">
@@ -4178,27 +4157,27 @@
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>I-03</t>
+          <t>I-02</t>
         </is>
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>내부 FastAPI→Spring</t>
+          <t>내부 Spring→FastAPI</t>
         </is>
       </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t>POST</t>
+          <t>GET</t>
         </is>
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>/internal/transfer-requests</t>
+          <t>/internal/details/{detailId}</t>
         </is>
       </c>
       <c r="E46" s="2" t="inlineStr">
         <is>
-          <t>송금 요청 생성(확인 카드용)</t>
+          <t>상세 보고서 생성</t>
         </is>
       </c>
       <c r="F46" s="2" t="inlineStr">
@@ -4208,59 +4187,101 @@
       </c>
       <c r="G46" s="2" t="inlineStr">
         <is>
-          <t>FR-009, NFR-001, NFR-005, NFR-006</t>
+          <t>FR-016, NFR-005, NFR-006</t>
         </is>
       </c>
       <c r="H46" s="2" t="inlineStr">
         <is>
-          <t>LangGraph 도구. 실행은 하지 않음</t>
+          <t>FastAPI 쪽 API</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
+          <t>I-03</t>
+        </is>
+      </c>
+      <c r="B47" s="2" t="inlineStr">
+        <is>
+          <t>내부 FastAPI→Spring</t>
+        </is>
+      </c>
+      <c r="C47" s="2" t="inlineStr">
+        <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="D47" s="2" t="inlineStr">
+        <is>
+          <t>/internal/transfer-requests</t>
+        </is>
+      </c>
+      <c r="E47" s="2" t="inlineStr">
+        <is>
+          <t>송금 요청 생성(확인 카드용)</t>
+        </is>
+      </c>
+      <c r="F47" s="2" t="inlineStr">
+        <is>
+          <t>Bearer(사용자 JWT 전달)</t>
+        </is>
+      </c>
+      <c r="G47" s="2" t="inlineStr">
+        <is>
+          <t>FR-009, NFR-001, NFR-005, NFR-006</t>
+        </is>
+      </c>
+      <c r="H47" s="2" t="inlineStr">
+        <is>
+          <t>LangGraph 도구. 실행은 하지 않음</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="2" t="inlineStr">
+        <is>
           <t>I-04</t>
         </is>
       </c>
-      <c r="B47" s="2" t="inlineStr">
+      <c r="B48" s="2" t="inlineStr">
         <is>
           <t>내부 FastAPI→Spring</t>
         </is>
       </c>
-      <c r="C47" s="2" t="inlineStr">
+      <c r="C48" s="2" t="inlineStr">
         <is>
           <t>GET</t>
         </is>
       </c>
-      <c r="D47" s="2" t="inlineStr">
+      <c r="D48" s="2" t="inlineStr">
         <is>
           <t>/internal/transfers?from&amp;to&amp;cursor&amp;size</t>
         </is>
       </c>
-      <c r="E47" s="2" t="inlineStr">
+      <c r="E48" s="2" t="inlineStr">
         <is>
           <t>송금 내역·합계 조회</t>
         </is>
       </c>
-      <c r="F47" s="2" t="inlineStr">
+      <c r="F48" s="2" t="inlineStr">
         <is>
           <t>Bearer(사용자 JWT 전달)</t>
         </is>
       </c>
-      <c r="G47" s="2" t="inlineStr">
+      <c r="G48" s="2" t="inlineStr">
         <is>
           <t>FR-012, NFR-002, NFR-005, NFR-006</t>
         </is>
       </c>
-      <c r="H47" s="2" t="inlineStr">
+      <c r="H48" s="2" t="inlineStr">
         <is>
           <t>LangGraph 도구. 합계는 Spring 계산</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A30:H47"/>
+  <autoFilter ref="A31:H48"/>
   <mergeCells count="28">
     <mergeCell ref="C10:H10"/>
     <mergeCell ref="C16:H16"/>
@@ -4301,7 +4322,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G164"/>
+  <dimension ref="A1:G165"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -5602,39 +5623,27 @@
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>E-07</t>
+          <t>E-06</t>
         </is>
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>요청</t>
+          <t>에러</t>
         </is>
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t>Header Authorization</t>
-        </is>
-      </c>
-      <c r="D39" s="2" t="inlineStr">
-        <is>
-          <t>String</t>
-        </is>
-      </c>
-      <c r="E39" s="2" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+          <t>INVALID_AMOUNT</t>
+        </is>
+      </c>
+      <c r="D39" s="2" t="n"/>
+      <c r="E39" s="2" t="n"/>
       <c r="F39" s="2" t="inlineStr">
         <is>
-          <t>Bearer {JWT}</t>
-        </is>
-      </c>
-      <c r="G39" s="2" t="inlineStr">
-        <is>
-          <t>Bearer eyJ...</t>
-        </is>
-      </c>
+          <t>충전 금액이 0 이하</t>
+        </is>
+      </c>
+      <c r="G39" s="2" t="n"/>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -5649,7 +5658,7 @@
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>alias</t>
+          <t>Header Authorization</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
@@ -5664,12 +5673,12 @@
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>별칭</t>
+          <t>Bearer {JWT}</t>
         </is>
       </c>
       <c r="G40" s="2" t="inlineStr">
         <is>
-          <t>엄마</t>
+          <t>Bearer eyJ...</t>
         </is>
       </c>
     </row>
@@ -5686,7 +5695,7 @@
       </c>
       <c r="C41" s="2" t="inlineStr">
         <is>
-          <t>accountNumber</t>
+          <t>alias</t>
         </is>
       </c>
       <c r="D41" s="2" t="inlineStr">
@@ -5701,12 +5710,12 @@
       </c>
       <c r="F41" s="2" t="inlineStr">
         <is>
-          <t>상대 계좌번호</t>
+          <t>별칭</t>
         </is>
       </c>
       <c r="G41" s="2" t="inlineStr">
         <is>
-          <t>123456789012</t>
+          <t>엄마</t>
         </is>
       </c>
     </row>
@@ -5718,17 +5727,17 @@
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>응답</t>
+          <t>요청</t>
         </is>
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>data.aliasId</t>
+          <t>accountNumber</t>
         </is>
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>Long</t>
+          <t>String</t>
         </is>
       </c>
       <c r="E42" s="2" t="inlineStr">
@@ -5738,12 +5747,12 @@
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
-          <t>별칭 ID</t>
+          <t>상대 계좌번호</t>
         </is>
       </c>
       <c r="G42" s="2" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>123456789012</t>
         </is>
       </c>
     </row>
@@ -5760,12 +5769,12 @@
       </c>
       <c r="C43" s="2" t="inlineStr">
         <is>
-          <t>data.alias</t>
+          <t>data.aliasId</t>
         </is>
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>String</t>
+          <t>Long</t>
         </is>
       </c>
       <c r="E43" s="2" t="inlineStr">
@@ -5775,12 +5784,12 @@
       </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
-          <t>별칭</t>
+          <t>별칭 ID</t>
         </is>
       </c>
       <c r="G43" s="2" t="inlineStr">
         <is>
-          <t>엄마</t>
+          <t>3</t>
         </is>
       </c>
     </row>
@@ -5797,7 +5806,7 @@
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>data.accountNumber</t>
+          <t>data.alias</t>
         </is>
       </c>
       <c r="D44" s="2" t="inlineStr">
@@ -5812,12 +5821,12 @@
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
-          <t>계좌번호</t>
+          <t>별칭</t>
         </is>
       </c>
       <c r="G44" s="2" t="inlineStr">
         <is>
-          <t>123456789012</t>
+          <t>엄마</t>
         </is>
       </c>
     </row>
@@ -5834,7 +5843,7 @@
       </c>
       <c r="C45" s="2" t="inlineStr">
         <is>
-          <t>data.ownerName</t>
+          <t>data.accountNumber</t>
         </is>
       </c>
       <c r="D45" s="2" t="inlineStr">
@@ -5849,12 +5858,12 @@
       </c>
       <c r="F45" s="2" t="inlineStr">
         <is>
-          <t>예금주 이름</t>
+          <t>계좌번호</t>
         </is>
       </c>
       <c r="G45" s="2" t="inlineStr">
         <is>
-          <t>김영희</t>
+          <t>123456789012</t>
         </is>
       </c>
     </row>
@@ -5866,22 +5875,34 @@
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>에러</t>
+          <t>응답</t>
         </is>
       </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t>AUTH_INVALID</t>
-        </is>
-      </c>
-      <c r="D46" s="2" t="inlineStr"/>
-      <c r="E46" s="2" t="inlineStr"/>
+          <t>data.ownerName</t>
+        </is>
+      </c>
+      <c r="D46" s="2" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="E46" s="2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
-          <t>JWT 없음·만료·위조, 로그인 실패</t>
-        </is>
-      </c>
-      <c r="G46" s="2" t="inlineStr"/>
+          <t>예금주 이름</t>
+        </is>
+      </c>
+      <c r="G46" s="2" t="inlineStr">
+        <is>
+          <t>김영희</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
@@ -5896,14 +5917,14 @@
       </c>
       <c r="C47" s="2" t="inlineStr">
         <is>
-          <t>ACCOUNT_NOT_FOUND</t>
+          <t>AUTH_INVALID</t>
         </is>
       </c>
       <c r="D47" s="2" t="inlineStr"/>
       <c r="E47" s="2" t="inlineStr"/>
       <c r="F47" s="2" t="inlineStr">
         <is>
-          <t>계좌 없음</t>
+          <t>JWT 없음·만료·위조, 로그인 실패</t>
         </is>
       </c>
       <c r="G47" s="2" t="inlineStr"/>
@@ -5911,39 +5932,27 @@
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>E-08</t>
+          <t>E-07</t>
         </is>
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>요청</t>
+          <t>에러</t>
         </is>
       </c>
       <c r="C48" s="2" t="inlineStr">
         <is>
-          <t>Header Authorization</t>
-        </is>
-      </c>
-      <c r="D48" s="2" t="inlineStr">
-        <is>
-          <t>String</t>
-        </is>
-      </c>
-      <c r="E48" s="2" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+          <t>ACCOUNT_NOT_FOUND</t>
+        </is>
+      </c>
+      <c r="D48" s="2" t="inlineStr"/>
+      <c r="E48" s="2" t="inlineStr"/>
       <c r="F48" s="2" t="inlineStr">
         <is>
-          <t>Bearer {JWT}</t>
-        </is>
-      </c>
-      <c r="G48" s="2" t="inlineStr">
-        <is>
-          <t>Bearer eyJ...</t>
-        </is>
-      </c>
+          <t>계좌 없음</t>
+        </is>
+      </c>
+      <c r="G48" s="2" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
@@ -5953,17 +5962,17 @@
       </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
-          <t>응답</t>
+          <t>요청</t>
         </is>
       </c>
       <c r="C49" s="2" t="inlineStr">
         <is>
-          <t>data.aliases[].aliasId</t>
+          <t>Header Authorization</t>
         </is>
       </c>
       <c r="D49" s="2" t="inlineStr">
         <is>
-          <t>Long</t>
+          <t>String</t>
         </is>
       </c>
       <c r="E49" s="2" t="inlineStr">
@@ -5973,12 +5982,12 @@
       </c>
       <c r="F49" s="2" t="inlineStr">
         <is>
-          <t>별칭 ID</t>
+          <t>Bearer {JWT}</t>
         </is>
       </c>
       <c r="G49" s="2" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>Bearer eyJ...</t>
         </is>
       </c>
     </row>
@@ -5995,12 +6004,12 @@
       </c>
       <c r="C50" s="2" t="inlineStr">
         <is>
-          <t>data.aliases[].alias</t>
+          <t>data.aliases[].aliasId</t>
         </is>
       </c>
       <c r="D50" s="2" t="inlineStr">
         <is>
-          <t>String</t>
+          <t>Long</t>
         </is>
       </c>
       <c r="E50" s="2" t="inlineStr">
@@ -6010,12 +6019,12 @@
       </c>
       <c r="F50" s="2" t="inlineStr">
         <is>
-          <t>별칭</t>
+          <t>별칭 ID</t>
         </is>
       </c>
       <c r="G50" s="2" t="inlineStr">
         <is>
-          <t>엄마</t>
+          <t>3</t>
         </is>
       </c>
     </row>
@@ -6032,7 +6041,7 @@
       </c>
       <c r="C51" s="2" t="inlineStr">
         <is>
-          <t>data.aliases[].accountNumber</t>
+          <t>data.aliases[].alias</t>
         </is>
       </c>
       <c r="D51" s="2" t="inlineStr">
@@ -6047,12 +6056,12 @@
       </c>
       <c r="F51" s="2" t="inlineStr">
         <is>
-          <t>계좌번호</t>
+          <t>별칭</t>
         </is>
       </c>
       <c r="G51" s="2" t="inlineStr">
         <is>
-          <t>123456789012</t>
+          <t>엄마</t>
         </is>
       </c>
     </row>
@@ -6069,7 +6078,7 @@
       </c>
       <c r="C52" s="2" t="inlineStr">
         <is>
-          <t>data.aliases[].ownerName</t>
+          <t>data.aliases[].accountNumber</t>
         </is>
       </c>
       <c r="D52" s="2" t="inlineStr">
@@ -6084,12 +6093,12 @@
       </c>
       <c r="F52" s="2" t="inlineStr">
         <is>
-          <t>예금주 이름</t>
+          <t>계좌번호</t>
         </is>
       </c>
       <c r="G52" s="2" t="inlineStr">
         <is>
-          <t>김영희</t>
+          <t>123456789012</t>
         </is>
       </c>
     </row>
@@ -6101,59 +6110,59 @@
       </c>
       <c r="B53" s="2" t="inlineStr">
         <is>
-          <t>에러</t>
+          <t>응답</t>
         </is>
       </c>
       <c r="C53" s="2" t="inlineStr">
         <is>
-          <t>AUTH_INVALID</t>
-        </is>
-      </c>
-      <c r="D53" s="2" t="inlineStr"/>
-      <c r="E53" s="2" t="inlineStr"/>
+          <t>data.aliases[].ownerName</t>
+        </is>
+      </c>
+      <c r="D53" s="2" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="E53" s="2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="F53" s="2" t="inlineStr">
         <is>
-          <t>JWT 없음·만료·위조, 로그인 실패</t>
-        </is>
-      </c>
-      <c r="G53" s="2" t="inlineStr"/>
+          <t>예금주 이름</t>
+        </is>
+      </c>
+      <c r="G53" s="2" t="inlineStr">
+        <is>
+          <t>김영희</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>E-09</t>
+          <t>E-08</t>
         </is>
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>요청</t>
+          <t>에러</t>
         </is>
       </c>
       <c r="C54" s="2" t="inlineStr">
         <is>
-          <t>Header Authorization</t>
-        </is>
-      </c>
-      <c r="D54" s="2" t="inlineStr">
-        <is>
-          <t>String</t>
-        </is>
-      </c>
-      <c r="E54" s="2" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+          <t>AUTH_INVALID</t>
+        </is>
+      </c>
+      <c r="D54" s="2" t="inlineStr"/>
+      <c r="E54" s="2" t="inlineStr"/>
       <c r="F54" s="2" t="inlineStr">
         <is>
-          <t>Bearer {JWT}</t>
-        </is>
-      </c>
-      <c r="G54" s="2" t="inlineStr">
-        <is>
-          <t>Bearer eyJ...</t>
-        </is>
-      </c>
+          <t>JWT 없음·만료·위조, 로그인 실패</t>
+        </is>
+      </c>
+      <c r="G54" s="2" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
@@ -6168,27 +6177,27 @@
       </c>
       <c r="C55" s="2" t="inlineStr">
         <is>
-          <t>Query cursor</t>
+          <t>Header Authorization</t>
         </is>
       </c>
       <c r="D55" s="2" t="inlineStr">
         <is>
-          <t>Long</t>
+          <t>String</t>
         </is>
       </c>
       <c r="E55" s="2" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="F55" s="2" t="inlineStr">
         <is>
-          <t>이전 응답의 nextCursor. 없으면 최신부터</t>
+          <t>Bearer {JWT}</t>
         </is>
       </c>
       <c r="G55" s="2" t="inlineStr">
         <is>
-          <t>1025</t>
+          <t>Bearer eyJ...</t>
         </is>
       </c>
     </row>
@@ -6205,12 +6214,12 @@
       </c>
       <c r="C56" s="2" t="inlineStr">
         <is>
-          <t>Query size</t>
+          <t>Query cursor</t>
         </is>
       </c>
       <c r="D56" s="2" t="inlineStr">
         <is>
-          <t>Integer</t>
+          <t>Long</t>
         </is>
       </c>
       <c r="E56" s="2" t="inlineStr">
@@ -6220,12 +6229,12 @@
       </c>
       <c r="F56" s="2" t="inlineStr">
         <is>
-          <t>묶음 크기(기본 20)</t>
+          <t>이전 응답의 nextCursor. 없으면 최신부터</t>
         </is>
       </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>1025</t>
         </is>
       </c>
     </row>
@@ -6237,32 +6246,32 @@
       </c>
       <c r="B57" s="2" t="inlineStr">
         <is>
-          <t>응답</t>
+          <t>요청</t>
         </is>
       </c>
       <c r="C57" s="2" t="inlineStr">
         <is>
-          <t>data.items[].transferId</t>
+          <t>Query size</t>
         </is>
       </c>
       <c r="D57" s="2" t="inlineStr">
         <is>
-          <t>Long</t>
+          <t>Integer</t>
         </is>
       </c>
       <c r="E57" s="2" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="F57" s="2" t="inlineStr">
         <is>
-          <t>송금 ID</t>
+          <t>묶음 크기(기본 20)</t>
         </is>
       </c>
       <c r="G57" s="2" t="inlineStr">
         <is>
-          <t>1024</t>
+          <t>20</t>
         </is>
       </c>
     </row>
@@ -6279,12 +6288,12 @@
       </c>
       <c r="C58" s="2" t="inlineStr">
         <is>
-          <t>data.items[].direction</t>
+          <t>data.items[].transferId</t>
         </is>
       </c>
       <c r="D58" s="2" t="inlineStr">
         <is>
-          <t>String</t>
+          <t>Long</t>
         </is>
       </c>
       <c r="E58" s="2" t="inlineStr">
@@ -6294,12 +6303,12 @@
       </c>
       <c r="F58" s="2" t="inlineStr">
         <is>
-          <t>SENT / RECEIVED</t>
+          <t>송금 ID</t>
         </is>
       </c>
       <c r="G58" s="2" t="inlineStr">
         <is>
-          <t>SENT</t>
+          <t>1024</t>
         </is>
       </c>
     </row>
@@ -6316,7 +6325,7 @@
       </c>
       <c r="C59" s="2" t="inlineStr">
         <is>
-          <t>data.items[].counterpartName</t>
+          <t>data.items[].direction</t>
         </is>
       </c>
       <c r="D59" s="2" t="inlineStr">
@@ -6331,12 +6340,12 @@
       </c>
       <c r="F59" s="2" t="inlineStr">
         <is>
-          <t>상대 이름</t>
+          <t>SENT / RECEIVED</t>
         </is>
       </c>
       <c r="G59" s="2" t="inlineStr">
         <is>
-          <t>김영희</t>
+          <t>SENT</t>
         </is>
       </c>
     </row>
@@ -6353,7 +6362,7 @@
       </c>
       <c r="C60" s="2" t="inlineStr">
         <is>
-          <t>data.items[].counterpartAccountNumber</t>
+          <t>data.items[].counterpartName</t>
         </is>
       </c>
       <c r="D60" s="2" t="inlineStr">
@@ -6368,12 +6377,12 @@
       </c>
       <c r="F60" s="2" t="inlineStr">
         <is>
-          <t>상대 계좌</t>
+          <t>상대 이름</t>
         </is>
       </c>
       <c r="G60" s="2" t="inlineStr">
         <is>
-          <t>123456789012</t>
+          <t>김영희</t>
         </is>
       </c>
     </row>
@@ -6390,12 +6399,12 @@
       </c>
       <c r="C61" s="2" t="inlineStr">
         <is>
-          <t>data.items[].amount</t>
+          <t>data.items[].counterpartAccountNumber</t>
         </is>
       </c>
       <c r="D61" s="2" t="inlineStr">
         <is>
-          <t>Long</t>
+          <t>String</t>
         </is>
       </c>
       <c r="E61" s="2" t="inlineStr">
@@ -6405,12 +6414,12 @@
       </c>
       <c r="F61" s="2" t="inlineStr">
         <is>
-          <t>금액(원)</t>
+          <t>상대 계좌</t>
         </is>
       </c>
       <c r="G61" s="2" t="inlineStr">
         <is>
-          <t>10000</t>
+          <t>123456789012</t>
         </is>
       </c>
     </row>
@@ -6427,12 +6436,12 @@
       </c>
       <c r="C62" s="2" t="inlineStr">
         <is>
-          <t>data.items[].createdAt</t>
+          <t>data.items[].amount</t>
         </is>
       </c>
       <c r="D62" s="2" t="inlineStr">
         <is>
-          <t>String</t>
+          <t>Long</t>
         </is>
       </c>
       <c r="E62" s="2" t="inlineStr">
@@ -6442,12 +6451,12 @@
       </c>
       <c r="F62" s="2" t="inlineStr">
         <is>
-          <t>시각(ISO-8601)</t>
+          <t>금액(원)</t>
         </is>
       </c>
       <c r="G62" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T10:01:00+09:00</t>
+          <t>10000</t>
         </is>
       </c>
     </row>
@@ -6464,27 +6473,27 @@
       </c>
       <c r="C63" s="2" t="inlineStr">
         <is>
-          <t>data.nextCursor</t>
+          <t>data.items[].createdAt</t>
         </is>
       </c>
       <c r="D63" s="2" t="inlineStr">
         <is>
-          <t>Long</t>
+          <t>String</t>
         </is>
       </c>
       <c r="E63" s="2" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="F63" s="2" t="inlineStr">
         <is>
-          <t>다음 요청의 cursor(마지막 transferId). 없으면 null</t>
+          <t>시각(ISO-8601)</t>
         </is>
       </c>
       <c r="G63" s="2" t="inlineStr">
         <is>
-          <t>1005</t>
+          <t>2026-09-27T10:01:00+09:00</t>
         </is>
       </c>
     </row>
@@ -6501,27 +6510,27 @@
       </c>
       <c r="C64" s="2" t="inlineStr">
         <is>
-          <t>data.hasNext</t>
+          <t>data.nextCursor</t>
         </is>
       </c>
       <c r="D64" s="2" t="inlineStr">
         <is>
-          <t>Boolean</t>
+          <t>Long</t>
         </is>
       </c>
       <c r="E64" s="2" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="F64" s="2" t="inlineStr">
         <is>
-          <t>다음 묶음 존재 여부</t>
+          <t>다음 요청의 cursor(마지막 transferId). 없으면 null</t>
         </is>
       </c>
       <c r="G64" s="2" t="inlineStr">
         <is>
-          <t>true</t>
+          <t>1005</t>
         </is>
       </c>
     </row>
@@ -6533,59 +6542,59 @@
       </c>
       <c r="B65" s="2" t="inlineStr">
         <is>
-          <t>에러</t>
+          <t>응답</t>
         </is>
       </c>
       <c r="C65" s="2" t="inlineStr">
         <is>
-          <t>AUTH_INVALID</t>
-        </is>
-      </c>
-      <c r="D65" s="2" t="inlineStr"/>
-      <c r="E65" s="2" t="inlineStr"/>
+          <t>data.hasNext</t>
+        </is>
+      </c>
+      <c r="D65" s="2" t="inlineStr">
+        <is>
+          <t>Boolean</t>
+        </is>
+      </c>
+      <c r="E65" s="2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="F65" s="2" t="inlineStr">
         <is>
-          <t>JWT 없음·만료·위조, 로그인 실패</t>
-        </is>
-      </c>
-      <c r="G65" s="2" t="inlineStr"/>
+          <t>다음 묶음 존재 여부</t>
+        </is>
+      </c>
+      <c r="G65" s="2" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>E-10</t>
+          <t>E-09</t>
         </is>
       </c>
       <c r="B66" s="2" t="inlineStr">
         <is>
-          <t>요청</t>
+          <t>에러</t>
         </is>
       </c>
       <c r="C66" s="2" t="inlineStr">
         <is>
-          <t>Header Authorization</t>
-        </is>
-      </c>
-      <c r="D66" s="2" t="inlineStr">
-        <is>
-          <t>String</t>
-        </is>
-      </c>
-      <c r="E66" s="2" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+          <t>AUTH_INVALID</t>
+        </is>
+      </c>
+      <c r="D66" s="2" t="inlineStr"/>
+      <c r="E66" s="2" t="inlineStr"/>
       <c r="F66" s="2" t="inlineStr">
         <is>
-          <t>Bearer {JWT}</t>
-        </is>
-      </c>
-      <c r="G66" s="2" t="inlineStr">
-        <is>
-          <t>Bearer eyJ...</t>
-        </is>
-      </c>
+          <t>JWT 없음·만료·위조, 로그인 실패</t>
+        </is>
+      </c>
+      <c r="G66" s="2" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
@@ -6595,12 +6604,12 @@
       </c>
       <c r="B67" s="2" t="inlineStr">
         <is>
-          <t>응답</t>
+          <t>요청</t>
         </is>
       </c>
       <c r="C67" s="2" t="inlineStr">
         <is>
-          <t>data.threadId</t>
+          <t>Header Authorization</t>
         </is>
       </c>
       <c r="D67" s="2" t="inlineStr">
@@ -6615,12 +6624,12 @@
       </c>
       <c r="F67" s="2" t="inlineStr">
         <is>
-          <t>Spring이 발급, 사용자와 묶어 저장</t>
+          <t>Bearer {JWT}</t>
         </is>
       </c>
       <c r="G67" s="2" t="inlineStr">
         <is>
-          <t>th_5b21...</t>
+          <t>Bearer eyJ...</t>
         </is>
       </c>
     </row>
@@ -6632,59 +6641,59 @@
       </c>
       <c r="B68" s="2" t="inlineStr">
         <is>
-          <t>에러</t>
+          <t>응답</t>
         </is>
       </c>
       <c r="C68" s="2" t="inlineStr">
         <is>
-          <t>AUTH_INVALID</t>
-        </is>
-      </c>
-      <c r="D68" s="2" t="inlineStr"/>
-      <c r="E68" s="2" t="inlineStr"/>
+          <t>data.threadId</t>
+        </is>
+      </c>
+      <c r="D68" s="2" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="E68" s="2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="F68" s="2" t="inlineStr">
         <is>
-          <t>JWT 없음·만료·위조, 로그인 실패</t>
-        </is>
-      </c>
-      <c r="G68" s="2" t="inlineStr"/>
+          <t>Spring이 발급, 사용자와 묶어 저장</t>
+        </is>
+      </c>
+      <c r="G68" s="2" t="inlineStr">
+        <is>
+          <t>th_5b21...</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
         <is>
-          <t>E-11</t>
+          <t>E-10</t>
         </is>
       </c>
       <c r="B69" s="2" t="inlineStr">
         <is>
-          <t>요청</t>
+          <t>에러</t>
         </is>
       </c>
       <c r="C69" s="2" t="inlineStr">
         <is>
-          <t>Header Authorization</t>
-        </is>
-      </c>
-      <c r="D69" s="2" t="inlineStr">
-        <is>
-          <t>String</t>
-        </is>
-      </c>
-      <c r="E69" s="2" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+          <t>AUTH_INVALID</t>
+        </is>
+      </c>
+      <c r="D69" s="2" t="inlineStr"/>
+      <c r="E69" s="2" t="inlineStr"/>
       <c r="F69" s="2" t="inlineStr">
         <is>
-          <t>Bearer {JWT}</t>
-        </is>
-      </c>
-      <c r="G69" s="2" t="inlineStr">
-        <is>
-          <t>Bearer eyJ...</t>
-        </is>
-      </c>
+          <t>JWT 없음·만료·위조, 로그인 실패</t>
+        </is>
+      </c>
+      <c r="G69" s="2" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
@@ -6699,7 +6708,7 @@
       </c>
       <c r="C70" s="2" t="inlineStr">
         <is>
-          <t>Path threadId</t>
+          <t>Header Authorization</t>
         </is>
       </c>
       <c r="D70" s="2" t="inlineStr">
@@ -6714,12 +6723,12 @@
       </c>
       <c r="F70" s="2" t="inlineStr">
         <is>
-          <t>대화 ID</t>
+          <t>Bearer {JWT}</t>
         </is>
       </c>
       <c r="G70" s="2" t="inlineStr">
         <is>
-          <t>th_5b21...</t>
+          <t>Bearer eyJ...</t>
         </is>
       </c>
     </row>
@@ -6736,7 +6745,7 @@
       </c>
       <c r="C71" s="2" t="inlineStr">
         <is>
-          <t>message</t>
+          <t>Path threadId</t>
         </is>
       </c>
       <c r="D71" s="2" t="inlineStr">
@@ -6751,12 +6760,12 @@
       </c>
       <c r="F71" s="2" t="inlineStr">
         <is>
-          <t>사용자 메시지</t>
+          <t>대화 ID</t>
         </is>
       </c>
       <c r="G71" s="2" t="inlineStr">
         <is>
-          <t>엄마한테 1만원 보내줘</t>
+          <t>th_5b21...</t>
         </is>
       </c>
     </row>
@@ -6768,12 +6777,12 @@
       </c>
       <c r="B72" s="2" t="inlineStr">
         <is>
-          <t>응답</t>
+          <t>요청</t>
         </is>
       </c>
       <c r="C72" s="2" t="inlineStr">
         <is>
-          <t>data.reply</t>
+          <t>message</t>
         </is>
       </c>
       <c r="D72" s="2" t="inlineStr">
@@ -6788,12 +6797,12 @@
       </c>
       <c r="F72" s="2" t="inlineStr">
         <is>
-          <t>요약 답변. 가드에 걸리면 고정 문장</t>
+          <t>사용자 메시지</t>
         </is>
       </c>
       <c r="G72" s="2" t="inlineStr">
         <is>
-          <t>삼성전자 2분기 영업이익은 ...</t>
+          <t>엄마한테 1만원 보내줘</t>
         </is>
       </c>
     </row>
@@ -6810,7 +6819,7 @@
       </c>
       <c r="C73" s="2" t="inlineStr">
         <is>
-          <t>data.guard</t>
+          <t>data.reply</t>
         </is>
       </c>
       <c r="D73" s="2" t="inlineStr">
@@ -6825,12 +6834,12 @@
       </c>
       <c r="F73" s="2" t="inlineStr">
         <is>
-          <t>판정 코드: PASS / INJECTION / NUMBER_UNVERIFIED / ADVICE / PROMPT_LEAK</t>
+          <t>요약 답변. 가드에 걸리면 고정 문장</t>
         </is>
       </c>
       <c r="G73" s="2" t="inlineStr">
         <is>
-          <t>PASS</t>
+          <t>삼성전자 2분기 영업이익은 ...</t>
         </is>
       </c>
     </row>
@@ -6847,7 +6856,7 @@
       </c>
       <c r="C74" s="2" t="inlineStr">
         <is>
-          <t>data.transferCard.requestId</t>
+          <t>data.guard</t>
         </is>
       </c>
       <c r="D74" s="2" t="inlineStr">
@@ -6857,17 +6866,17 @@
       </c>
       <c r="E74" s="2" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="F74" s="2" t="inlineStr">
         <is>
-          <t>송금 요청ID(1회용)</t>
+          <t>판정 코드: PASS / INJECTION / NUMBER_UNVERIFIED / ADVICE / PROMPT_LEAK</t>
         </is>
       </c>
       <c r="G74" s="2" t="inlineStr">
         <is>
-          <t>tr_7f3a...</t>
+          <t>PASS</t>
         </is>
       </c>
     </row>
@@ -6884,7 +6893,7 @@
       </c>
       <c r="C75" s="2" t="inlineStr">
         <is>
-          <t>data.transferCard.recipientName</t>
+          <t>data.transferCard.requestId</t>
         </is>
       </c>
       <c r="D75" s="2" t="inlineStr">
@@ -6899,12 +6908,12 @@
       </c>
       <c r="F75" s="2" t="inlineStr">
         <is>
-          <t>수취인 이름</t>
+          <t>송금 요청ID(1회용)</t>
         </is>
       </c>
       <c r="G75" s="2" t="inlineStr">
         <is>
-          <t>김영희</t>
+          <t>tr_7f3a...</t>
         </is>
       </c>
     </row>
@@ -6921,7 +6930,7 @@
       </c>
       <c r="C76" s="2" t="inlineStr">
         <is>
-          <t>data.transferCard.recipientAccountNumber</t>
+          <t>data.transferCard.recipientName</t>
         </is>
       </c>
       <c r="D76" s="2" t="inlineStr">
@@ -6936,12 +6945,12 @@
       </c>
       <c r="F76" s="2" t="inlineStr">
         <is>
-          <t>수취인 계좌</t>
+          <t>수취인 이름</t>
         </is>
       </c>
       <c r="G76" s="2" t="inlineStr">
         <is>
-          <t>123456789012</t>
+          <t>김영희</t>
         </is>
       </c>
     </row>
@@ -6958,7 +6967,7 @@
       </c>
       <c r="C77" s="2" t="inlineStr">
         <is>
-          <t>data.transferCard.fromAccountNumber</t>
+          <t>data.transferCard.recipientAccountNumber</t>
         </is>
       </c>
       <c r="D77" s="2" t="inlineStr">
@@ -6973,12 +6982,12 @@
       </c>
       <c r="F77" s="2" t="inlineStr">
         <is>
-          <t>출금 계좌(대표 계좌)</t>
+          <t>수취인 계좌</t>
         </is>
       </c>
       <c r="G77" s="2" t="inlineStr">
         <is>
-          <t>987654321098</t>
+          <t>123456789012</t>
         </is>
       </c>
     </row>
@@ -6995,12 +7004,12 @@
       </c>
       <c r="C78" s="2" t="inlineStr">
         <is>
-          <t>data.transferCard.amount</t>
+          <t>data.transferCard.fromAccountNumber</t>
         </is>
       </c>
       <c r="D78" s="2" t="inlineStr">
         <is>
-          <t>Long</t>
+          <t>String</t>
         </is>
       </c>
       <c r="E78" s="2" t="inlineStr">
@@ -7010,12 +7019,12 @@
       </c>
       <c r="F78" s="2" t="inlineStr">
         <is>
-          <t>금액(원)</t>
+          <t>출금 계좌(대표 계좌)</t>
         </is>
       </c>
       <c r="G78" s="2" t="inlineStr">
         <is>
-          <t>10000</t>
+          <t>987654321098</t>
         </is>
       </c>
     </row>
@@ -7032,12 +7041,12 @@
       </c>
       <c r="C79" s="2" t="inlineStr">
         <is>
-          <t>data.transferCard.expiresAt</t>
+          <t>data.transferCard.amount</t>
         </is>
       </c>
       <c r="D79" s="2" t="inlineStr">
         <is>
-          <t>String</t>
+          <t>Long</t>
         </is>
       </c>
       <c r="E79" s="2" t="inlineStr">
@@ -7047,12 +7056,12 @@
       </c>
       <c r="F79" s="2" t="inlineStr">
         <is>
-          <t>만료 시각(생성 + 5분, ISO-8601)</t>
+          <t>금액(원)</t>
         </is>
       </c>
       <c r="G79" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T10:05:00+09:00</t>
+          <t>10000</t>
         </is>
       </c>
     </row>
@@ -7069,12 +7078,12 @@
       </c>
       <c r="C80" s="2" t="inlineStr">
         <is>
-          <t>data.table.columns</t>
+          <t>data.transferCard.expiresAt</t>
         </is>
       </c>
       <c r="D80" s="2" t="inlineStr">
         <is>
-          <t>String[]</t>
+          <t>String</t>
         </is>
       </c>
       <c r="E80" s="2" t="inlineStr">
@@ -7084,12 +7093,12 @@
       </c>
       <c r="F80" s="2" t="inlineStr">
         <is>
-          <t>표 머리글</t>
+          <t>만료 시각(생성 + 5분, ISO-8601)</t>
         </is>
       </c>
       <c r="G80" s="2" t="inlineStr">
         <is>
-          <t>["항목","삼성전자","SK하이닉스"]</t>
+          <t>2026-09-27T10:05:00+09:00</t>
         </is>
       </c>
     </row>
@@ -7106,12 +7115,12 @@
       </c>
       <c r="C81" s="2" t="inlineStr">
         <is>
-          <t>data.table.rows</t>
+          <t>data.table.columns</t>
         </is>
       </c>
       <c r="D81" s="2" t="inlineStr">
         <is>
-          <t>String[][]</t>
+          <t>String[]</t>
         </is>
       </c>
       <c r="E81" s="2" t="inlineStr">
@@ -7121,12 +7130,12 @@
       </c>
       <c r="F81" s="2" t="inlineStr">
         <is>
-          <t>표 행</t>
+          <t>표 머리글</t>
         </is>
       </c>
       <c r="G81" s="2" t="inlineStr">
         <is>
-          <t>[["영업이익","...","..."]]</t>
+          <t>["항목","삼성전자","SK하이닉스"]</t>
         </is>
       </c>
     </row>
@@ -7143,12 +7152,12 @@
       </c>
       <c r="C82" s="2" t="inlineStr">
         <is>
-          <t>data.table.note</t>
+          <t>data.table.rows</t>
         </is>
       </c>
       <c r="D82" s="2" t="inlineStr">
         <is>
-          <t>String</t>
+          <t>String[][]</t>
         </is>
       </c>
       <c r="E82" s="2" t="inlineStr">
@@ -7158,12 +7167,12 @@
       </c>
       <c r="F82" s="2" t="inlineStr">
         <is>
-          <t>재무제표 기준(연결/별도)·미공시 표시</t>
+          <t>표 행</t>
         </is>
       </c>
       <c r="G82" s="2" t="inlineStr">
         <is>
-          <t>연결 기준</t>
+          <t>[["영업이익","...","..."]]</t>
         </is>
       </c>
     </row>
@@ -7180,7 +7189,7 @@
       </c>
       <c r="C83" s="2" t="inlineStr">
         <is>
-          <t>data.detailId</t>
+          <t>data.table.note</t>
         </is>
       </c>
       <c r="D83" s="2" t="inlineStr">
@@ -7195,12 +7204,12 @@
       </c>
       <c r="F83" s="2" t="inlineStr">
         <is>
-          <t>상세 보기 ID(분석 답변일 때)</t>
+          <t>재무제표 기준(연결/별도)·미공시 표시</t>
         </is>
       </c>
       <c r="G83" s="2" t="inlineStr">
         <is>
-          <t>dt_91c2...</t>
+          <t>연결 기준</t>
         </is>
       </c>
     </row>
@@ -7212,22 +7221,34 @@
       </c>
       <c r="B84" s="2" t="inlineStr">
         <is>
-          <t>에러</t>
+          <t>응답</t>
         </is>
       </c>
       <c r="C84" s="2" t="inlineStr">
         <is>
-          <t>AUTH_INVALID</t>
-        </is>
-      </c>
-      <c r="D84" s="2" t="inlineStr"/>
-      <c r="E84" s="2" t="inlineStr"/>
+          <t>data.detailId</t>
+        </is>
+      </c>
+      <c r="D84" s="2" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="E84" s="2" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="F84" s="2" t="inlineStr">
         <is>
-          <t>JWT 없음·만료·위조, 로그인 실패</t>
-        </is>
-      </c>
-      <c r="G84" s="2" t="inlineStr"/>
+          <t>상세 보기 ID(분석 답변일 때)</t>
+        </is>
+      </c>
+      <c r="G84" s="2" t="inlineStr">
+        <is>
+          <t>dt_91c2...</t>
+        </is>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
@@ -7242,14 +7263,14 @@
       </c>
       <c r="C85" s="2" t="inlineStr">
         <is>
-          <t>THREAD_NOT_FOUND</t>
+          <t>AUTH_INVALID</t>
         </is>
       </c>
       <c r="D85" s="2" t="inlineStr"/>
       <c r="E85" s="2" t="inlineStr"/>
       <c r="F85" s="2" t="inlineStr">
         <is>
-          <t>대화 없음(또는 남의 대화)</t>
+          <t>JWT 없음·만료·위조, 로그인 실패</t>
         </is>
       </c>
       <c r="G85" s="2" t="inlineStr"/>
@@ -7267,14 +7288,14 @@
       </c>
       <c r="C86" s="2" t="inlineStr">
         <is>
-          <t>RATE_LIMITED</t>
+          <t>THREAD_NOT_FOUND</t>
         </is>
       </c>
       <c r="D86" s="2" t="inlineStr"/>
       <c r="E86" s="2" t="inlineStr"/>
       <c r="F86" s="2" t="inlineStr">
         <is>
-          <t>사용자별 채팅 호출 제한 초과</t>
+          <t>대화 없음(또는 남의 대화)</t>
         </is>
       </c>
       <c r="G86" s="2" t="inlineStr"/>
@@ -7292,14 +7313,14 @@
       </c>
       <c r="C87" s="2" t="inlineStr">
         <is>
-          <t>AI_SERVER_UNAVAILABLE</t>
+          <t>RATE_LIMITED</t>
         </is>
       </c>
       <c r="D87" s="2" t="inlineStr"/>
       <c r="E87" s="2" t="inlineStr"/>
       <c r="F87" s="2" t="inlineStr">
         <is>
-          <t>FastAPI 장애·지연 — 채팅만 실패, 송금·계좌는 정상(장애 격리)</t>
+          <t>사용자별 채팅 호출 제한 초과</t>
         </is>
       </c>
       <c r="G87" s="2" t="inlineStr"/>
@@ -7307,39 +7328,27 @@
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
         <is>
-          <t>E-12</t>
+          <t>E-11</t>
         </is>
       </c>
       <c r="B88" s="2" t="inlineStr">
         <is>
-          <t>요청</t>
+          <t>에러</t>
         </is>
       </c>
       <c r="C88" s="2" t="inlineStr">
         <is>
-          <t>Header Authorization</t>
-        </is>
-      </c>
-      <c r="D88" s="2" t="inlineStr">
-        <is>
-          <t>String</t>
-        </is>
-      </c>
-      <c r="E88" s="2" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+          <t>AI_SERVER_UNAVAILABLE</t>
+        </is>
+      </c>
+      <c r="D88" s="2" t="inlineStr"/>
+      <c r="E88" s="2" t="inlineStr"/>
       <c r="F88" s="2" t="inlineStr">
         <is>
-          <t>Bearer {JWT}</t>
-        </is>
-      </c>
-      <c r="G88" s="2" t="inlineStr">
-        <is>
-          <t>Bearer eyJ...</t>
-        </is>
-      </c>
+          <t>FastAPI 장애·지연 — 채팅만 실패, 송금·계좌는 정상(장애 격리)</t>
+        </is>
+      </c>
+      <c r="G88" s="2" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
@@ -7354,7 +7363,7 @@
       </c>
       <c r="C89" s="2" t="inlineStr">
         <is>
-          <t>Path requestId</t>
+          <t>Header Authorization</t>
         </is>
       </c>
       <c r="D89" s="2" t="inlineStr">
@@ -7369,12 +7378,12 @@
       </c>
       <c r="F89" s="2" t="inlineStr">
         <is>
-          <t>확인 카드의 요청ID</t>
+          <t>Bearer {JWT}</t>
         </is>
       </c>
       <c r="G89" s="2" t="inlineStr">
         <is>
-          <t>tr_7f3a...</t>
+          <t>Bearer eyJ...</t>
         </is>
       </c>
     </row>
@@ -7386,17 +7395,17 @@
       </c>
       <c r="B90" s="2" t="inlineStr">
         <is>
-          <t>응답</t>
+          <t>요청</t>
         </is>
       </c>
       <c r="C90" s="2" t="inlineStr">
         <is>
-          <t>data.transferId</t>
+          <t>Path requestId</t>
         </is>
       </c>
       <c r="D90" s="2" t="inlineStr">
         <is>
-          <t>Long</t>
+          <t>String</t>
         </is>
       </c>
       <c r="E90" s="2" t="inlineStr">
@@ -7406,12 +7415,12 @@
       </c>
       <c r="F90" s="2" t="inlineStr">
         <is>
-          <t>송금 ID</t>
+          <t>확인 카드의 요청ID</t>
         </is>
       </c>
       <c r="G90" s="2" t="inlineStr">
         <is>
-          <t>1026</t>
+          <t>tr_7f3a...</t>
         </is>
       </c>
     </row>
@@ -7428,12 +7437,12 @@
       </c>
       <c r="C91" s="2" t="inlineStr">
         <is>
-          <t>data.recipientName</t>
+          <t>data.transferId</t>
         </is>
       </c>
       <c r="D91" s="2" t="inlineStr">
         <is>
-          <t>String</t>
+          <t>Long</t>
         </is>
       </c>
       <c r="E91" s="2" t="inlineStr">
@@ -7443,12 +7452,12 @@
       </c>
       <c r="F91" s="2" t="inlineStr">
         <is>
-          <t>수취인 이름</t>
+          <t>송금 ID</t>
         </is>
       </c>
       <c r="G91" s="2" t="inlineStr">
         <is>
-          <t>김영희</t>
+          <t>1026</t>
         </is>
       </c>
     </row>
@@ -7465,12 +7474,12 @@
       </c>
       <c r="C92" s="2" t="inlineStr">
         <is>
-          <t>data.amount</t>
+          <t>data.recipientName</t>
         </is>
       </c>
       <c r="D92" s="2" t="inlineStr">
         <is>
-          <t>Long</t>
+          <t>String</t>
         </is>
       </c>
       <c r="E92" s="2" t="inlineStr">
@@ -7480,12 +7489,12 @@
       </c>
       <c r="F92" s="2" t="inlineStr">
         <is>
-          <t>금액(원)</t>
+          <t>수취인 이름</t>
         </is>
       </c>
       <c r="G92" s="2" t="inlineStr">
         <is>
-          <t>10000</t>
+          <t>김영희</t>
         </is>
       </c>
     </row>
@@ -7502,12 +7511,12 @@
       </c>
       <c r="C93" s="2" t="inlineStr">
         <is>
-          <t>data.fromAccountNumber</t>
+          <t>data.amount</t>
         </is>
       </c>
       <c r="D93" s="2" t="inlineStr">
         <is>
-          <t>String</t>
+          <t>Long</t>
         </is>
       </c>
       <c r="E93" s="2" t="inlineStr">
@@ -7517,12 +7526,12 @@
       </c>
       <c r="F93" s="2" t="inlineStr">
         <is>
-          <t>출금 계좌</t>
+          <t>금액(원)</t>
         </is>
       </c>
       <c r="G93" s="2" t="inlineStr">
         <is>
-          <t>987654321098</t>
+          <t>10000</t>
         </is>
       </c>
     </row>
@@ -7539,12 +7548,12 @@
       </c>
       <c r="C94" s="2" t="inlineStr">
         <is>
-          <t>data.balanceAfter</t>
+          <t>data.fromAccountNumber</t>
         </is>
       </c>
       <c r="D94" s="2" t="inlineStr">
         <is>
-          <t>Long</t>
+          <t>String</t>
         </is>
       </c>
       <c r="E94" s="2" t="inlineStr">
@@ -7554,12 +7563,12 @@
       </c>
       <c r="F94" s="2" t="inlineStr">
         <is>
-          <t>송금 후 잔액(원)</t>
+          <t>출금 계좌</t>
         </is>
       </c>
       <c r="G94" s="2" t="inlineStr">
         <is>
-          <t>140000</t>
+          <t>987654321098</t>
         </is>
       </c>
     </row>
@@ -7571,22 +7580,34 @@
       </c>
       <c r="B95" s="2" t="inlineStr">
         <is>
-          <t>에러</t>
+          <t>응답</t>
         </is>
       </c>
       <c r="C95" s="2" t="inlineStr">
         <is>
-          <t>AUTH_INVALID</t>
-        </is>
-      </c>
-      <c r="D95" s="2" t="inlineStr"/>
-      <c r="E95" s="2" t="inlineStr"/>
+          <t>data.balanceAfter</t>
+        </is>
+      </c>
+      <c r="D95" s="2" t="inlineStr">
+        <is>
+          <t>Long</t>
+        </is>
+      </c>
+      <c r="E95" s="2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="F95" s="2" t="inlineStr">
         <is>
-          <t>JWT 없음·만료·위조, 로그인 실패</t>
-        </is>
-      </c>
-      <c r="G95" s="2" t="inlineStr"/>
+          <t>송금 후 잔액(원)</t>
+        </is>
+      </c>
+      <c r="G95" s="2" t="inlineStr">
+        <is>
+          <t>140000</t>
+        </is>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
@@ -7601,14 +7622,14 @@
       </c>
       <c r="C96" s="2" t="inlineStr">
         <is>
-          <t>TRANSFER_REQUEST_NOT_FOUND</t>
+          <t>AUTH_INVALID</t>
         </is>
       </c>
       <c r="D96" s="2" t="inlineStr"/>
       <c r="E96" s="2" t="inlineStr"/>
       <c r="F96" s="2" t="inlineStr">
         <is>
-          <t>송금 요청 없음(또는 남의 요청)</t>
+          <t>JWT 없음·만료·위조, 로그인 실패</t>
         </is>
       </c>
       <c r="G96" s="2" t="inlineStr"/>
@@ -7626,14 +7647,14 @@
       </c>
       <c r="C97" s="2" t="inlineStr">
         <is>
-          <t>TRANSFER_REQUEST_EXPIRED</t>
+          <t>TRANSFER_REQUEST_NOT_FOUND</t>
         </is>
       </c>
       <c r="D97" s="2" t="inlineStr"/>
       <c r="E97" s="2" t="inlineStr"/>
       <c r="F97" s="2" t="inlineStr">
         <is>
-          <t>송금 요청 5분 만료</t>
+          <t>송금 요청 없음(또는 남의 요청)</t>
         </is>
       </c>
       <c r="G97" s="2" t="inlineStr"/>
@@ -7651,14 +7672,14 @@
       </c>
       <c r="C98" s="2" t="inlineStr">
         <is>
-          <t>TRANSFER_REQUEST_ALREADY_USED</t>
+          <t>TRANSFER_REQUEST_EXPIRED</t>
         </is>
       </c>
       <c r="D98" s="2" t="inlineStr"/>
       <c r="E98" s="2" t="inlineStr"/>
       <c r="F98" s="2" t="inlineStr">
         <is>
-          <t>이미 확정된 송금 요청</t>
+          <t>송금 요청 5분 만료</t>
         </is>
       </c>
       <c r="G98" s="2" t="inlineStr"/>
@@ -7676,14 +7697,14 @@
       </c>
       <c r="C99" s="2" t="inlineStr">
         <is>
-          <t>ACCOUNT_NOT_OWNED</t>
+          <t>TRANSFER_REQUEST_ALREADY_USED</t>
         </is>
       </c>
       <c r="D99" s="2" t="inlineStr"/>
       <c r="E99" s="2" t="inlineStr"/>
       <c r="F99" s="2" t="inlineStr">
         <is>
-          <t>내 계좌가 아님</t>
+          <t>이미 확정된 송금 요청</t>
         </is>
       </c>
       <c r="G99" s="2" t="inlineStr"/>
@@ -7701,14 +7722,14 @@
       </c>
       <c r="C100" s="2" t="inlineStr">
         <is>
-          <t>INSUFFICIENT_BALANCE</t>
+          <t>ACCOUNT_NOT_OWNED</t>
         </is>
       </c>
       <c r="D100" s="2" t="inlineStr"/>
       <c r="E100" s="2" t="inlineStr"/>
       <c r="F100" s="2" t="inlineStr">
         <is>
-          <t>잔액 부족</t>
+          <t>내 계좌가 아님</t>
         </is>
       </c>
       <c r="G100" s="2" t="inlineStr"/>
@@ -7716,39 +7737,27 @@
     <row r="101">
       <c r="A101" s="2" t="inlineStr">
         <is>
-          <t>E-13</t>
+          <t>E-12</t>
         </is>
       </c>
       <c r="B101" s="2" t="inlineStr">
         <is>
-          <t>요청</t>
+          <t>에러</t>
         </is>
       </c>
       <c r="C101" s="2" t="inlineStr">
         <is>
-          <t>Header Authorization</t>
-        </is>
-      </c>
-      <c r="D101" s="2" t="inlineStr">
-        <is>
-          <t>String</t>
-        </is>
-      </c>
-      <c r="E101" s="2" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+          <t>INSUFFICIENT_BALANCE</t>
+        </is>
+      </c>
+      <c r="D101" s="2" t="inlineStr"/>
+      <c r="E101" s="2" t="inlineStr"/>
       <c r="F101" s="2" t="inlineStr">
         <is>
-          <t>Bearer {JWT}</t>
-        </is>
-      </c>
-      <c r="G101" s="2" t="inlineStr">
-        <is>
-          <t>Bearer eyJ...</t>
-        </is>
-      </c>
+          <t>잔액 부족</t>
+        </is>
+      </c>
+      <c r="G101" s="2" t="inlineStr"/>
     </row>
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
@@ -7763,7 +7772,7 @@
       </c>
       <c r="C102" s="2" t="inlineStr">
         <is>
-          <t>Path detailId</t>
+          <t>Header Authorization</t>
         </is>
       </c>
       <c r="D102" s="2" t="inlineStr">
@@ -7778,12 +7787,12 @@
       </c>
       <c r="F102" s="2" t="inlineStr">
         <is>
-          <t>답변의 detailId</t>
+          <t>Bearer {JWT}</t>
         </is>
       </c>
       <c r="G102" s="2" t="inlineStr">
         <is>
-          <t>dt_91c2...</t>
+          <t>Bearer eyJ...</t>
         </is>
       </c>
     </row>
@@ -7795,12 +7804,12 @@
       </c>
       <c r="B103" s="2" t="inlineStr">
         <is>
-          <t>응답</t>
+          <t>요청</t>
         </is>
       </c>
       <c r="C103" s="2" t="inlineStr">
         <is>
-          <t>data.detailId</t>
+          <t>Path detailId</t>
         </is>
       </c>
       <c r="D103" s="2" t="inlineStr">
@@ -7815,7 +7824,7 @@
       </c>
       <c r="F103" s="2" t="inlineStr">
         <is>
-          <t>상세 보기 ID</t>
+          <t>답변의 detailId</t>
         </is>
       </c>
       <c r="G103" s="2" t="inlineStr">
@@ -7837,7 +7846,7 @@
       </c>
       <c r="C104" s="2" t="inlineStr">
         <is>
-          <t>data.report</t>
+          <t>data.detailId</t>
         </is>
       </c>
       <c r="D104" s="2" t="inlineStr">
@@ -7852,12 +7861,12 @@
       </c>
       <c r="F104" s="2" t="inlineStr">
         <is>
-          <t>상세 보고서 본문(클릭할 때 생성)</t>
+          <t>상세 보기 ID</t>
         </is>
       </c>
       <c r="G104" s="2" t="inlineStr">
         <is>
-          <t>...</t>
+          <t>dt_91c2...</t>
         </is>
       </c>
     </row>
@@ -7874,27 +7883,27 @@
       </c>
       <c r="C105" s="2" t="inlineStr">
         <is>
-          <t>data.table.columns</t>
+          <t>data.report</t>
         </is>
       </c>
       <c r="D105" s="2" t="inlineStr">
         <is>
-          <t>String[]</t>
+          <t>String</t>
         </is>
       </c>
       <c r="E105" s="2" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="F105" s="2" t="inlineStr">
         <is>
-          <t>표 머리글</t>
+          <t>상세 보고서 본문(클릭할 때 생성)</t>
         </is>
       </c>
       <c r="G105" s="2" t="inlineStr">
         <is>
-          <t>["항목", ...]</t>
+          <t>...</t>
         </is>
       </c>
     </row>
@@ -7911,12 +7920,12 @@
       </c>
       <c r="C106" s="2" t="inlineStr">
         <is>
-          <t>data.table.rows</t>
+          <t>data.table.columns</t>
         </is>
       </c>
       <c r="D106" s="2" t="inlineStr">
         <is>
-          <t>String[][]</t>
+          <t>String[]</t>
         </is>
       </c>
       <c r="E106" s="2" t="inlineStr">
@@ -7926,12 +7935,12 @@
       </c>
       <c r="F106" s="2" t="inlineStr">
         <is>
-          <t>표 행</t>
+          <t>표 머리글</t>
         </is>
       </c>
       <c r="G106" s="2" t="inlineStr">
         <is>
-          <t>[[...]]</t>
+          <t>["항목", ...]</t>
         </is>
       </c>
     </row>
@@ -7948,12 +7957,12 @@
       </c>
       <c r="C107" s="2" t="inlineStr">
         <is>
-          <t>data.table.note</t>
+          <t>data.table.rows</t>
         </is>
       </c>
       <c r="D107" s="2" t="inlineStr">
         <is>
-          <t>String</t>
+          <t>String[][]</t>
         </is>
       </c>
       <c r="E107" s="2" t="inlineStr">
@@ -7963,12 +7972,12 @@
       </c>
       <c r="F107" s="2" t="inlineStr">
         <is>
-          <t>재무제표 기준·미공시 표시</t>
+          <t>표 행</t>
         </is>
       </c>
       <c r="G107" s="2" t="inlineStr">
         <is>
-          <t>연결 기준</t>
+          <t>[[...]]</t>
         </is>
       </c>
     </row>
@@ -7980,22 +7989,34 @@
       </c>
       <c r="B108" s="2" t="inlineStr">
         <is>
-          <t>에러</t>
+          <t>응답</t>
         </is>
       </c>
       <c r="C108" s="2" t="inlineStr">
         <is>
-          <t>AUTH_INVALID</t>
-        </is>
-      </c>
-      <c r="D108" s="2" t="inlineStr"/>
-      <c r="E108" s="2" t="inlineStr"/>
+          <t>data.table.note</t>
+        </is>
+      </c>
+      <c r="D108" s="2" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="E108" s="2" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="F108" s="2" t="inlineStr">
         <is>
-          <t>JWT 없음·만료·위조, 로그인 실패</t>
-        </is>
-      </c>
-      <c r="G108" s="2" t="inlineStr"/>
+          <t>재무제표 기준·미공시 표시</t>
+        </is>
+      </c>
+      <c r="G108" s="2" t="inlineStr">
+        <is>
+          <t>연결 기준</t>
+        </is>
+      </c>
     </row>
     <row r="109">
       <c r="A109" s="2" t="inlineStr">
@@ -8010,14 +8031,14 @@
       </c>
       <c r="C109" s="2" t="inlineStr">
         <is>
-          <t>DETAIL_NOT_FOUND</t>
+          <t>AUTH_INVALID</t>
         </is>
       </c>
       <c r="D109" s="2" t="inlineStr"/>
       <c r="E109" s="2" t="inlineStr"/>
       <c r="F109" s="2" t="inlineStr">
         <is>
-          <t>상세 보기 대상 없음(또는 남의 것)</t>
+          <t>JWT 없음·만료·위조, 로그인 실패</t>
         </is>
       </c>
       <c r="G109" s="2" t="inlineStr"/>
@@ -8035,14 +8056,14 @@
       </c>
       <c r="C110" s="2" t="inlineStr">
         <is>
-          <t>AI_SERVER_UNAVAILABLE</t>
+          <t>DETAIL_NOT_FOUND</t>
         </is>
       </c>
       <c r="D110" s="2" t="inlineStr"/>
       <c r="E110" s="2" t="inlineStr"/>
       <c r="F110" s="2" t="inlineStr">
         <is>
-          <t>FastAPI 장애·지연 — 채팅만 실패, 송금·계좌는 정상(장애 격리)</t>
+          <t>상세 보기 대상 없음(또는 남의 것)</t>
         </is>
       </c>
       <c r="G110" s="2" t="inlineStr"/>
@@ -8050,39 +8071,27 @@
     <row r="111">
       <c r="A111" s="2" t="inlineStr">
         <is>
-          <t>I-01</t>
+          <t>E-13</t>
         </is>
       </c>
       <c r="B111" s="2" t="inlineStr">
         <is>
-          <t>요청</t>
+          <t>에러</t>
         </is>
       </c>
       <c r="C111" s="2" t="inlineStr">
         <is>
-          <t>Header Authorization</t>
-        </is>
-      </c>
-      <c r="D111" s="2" t="inlineStr">
-        <is>
-          <t>String</t>
-        </is>
-      </c>
-      <c r="E111" s="2" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+          <t>AI_SERVER_UNAVAILABLE</t>
+        </is>
+      </c>
+      <c r="D111" s="2" t="inlineStr"/>
+      <c r="E111" s="2" t="inlineStr"/>
       <c r="F111" s="2" t="inlineStr">
         <is>
-          <t>Bearer {JWT}</t>
-        </is>
-      </c>
-      <c r="G111" s="2" t="inlineStr">
-        <is>
-          <t>Bearer eyJ...</t>
-        </is>
-      </c>
+          <t>FastAPI 장애·지연 — 채팅만 실패, 송금·계좌는 정상(장애 격리)</t>
+        </is>
+      </c>
+      <c r="G111" s="2" t="inlineStr"/>
     </row>
     <row r="112">
       <c r="A112" s="2" t="inlineStr">
@@ -8097,7 +8106,7 @@
       </c>
       <c r="C112" s="2" t="inlineStr">
         <is>
-          <t>threadId</t>
+          <t>Header Authorization</t>
         </is>
       </c>
       <c r="D112" s="2" t="inlineStr">
@@ -8112,12 +8121,12 @@
       </c>
       <c r="F112" s="2" t="inlineStr">
         <is>
-          <t>대화 ID(체크포인터 키)</t>
+          <t>Bearer {JWT}</t>
         </is>
       </c>
       <c r="G112" s="2" t="inlineStr">
         <is>
-          <t>th_5b21...</t>
+          <t>Bearer eyJ...</t>
         </is>
       </c>
     </row>
@@ -8134,7 +8143,7 @@
       </c>
       <c r="C113" s="2" t="inlineStr">
         <is>
-          <t>message</t>
+          <t>threadId</t>
         </is>
       </c>
       <c r="D113" s="2" t="inlineStr">
@@ -8149,12 +8158,12 @@
       </c>
       <c r="F113" s="2" t="inlineStr">
         <is>
-          <t>사용자 메시지</t>
+          <t>대화 ID(체크포인터 키)</t>
         </is>
       </c>
       <c r="G113" s="2" t="inlineStr">
         <is>
-          <t>엄마한테 1만원 보내줘</t>
+          <t>th_5b21...</t>
         </is>
       </c>
     </row>
@@ -8166,12 +8175,12 @@
       </c>
       <c r="B114" s="2" t="inlineStr">
         <is>
-          <t>응답</t>
+          <t>요청</t>
         </is>
       </c>
       <c r="C114" s="2" t="inlineStr">
         <is>
-          <t>data.reply</t>
+          <t>message</t>
         </is>
       </c>
       <c r="D114" s="2" t="inlineStr">
@@ -8186,12 +8195,12 @@
       </c>
       <c r="F114" s="2" t="inlineStr">
         <is>
-          <t>요약 답변. 가드에 걸리면 고정 문장</t>
+          <t>사용자 메시지</t>
         </is>
       </c>
       <c r="G114" s="2" t="inlineStr">
         <is>
-          <t>삼성전자 2분기 영업이익은 ...</t>
+          <t>엄마한테 1만원 보내줘</t>
         </is>
       </c>
     </row>
@@ -8208,7 +8217,7 @@
       </c>
       <c r="C115" s="2" t="inlineStr">
         <is>
-          <t>data.guard</t>
+          <t>data.reply</t>
         </is>
       </c>
       <c r="D115" s="2" t="inlineStr">
@@ -8223,12 +8232,12 @@
       </c>
       <c r="F115" s="2" t="inlineStr">
         <is>
-          <t>판정 코드: PASS / INJECTION / NUMBER_UNVERIFIED / ADVICE / PROMPT_LEAK</t>
+          <t>요약 답변. 가드에 걸리면 고정 문장</t>
         </is>
       </c>
       <c r="G115" s="2" t="inlineStr">
         <is>
-          <t>PASS</t>
+          <t>삼성전자 2분기 영업이익은 ...</t>
         </is>
       </c>
     </row>
@@ -8245,7 +8254,7 @@
       </c>
       <c r="C116" s="2" t="inlineStr">
         <is>
-          <t>data.transferCard.requestId</t>
+          <t>data.guard</t>
         </is>
       </c>
       <c r="D116" s="2" t="inlineStr">
@@ -8255,17 +8264,17 @@
       </c>
       <c r="E116" s="2" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="F116" s="2" t="inlineStr">
         <is>
-          <t>송금 요청ID(1회용)</t>
+          <t>판정 코드: PASS / INJECTION / NUMBER_UNVERIFIED / ADVICE / PROMPT_LEAK</t>
         </is>
       </c>
       <c r="G116" s="2" t="inlineStr">
         <is>
-          <t>tr_7f3a...</t>
+          <t>PASS</t>
         </is>
       </c>
     </row>
@@ -8282,7 +8291,7 @@
       </c>
       <c r="C117" s="2" t="inlineStr">
         <is>
-          <t>data.transferCard.recipientName</t>
+          <t>data.transferCard.requestId</t>
         </is>
       </c>
       <c r="D117" s="2" t="inlineStr">
@@ -8297,12 +8306,12 @@
       </c>
       <c r="F117" s="2" t="inlineStr">
         <is>
-          <t>수취인 이름</t>
+          <t>송금 요청ID(1회용)</t>
         </is>
       </c>
       <c r="G117" s="2" t="inlineStr">
         <is>
-          <t>김영희</t>
+          <t>tr_7f3a...</t>
         </is>
       </c>
     </row>
@@ -8319,7 +8328,7 @@
       </c>
       <c r="C118" s="2" t="inlineStr">
         <is>
-          <t>data.transferCard.recipientAccountNumber</t>
+          <t>data.transferCard.recipientName</t>
         </is>
       </c>
       <c r="D118" s="2" t="inlineStr">
@@ -8334,12 +8343,12 @@
       </c>
       <c r="F118" s="2" t="inlineStr">
         <is>
-          <t>수취인 계좌</t>
+          <t>수취인 이름</t>
         </is>
       </c>
       <c r="G118" s="2" t="inlineStr">
         <is>
-          <t>123456789012</t>
+          <t>김영희</t>
         </is>
       </c>
     </row>
@@ -8356,7 +8365,7 @@
       </c>
       <c r="C119" s="2" t="inlineStr">
         <is>
-          <t>data.transferCard.fromAccountNumber</t>
+          <t>data.transferCard.recipientAccountNumber</t>
         </is>
       </c>
       <c r="D119" s="2" t="inlineStr">
@@ -8371,12 +8380,12 @@
       </c>
       <c r="F119" s="2" t="inlineStr">
         <is>
-          <t>출금 계좌(대표 계좌)</t>
+          <t>수취인 계좌</t>
         </is>
       </c>
       <c r="G119" s="2" t="inlineStr">
         <is>
-          <t>987654321098</t>
+          <t>123456789012</t>
         </is>
       </c>
     </row>
@@ -8393,12 +8402,12 @@
       </c>
       <c r="C120" s="2" t="inlineStr">
         <is>
-          <t>data.transferCard.amount</t>
+          <t>data.transferCard.fromAccountNumber</t>
         </is>
       </c>
       <c r="D120" s="2" t="inlineStr">
         <is>
-          <t>Long</t>
+          <t>String</t>
         </is>
       </c>
       <c r="E120" s="2" t="inlineStr">
@@ -8408,12 +8417,12 @@
       </c>
       <c r="F120" s="2" t="inlineStr">
         <is>
-          <t>금액(원)</t>
+          <t>출금 계좌(대표 계좌)</t>
         </is>
       </c>
       <c r="G120" s="2" t="inlineStr">
         <is>
-          <t>10000</t>
+          <t>987654321098</t>
         </is>
       </c>
     </row>
@@ -8430,12 +8439,12 @@
       </c>
       <c r="C121" s="2" t="inlineStr">
         <is>
-          <t>data.transferCard.expiresAt</t>
+          <t>data.transferCard.amount</t>
         </is>
       </c>
       <c r="D121" s="2" t="inlineStr">
         <is>
-          <t>String</t>
+          <t>Long</t>
         </is>
       </c>
       <c r="E121" s="2" t="inlineStr">
@@ -8445,12 +8454,12 @@
       </c>
       <c r="F121" s="2" t="inlineStr">
         <is>
-          <t>만료 시각(생성 + 5분, ISO-8601)</t>
+          <t>금액(원)</t>
         </is>
       </c>
       <c r="G121" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T10:05:00+09:00</t>
+          <t>10000</t>
         </is>
       </c>
     </row>
@@ -8467,12 +8476,12 @@
       </c>
       <c r="C122" s="2" t="inlineStr">
         <is>
-          <t>data.table.columns</t>
+          <t>data.transferCard.expiresAt</t>
         </is>
       </c>
       <c r="D122" s="2" t="inlineStr">
         <is>
-          <t>String[]</t>
+          <t>String</t>
         </is>
       </c>
       <c r="E122" s="2" t="inlineStr">
@@ -8482,12 +8491,12 @@
       </c>
       <c r="F122" s="2" t="inlineStr">
         <is>
-          <t>표 머리글</t>
+          <t>만료 시각(생성 + 5분, ISO-8601)</t>
         </is>
       </c>
       <c r="G122" s="2" t="inlineStr">
         <is>
-          <t>["항목","삼성전자","SK하이닉스"]</t>
+          <t>2026-09-27T10:05:00+09:00</t>
         </is>
       </c>
     </row>
@@ -8504,12 +8513,12 @@
       </c>
       <c r="C123" s="2" t="inlineStr">
         <is>
-          <t>data.table.rows</t>
+          <t>data.table.columns</t>
         </is>
       </c>
       <c r="D123" s="2" t="inlineStr">
         <is>
-          <t>String[][]</t>
+          <t>String[]</t>
         </is>
       </c>
       <c r="E123" s="2" t="inlineStr">
@@ -8519,12 +8528,12 @@
       </c>
       <c r="F123" s="2" t="inlineStr">
         <is>
-          <t>표 행</t>
+          <t>표 머리글</t>
         </is>
       </c>
       <c r="G123" s="2" t="inlineStr">
         <is>
-          <t>[["영업이익","...","..."]]</t>
+          <t>["항목","삼성전자","SK하이닉스"]</t>
         </is>
       </c>
     </row>
@@ -8541,12 +8550,12 @@
       </c>
       <c r="C124" s="2" t="inlineStr">
         <is>
-          <t>data.table.note</t>
+          <t>data.table.rows</t>
         </is>
       </c>
       <c r="D124" s="2" t="inlineStr">
         <is>
-          <t>String</t>
+          <t>String[][]</t>
         </is>
       </c>
       <c r="E124" s="2" t="inlineStr">
@@ -8556,12 +8565,12 @@
       </c>
       <c r="F124" s="2" t="inlineStr">
         <is>
-          <t>재무제표 기준(연결/별도)·미공시 표시</t>
+          <t>표 행</t>
         </is>
       </c>
       <c r="G124" s="2" t="inlineStr">
         <is>
-          <t>연결 기준</t>
+          <t>[["영업이익","...","..."]]</t>
         </is>
       </c>
     </row>
@@ -8578,7 +8587,7 @@
       </c>
       <c r="C125" s="2" t="inlineStr">
         <is>
-          <t>data.detailId</t>
+          <t>data.table.note</t>
         </is>
       </c>
       <c r="D125" s="2" t="inlineStr">
@@ -8593,12 +8602,12 @@
       </c>
       <c r="F125" s="2" t="inlineStr">
         <is>
-          <t>상세 보기 ID(분석 답변일 때)</t>
+          <t>재무제표 기준(연결/별도)·미공시 표시</t>
         </is>
       </c>
       <c r="G125" s="2" t="inlineStr">
         <is>
-          <t>dt_91c2...</t>
+          <t>연결 기준</t>
         </is>
       </c>
     </row>
@@ -8610,59 +8619,59 @@
       </c>
       <c r="B126" s="2" t="inlineStr">
         <is>
-          <t>에러</t>
+          <t>응답</t>
         </is>
       </c>
       <c r="C126" s="2" t="inlineStr">
         <is>
-          <t>AUTH_INVALID</t>
-        </is>
-      </c>
-      <c r="D126" s="2" t="inlineStr"/>
-      <c r="E126" s="2" t="inlineStr"/>
+          <t>data.detailId</t>
+        </is>
+      </c>
+      <c r="D126" s="2" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="E126" s="2" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="F126" s="2" t="inlineStr">
         <is>
-          <t>JWT 없음·만료·위조, 로그인 실패</t>
-        </is>
-      </c>
-      <c r="G126" s="2" t="inlineStr"/>
+          <t>상세 보기 ID(분석 답변일 때)</t>
+        </is>
+      </c>
+      <c r="G126" s="2" t="inlineStr">
+        <is>
+          <t>dt_91c2...</t>
+        </is>
+      </c>
     </row>
     <row r="127">
       <c r="A127" s="2" t="inlineStr">
         <is>
-          <t>I-02</t>
+          <t>I-01</t>
         </is>
       </c>
       <c r="B127" s="2" t="inlineStr">
         <is>
-          <t>요청</t>
+          <t>에러</t>
         </is>
       </c>
       <c r="C127" s="2" t="inlineStr">
         <is>
-          <t>Header Authorization</t>
-        </is>
-      </c>
-      <c r="D127" s="2" t="inlineStr">
-        <is>
-          <t>String</t>
-        </is>
-      </c>
-      <c r="E127" s="2" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+          <t>AUTH_INVALID</t>
+        </is>
+      </c>
+      <c r="D127" s="2" t="inlineStr"/>
+      <c r="E127" s="2" t="inlineStr"/>
       <c r="F127" s="2" t="inlineStr">
         <is>
-          <t>Bearer {JWT}</t>
-        </is>
-      </c>
-      <c r="G127" s="2" t="inlineStr">
-        <is>
-          <t>Bearer eyJ...</t>
-        </is>
-      </c>
+          <t>JWT 없음·만료·위조, 로그인 실패</t>
+        </is>
+      </c>
+      <c r="G127" s="2" t="inlineStr"/>
     </row>
     <row r="128">
       <c r="A128" s="2" t="inlineStr">
@@ -8677,7 +8686,7 @@
       </c>
       <c r="C128" s="2" t="inlineStr">
         <is>
-          <t>Path detailId</t>
+          <t>Header Authorization</t>
         </is>
       </c>
       <c r="D128" s="2" t="inlineStr">
@@ -8692,12 +8701,12 @@
       </c>
       <c r="F128" s="2" t="inlineStr">
         <is>
-          <t>상세 보기 ID</t>
+          <t>Bearer {JWT}</t>
         </is>
       </c>
       <c r="G128" s="2" t="inlineStr">
         <is>
-          <t>dt_91c2...</t>
+          <t>Bearer eyJ...</t>
         </is>
       </c>
     </row>
@@ -8709,12 +8718,12 @@
       </c>
       <c r="B129" s="2" t="inlineStr">
         <is>
-          <t>응답</t>
+          <t>요청</t>
         </is>
       </c>
       <c r="C129" s="2" t="inlineStr">
         <is>
-          <t>data.report</t>
+          <t>Path detailId</t>
         </is>
       </c>
       <c r="D129" s="2" t="inlineStr">
@@ -8729,12 +8738,12 @@
       </c>
       <c r="F129" s="2" t="inlineStr">
         <is>
-          <t>상세 보고서 본문</t>
+          <t>상세 보기 ID</t>
         </is>
       </c>
       <c r="G129" s="2" t="inlineStr">
         <is>
-          <t>...</t>
+          <t>dt_91c2...</t>
         </is>
       </c>
     </row>
@@ -8751,27 +8760,27 @@
       </c>
       <c r="C130" s="2" t="inlineStr">
         <is>
-          <t>data.table.columns</t>
+          <t>data.report</t>
         </is>
       </c>
       <c r="D130" s="2" t="inlineStr">
         <is>
-          <t>String[]</t>
+          <t>String</t>
         </is>
       </c>
       <c r="E130" s="2" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="F130" s="2" t="inlineStr">
         <is>
-          <t>표 머리글</t>
+          <t>상세 보고서 본문</t>
         </is>
       </c>
       <c r="G130" s="2" t="inlineStr">
         <is>
-          <t>["항목", ...]</t>
+          <t>...</t>
         </is>
       </c>
     </row>
@@ -8788,12 +8797,12 @@
       </c>
       <c r="C131" s="2" t="inlineStr">
         <is>
-          <t>data.table.rows</t>
+          <t>data.table.columns</t>
         </is>
       </c>
       <c r="D131" s="2" t="inlineStr">
         <is>
-          <t>String[][]</t>
+          <t>String[]</t>
         </is>
       </c>
       <c r="E131" s="2" t="inlineStr">
@@ -8803,12 +8812,12 @@
       </c>
       <c r="F131" s="2" t="inlineStr">
         <is>
-          <t>표 행</t>
+          <t>표 머리글</t>
         </is>
       </c>
       <c r="G131" s="2" t="inlineStr">
         <is>
-          <t>[[...]]</t>
+          <t>["항목", ...]</t>
         </is>
       </c>
     </row>
@@ -8825,12 +8834,12 @@
       </c>
       <c r="C132" s="2" t="inlineStr">
         <is>
-          <t>data.table.note</t>
+          <t>data.table.rows</t>
         </is>
       </c>
       <c r="D132" s="2" t="inlineStr">
         <is>
-          <t>String</t>
+          <t>String[][]</t>
         </is>
       </c>
       <c r="E132" s="2" t="inlineStr">
@@ -8840,12 +8849,12 @@
       </c>
       <c r="F132" s="2" t="inlineStr">
         <is>
-          <t>재무제표 기준·미공시 표시</t>
+          <t>표 행</t>
         </is>
       </c>
       <c r="G132" s="2" t="inlineStr">
         <is>
-          <t>연결 기준</t>
+          <t>[[...]]</t>
         </is>
       </c>
     </row>
@@ -8857,22 +8866,34 @@
       </c>
       <c r="B133" s="2" t="inlineStr">
         <is>
-          <t>에러</t>
+          <t>응답</t>
         </is>
       </c>
       <c r="C133" s="2" t="inlineStr">
         <is>
-          <t>AUTH_INVALID</t>
-        </is>
-      </c>
-      <c r="D133" s="2" t="inlineStr"/>
-      <c r="E133" s="2" t="inlineStr"/>
+          <t>data.table.note</t>
+        </is>
+      </c>
+      <c r="D133" s="2" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="E133" s="2" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="F133" s="2" t="inlineStr">
         <is>
-          <t>JWT 없음·만료·위조, 로그인 실패</t>
-        </is>
-      </c>
-      <c r="G133" s="2" t="inlineStr"/>
+          <t>재무제표 기준·미공시 표시</t>
+        </is>
+      </c>
+      <c r="G133" s="2" t="inlineStr">
+        <is>
+          <t>연결 기준</t>
+        </is>
+      </c>
     </row>
     <row r="134">
       <c r="A134" s="2" t="inlineStr">
@@ -8887,14 +8908,14 @@
       </c>
       <c r="C134" s="2" t="inlineStr">
         <is>
-          <t>DETAIL_NOT_FOUND</t>
+          <t>AUTH_INVALID</t>
         </is>
       </c>
       <c r="D134" s="2" t="inlineStr"/>
       <c r="E134" s="2" t="inlineStr"/>
       <c r="F134" s="2" t="inlineStr">
         <is>
-          <t>상세 보기 대상 없음(또는 남의 것)</t>
+          <t>JWT 없음·만료·위조, 로그인 실패</t>
         </is>
       </c>
       <c r="G134" s="2" t="inlineStr"/>
@@ -8902,39 +8923,27 @@
     <row r="135">
       <c r="A135" s="2" t="inlineStr">
         <is>
-          <t>I-03</t>
+          <t>I-02</t>
         </is>
       </c>
       <c r="B135" s="2" t="inlineStr">
         <is>
-          <t>요청</t>
+          <t>에러</t>
         </is>
       </c>
       <c r="C135" s="2" t="inlineStr">
         <is>
-          <t>Header Authorization</t>
-        </is>
-      </c>
-      <c r="D135" s="2" t="inlineStr">
-        <is>
-          <t>String</t>
-        </is>
-      </c>
-      <c r="E135" s="2" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+          <t>DETAIL_NOT_FOUND</t>
+        </is>
+      </c>
+      <c r="D135" s="2" t="inlineStr"/>
+      <c r="E135" s="2" t="inlineStr"/>
       <c r="F135" s="2" t="inlineStr">
         <is>
-          <t>Bearer {JWT}</t>
-        </is>
-      </c>
-      <c r="G135" s="2" t="inlineStr">
-        <is>
-          <t>Bearer eyJ...</t>
-        </is>
-      </c>
+          <t>상세 보기 대상 없음(또는 남의 것)</t>
+        </is>
+      </c>
+      <c r="G135" s="2" t="inlineStr"/>
     </row>
     <row r="136">
       <c r="A136" s="2" t="inlineStr">
@@ -8949,7 +8958,7 @@
       </c>
       <c r="C136" s="2" t="inlineStr">
         <is>
-          <t>recipientAccountNumber</t>
+          <t>Header Authorization</t>
         </is>
       </c>
       <c r="D136" s="2" t="inlineStr">
@@ -8959,17 +8968,17 @@
       </c>
       <c r="E136" s="2" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="F136" s="2" t="inlineStr">
         <is>
-          <t>수취인 계좌번호(alias와 둘 중 하나)</t>
+          <t>Bearer {JWT}</t>
         </is>
       </c>
       <c r="G136" s="2" t="inlineStr">
         <is>
-          <t>123456789012</t>
+          <t>Bearer eyJ...</t>
         </is>
       </c>
     </row>
@@ -8986,7 +8995,7 @@
       </c>
       <c r="C137" s="2" t="inlineStr">
         <is>
-          <t>alias</t>
+          <t>recipientAccountNumber</t>
         </is>
       </c>
       <c r="D137" s="2" t="inlineStr">
@@ -9001,12 +9010,12 @@
       </c>
       <c r="F137" s="2" t="inlineStr">
         <is>
-          <t>별칭(recipientAccountNumber와 둘 중 하나)</t>
+          <t>수취인 계좌번호(alias와 둘 중 하나)</t>
         </is>
       </c>
       <c r="G137" s="2" t="inlineStr">
         <is>
-          <t>엄마</t>
+          <t>123456789012</t>
         </is>
       </c>
     </row>
@@ -9023,27 +9032,27 @@
       </c>
       <c r="C138" s="2" t="inlineStr">
         <is>
-          <t>amount</t>
+          <t>alias</t>
         </is>
       </c>
       <c r="D138" s="2" t="inlineStr">
         <is>
-          <t>Long</t>
+          <t>String</t>
         </is>
       </c>
       <c r="E138" s="2" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="F138" s="2" t="inlineStr">
         <is>
-          <t>금액(원)</t>
+          <t>별칭(recipientAccountNumber와 둘 중 하나)</t>
         </is>
       </c>
       <c r="G138" s="2" t="inlineStr">
         <is>
-          <t>10000</t>
+          <t>엄마</t>
         </is>
       </c>
     </row>
@@ -9055,17 +9064,17 @@
       </c>
       <c r="B139" s="2" t="inlineStr">
         <is>
-          <t>응답</t>
+          <t>요청</t>
         </is>
       </c>
       <c r="C139" s="2" t="inlineStr">
         <is>
-          <t>data.requestId</t>
+          <t>amount</t>
         </is>
       </c>
       <c r="D139" s="2" t="inlineStr">
         <is>
-          <t>String</t>
+          <t>Long</t>
         </is>
       </c>
       <c r="E139" s="2" t="inlineStr">
@@ -9075,12 +9084,12 @@
       </c>
       <c r="F139" s="2" t="inlineStr">
         <is>
-          <t>송금 요청ID(1회용)</t>
+          <t>금액(원)</t>
         </is>
       </c>
       <c r="G139" s="2" t="inlineStr">
         <is>
-          <t>tr_7f3a...</t>
+          <t>10000</t>
         </is>
       </c>
     </row>
@@ -9097,7 +9106,7 @@
       </c>
       <c r="C140" s="2" t="inlineStr">
         <is>
-          <t>data.recipientName</t>
+          <t>data.requestId</t>
         </is>
       </c>
       <c r="D140" s="2" t="inlineStr">
@@ -9112,12 +9121,12 @@
       </c>
       <c r="F140" s="2" t="inlineStr">
         <is>
-          <t>수취인 이름</t>
+          <t>송금 요청ID(1회용)</t>
         </is>
       </c>
       <c r="G140" s="2" t="inlineStr">
         <is>
-          <t>김영희</t>
+          <t>tr_7f3a...</t>
         </is>
       </c>
     </row>
@@ -9134,7 +9143,7 @@
       </c>
       <c r="C141" s="2" t="inlineStr">
         <is>
-          <t>data.recipientAccountNumber</t>
+          <t>data.recipientName</t>
         </is>
       </c>
       <c r="D141" s="2" t="inlineStr">
@@ -9149,12 +9158,12 @@
       </c>
       <c r="F141" s="2" t="inlineStr">
         <is>
-          <t>수취인 계좌</t>
+          <t>수취인 이름</t>
         </is>
       </c>
       <c r="G141" s="2" t="inlineStr">
         <is>
-          <t>123456789012</t>
+          <t>김영희</t>
         </is>
       </c>
     </row>
@@ -9171,7 +9180,7 @@
       </c>
       <c r="C142" s="2" t="inlineStr">
         <is>
-          <t>data.fromAccountNumber</t>
+          <t>data.recipientAccountNumber</t>
         </is>
       </c>
       <c r="D142" s="2" t="inlineStr">
@@ -9186,12 +9195,12 @@
       </c>
       <c r="F142" s="2" t="inlineStr">
         <is>
-          <t>출금 계좌(대표 계좌)</t>
+          <t>수취인 계좌</t>
         </is>
       </c>
       <c r="G142" s="2" t="inlineStr">
         <is>
-          <t>987654321098</t>
+          <t>123456789012</t>
         </is>
       </c>
     </row>
@@ -9208,12 +9217,12 @@
       </c>
       <c r="C143" s="2" t="inlineStr">
         <is>
-          <t>data.amount</t>
+          <t>data.fromAccountNumber</t>
         </is>
       </c>
       <c r="D143" s="2" t="inlineStr">
         <is>
-          <t>Long</t>
+          <t>String</t>
         </is>
       </c>
       <c r="E143" s="2" t="inlineStr">
@@ -9223,12 +9232,12 @@
       </c>
       <c r="F143" s="2" t="inlineStr">
         <is>
-          <t>금액(원)</t>
+          <t>출금 계좌(대표 계좌)</t>
         </is>
       </c>
       <c r="G143" s="2" t="inlineStr">
         <is>
-          <t>10000</t>
+          <t>987654321098</t>
         </is>
       </c>
     </row>
@@ -9245,12 +9254,12 @@
       </c>
       <c r="C144" s="2" t="inlineStr">
         <is>
-          <t>data.expiresAt</t>
+          <t>data.amount</t>
         </is>
       </c>
       <c r="D144" s="2" t="inlineStr">
         <is>
-          <t>String</t>
+          <t>Long</t>
         </is>
       </c>
       <c r="E144" s="2" t="inlineStr">
@@ -9260,12 +9269,12 @@
       </c>
       <c r="F144" s="2" t="inlineStr">
         <is>
-          <t>만료 시각(생성 + 5분, ISO-8601)</t>
+          <t>금액(원)</t>
         </is>
       </c>
       <c r="G144" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T10:05:00+09:00</t>
+          <t>10000</t>
         </is>
       </c>
     </row>
@@ -9277,22 +9286,34 @@
       </c>
       <c r="B145" s="2" t="inlineStr">
         <is>
-          <t>에러</t>
+          <t>응답</t>
         </is>
       </c>
       <c r="C145" s="2" t="inlineStr">
         <is>
-          <t>AUTH_INVALID</t>
-        </is>
-      </c>
-      <c r="D145" s="2" t="inlineStr"/>
-      <c r="E145" s="2" t="inlineStr"/>
+          <t>data.expiresAt</t>
+        </is>
+      </c>
+      <c r="D145" s="2" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="E145" s="2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="F145" s="2" t="inlineStr">
         <is>
-          <t>JWT 없음·만료·위조, 로그인 실패</t>
-        </is>
-      </c>
-      <c r="G145" s="2" t="inlineStr"/>
+          <t>만료 시각(생성 + 5분, ISO-8601)</t>
+        </is>
+      </c>
+      <c r="G145" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-27T10:05:00+09:00</t>
+        </is>
+      </c>
     </row>
     <row r="146">
       <c r="A146" s="2" t="inlineStr">
@@ -9307,14 +9328,14 @@
       </c>
       <c r="C146" s="2" t="inlineStr">
         <is>
-          <t>ALIAS_NOT_FOUND</t>
+          <t>AUTH_INVALID</t>
         </is>
       </c>
       <c r="D146" s="2" t="inlineStr"/>
       <c r="E146" s="2" t="inlineStr"/>
       <c r="F146" s="2" t="inlineStr">
         <is>
-          <t>등록되지 않은 별칭</t>
+          <t>JWT 없음·만료·위조, 로그인 실패</t>
         </is>
       </c>
       <c r="G146" s="2" t="inlineStr"/>
@@ -9332,14 +9353,14 @@
       </c>
       <c r="C147" s="2" t="inlineStr">
         <is>
-          <t>ACCOUNT_NOT_FOUND</t>
+          <t>ALIAS_NOT_FOUND</t>
         </is>
       </c>
       <c r="D147" s="2" t="inlineStr"/>
       <c r="E147" s="2" t="inlineStr"/>
       <c r="F147" s="2" t="inlineStr">
         <is>
-          <t>계좌 없음</t>
+          <t>등록되지 않은 별칭</t>
         </is>
       </c>
       <c r="G147" s="2" t="inlineStr"/>
@@ -9347,39 +9368,27 @@
     <row r="148">
       <c r="A148" s="2" t="inlineStr">
         <is>
-          <t>I-04</t>
+          <t>I-03</t>
         </is>
       </c>
       <c r="B148" s="2" t="inlineStr">
         <is>
-          <t>요청</t>
+          <t>에러</t>
         </is>
       </c>
       <c r="C148" s="2" t="inlineStr">
         <is>
-          <t>Header Authorization</t>
-        </is>
-      </c>
-      <c r="D148" s="2" t="inlineStr">
-        <is>
-          <t>String</t>
-        </is>
-      </c>
-      <c r="E148" s="2" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+          <t>ACCOUNT_NOT_FOUND</t>
+        </is>
+      </c>
+      <c r="D148" s="2" t="inlineStr"/>
+      <c r="E148" s="2" t="inlineStr"/>
       <c r="F148" s="2" t="inlineStr">
         <is>
-          <t>Bearer {JWT}</t>
-        </is>
-      </c>
-      <c r="G148" s="2" t="inlineStr">
-        <is>
-          <t>Bearer eyJ...</t>
-        </is>
-      </c>
+          <t>계좌 없음</t>
+        </is>
+      </c>
+      <c r="G148" s="2" t="inlineStr"/>
     </row>
     <row r="149">
       <c r="A149" s="2" t="inlineStr">
@@ -9394,7 +9403,7 @@
       </c>
       <c r="C149" s="2" t="inlineStr">
         <is>
-          <t>Query from</t>
+          <t>Header Authorization</t>
         </is>
       </c>
       <c r="D149" s="2" t="inlineStr">
@@ -9409,12 +9418,12 @@
       </c>
       <c r="F149" s="2" t="inlineStr">
         <is>
-          <t>시작일(yyyy-MM-dd)</t>
+          <t>Bearer {JWT}</t>
         </is>
       </c>
       <c r="G149" s="2" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>Bearer eyJ...</t>
         </is>
       </c>
     </row>
@@ -9431,7 +9440,7 @@
       </c>
       <c r="C150" s="2" t="inlineStr">
         <is>
-          <t>Query to</t>
+          <t>Query from</t>
         </is>
       </c>
       <c r="D150" s="2" t="inlineStr">
@@ -9446,12 +9455,12 @@
       </c>
       <c r="F150" s="2" t="inlineStr">
         <is>
-          <t>종료일(yyyy-MM-dd)</t>
+          <t>시작일(yyyy-MM-dd)</t>
         </is>
       </c>
       <c r="G150" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-09-01</t>
         </is>
       </c>
     </row>
@@ -9468,25 +9477,29 @@
       </c>
       <c r="C151" s="2" t="inlineStr">
         <is>
-          <t>Query cursor</t>
+          <t>Query to</t>
         </is>
       </c>
       <c r="D151" s="2" t="inlineStr">
         <is>
-          <t>Long</t>
+          <t>String</t>
         </is>
       </c>
       <c r="E151" s="2" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="F151" s="2" t="inlineStr">
         <is>
-          <t>E-09와 같은 커서 규칙</t>
-        </is>
-      </c>
-      <c r="G151" s="2" t="inlineStr"/>
+          <t>종료일(yyyy-MM-dd)</t>
+        </is>
+      </c>
+      <c r="G151" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
     </row>
     <row r="152">
       <c r="A152" s="2" t="inlineStr">
@@ -9501,12 +9514,12 @@
       </c>
       <c r="C152" s="2" t="inlineStr">
         <is>
-          <t>Query size</t>
+          <t>Query cursor</t>
         </is>
       </c>
       <c r="D152" s="2" t="inlineStr">
         <is>
-          <t>Integer</t>
+          <t>Long</t>
         </is>
       </c>
       <c r="E152" s="2" t="inlineStr">
@@ -9516,14 +9529,10 @@
       </c>
       <c r="F152" s="2" t="inlineStr">
         <is>
-          <t>기본 20</t>
-        </is>
-      </c>
-      <c r="G152" s="2" t="inlineStr">
-        <is>
-          <t>20</t>
-        </is>
-      </c>
+          <t>E-09와 같은 커서 규칙</t>
+        </is>
+      </c>
+      <c r="G152" s="2" t="inlineStr"/>
     </row>
     <row r="153">
       <c r="A153" s="2" t="inlineStr">
@@ -9533,32 +9542,32 @@
       </c>
       <c r="B153" s="2" t="inlineStr">
         <is>
-          <t>응답</t>
+          <t>요청</t>
         </is>
       </c>
       <c r="C153" s="2" t="inlineStr">
         <is>
-          <t>data.sentTotal</t>
+          <t>Query size</t>
         </is>
       </c>
       <c r="D153" s="2" t="inlineStr">
         <is>
-          <t>Long</t>
+          <t>Integer</t>
         </is>
       </c>
       <c r="E153" s="2" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="F153" s="2" t="inlineStr">
         <is>
-          <t>기간 내 보낸 합계(원, Spring 계산)</t>
+          <t>기본 20</t>
         </is>
       </c>
       <c r="G153" s="2" t="inlineStr">
         <is>
-          <t>230000</t>
+          <t>20</t>
         </is>
       </c>
     </row>
@@ -9575,7 +9584,7 @@
       </c>
       <c r="C154" s="2" t="inlineStr">
         <is>
-          <t>data.receivedTotal</t>
+          <t>data.sentTotal</t>
         </is>
       </c>
       <c r="D154" s="2" t="inlineStr">
@@ -9590,12 +9599,12 @@
       </c>
       <c r="F154" s="2" t="inlineStr">
         <is>
-          <t>기간 내 받은 합계(원, Spring 계산)</t>
+          <t>기간 내 보낸 합계(원, Spring 계산)</t>
         </is>
       </c>
       <c r="G154" s="2" t="inlineStr">
         <is>
-          <t>50000</t>
+          <t>230000</t>
         </is>
       </c>
     </row>
@@ -9612,12 +9621,12 @@
       </c>
       <c r="C155" s="2" t="inlineStr">
         <is>
-          <t>data.count</t>
+          <t>data.receivedTotal</t>
         </is>
       </c>
       <c r="D155" s="2" t="inlineStr">
         <is>
-          <t>Integer</t>
+          <t>Long</t>
         </is>
       </c>
       <c r="E155" s="2" t="inlineStr">
@@ -9627,12 +9636,12 @@
       </c>
       <c r="F155" s="2" t="inlineStr">
         <is>
-          <t>기간 내 건수</t>
+          <t>기간 내 받은 합계(원, Spring 계산)</t>
         </is>
       </c>
       <c r="G155" s="2" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>50000</t>
         </is>
       </c>
     </row>
@@ -9649,12 +9658,12 @@
       </c>
       <c r="C156" s="2" t="inlineStr">
         <is>
-          <t>data.items[].transferId</t>
+          <t>data.count</t>
         </is>
       </c>
       <c r="D156" s="2" t="inlineStr">
         <is>
-          <t>Long</t>
+          <t>Integer</t>
         </is>
       </c>
       <c r="E156" s="2" t="inlineStr">
@@ -9664,12 +9673,12 @@
       </c>
       <c r="F156" s="2" t="inlineStr">
         <is>
-          <t>송금 ID</t>
+          <t>기간 내 건수</t>
         </is>
       </c>
       <c r="G156" s="2" t="inlineStr">
         <is>
-          <t>1024</t>
+          <t>7</t>
         </is>
       </c>
     </row>
@@ -9686,12 +9695,12 @@
       </c>
       <c r="C157" s="2" t="inlineStr">
         <is>
-          <t>data.items[].direction</t>
+          <t>data.items[].transferId</t>
         </is>
       </c>
       <c r="D157" s="2" t="inlineStr">
         <is>
-          <t>String</t>
+          <t>Long</t>
         </is>
       </c>
       <c r="E157" s="2" t="inlineStr">
@@ -9701,12 +9710,12 @@
       </c>
       <c r="F157" s="2" t="inlineStr">
         <is>
-          <t>SENT / RECEIVED</t>
+          <t>송금 ID</t>
         </is>
       </c>
       <c r="G157" s="2" t="inlineStr">
         <is>
-          <t>SENT</t>
+          <t>1024</t>
         </is>
       </c>
     </row>
@@ -9723,7 +9732,7 @@
       </c>
       <c r="C158" s="2" t="inlineStr">
         <is>
-          <t>data.items[].counterpartName</t>
+          <t>data.items[].direction</t>
         </is>
       </c>
       <c r="D158" s="2" t="inlineStr">
@@ -9738,12 +9747,12 @@
       </c>
       <c r="F158" s="2" t="inlineStr">
         <is>
-          <t>상대 이름</t>
+          <t>SENT / RECEIVED</t>
         </is>
       </c>
       <c r="G158" s="2" t="inlineStr">
         <is>
-          <t>김영희</t>
+          <t>SENT</t>
         </is>
       </c>
     </row>
@@ -9760,7 +9769,7 @@
       </c>
       <c r="C159" s="2" t="inlineStr">
         <is>
-          <t>data.items[].counterpartAccountNumber</t>
+          <t>data.items[].counterpartName</t>
         </is>
       </c>
       <c r="D159" s="2" t="inlineStr">
@@ -9775,12 +9784,12 @@
       </c>
       <c r="F159" s="2" t="inlineStr">
         <is>
-          <t>상대 계좌</t>
+          <t>상대 이름</t>
         </is>
       </c>
       <c r="G159" s="2" t="inlineStr">
         <is>
-          <t>123456789012</t>
+          <t>김영희</t>
         </is>
       </c>
     </row>
@@ -9797,12 +9806,12 @@
       </c>
       <c r="C160" s="2" t="inlineStr">
         <is>
-          <t>data.items[].amount</t>
+          <t>data.items[].counterpartAccountNumber</t>
         </is>
       </c>
       <c r="D160" s="2" t="inlineStr">
         <is>
-          <t>Long</t>
+          <t>String</t>
         </is>
       </c>
       <c r="E160" s="2" t="inlineStr">
@@ -9812,12 +9821,12 @@
       </c>
       <c r="F160" s="2" t="inlineStr">
         <is>
-          <t>금액(원)</t>
+          <t>상대 계좌</t>
         </is>
       </c>
       <c r="G160" s="2" t="inlineStr">
         <is>
-          <t>10000</t>
+          <t>123456789012</t>
         </is>
       </c>
     </row>
@@ -9834,12 +9843,12 @@
       </c>
       <c r="C161" s="2" t="inlineStr">
         <is>
-          <t>data.items[].createdAt</t>
+          <t>data.items[].amount</t>
         </is>
       </c>
       <c r="D161" s="2" t="inlineStr">
         <is>
-          <t>String</t>
+          <t>Long</t>
         </is>
       </c>
       <c r="E161" s="2" t="inlineStr">
@@ -9849,12 +9858,12 @@
       </c>
       <c r="F161" s="2" t="inlineStr">
         <is>
-          <t>시각(ISO-8601)</t>
+          <t>금액(원)</t>
         </is>
       </c>
       <c r="G161" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T10:01:00+09:00</t>
+          <t>10000</t>
         </is>
       </c>
     </row>
@@ -9871,27 +9880,27 @@
       </c>
       <c r="C162" s="2" t="inlineStr">
         <is>
-          <t>data.nextCursor</t>
+          <t>data.items[].createdAt</t>
         </is>
       </c>
       <c r="D162" s="2" t="inlineStr">
         <is>
-          <t>Long</t>
+          <t>String</t>
         </is>
       </c>
       <c r="E162" s="2" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="F162" s="2" t="inlineStr">
         <is>
-          <t>다음 요청의 cursor(마지막 transferId). 없으면 null</t>
+          <t>시각(ISO-8601)</t>
         </is>
       </c>
       <c r="G162" s="2" t="inlineStr">
         <is>
-          <t>1005</t>
+          <t>2026-09-27T10:01:00+09:00</t>
         </is>
       </c>
     </row>
@@ -9908,27 +9917,27 @@
       </c>
       <c r="C163" s="2" t="inlineStr">
         <is>
-          <t>data.hasNext</t>
+          <t>data.nextCursor</t>
         </is>
       </c>
       <c r="D163" s="2" t="inlineStr">
         <is>
-          <t>Boolean</t>
+          <t>Long</t>
         </is>
       </c>
       <c r="E163" s="2" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="F163" s="2" t="inlineStr">
         <is>
-          <t>다음 묶음 존재 여부</t>
+          <t>다음 요청의 cursor(마지막 transferId). 없으면 null</t>
         </is>
       </c>
       <c r="G163" s="2" t="inlineStr">
         <is>
-          <t>true</t>
+          <t>1005</t>
         </is>
       </c>
     </row>
@@ -9940,25 +9949,62 @@
       </c>
       <c r="B164" s="2" t="inlineStr">
         <is>
+          <t>응답</t>
+        </is>
+      </c>
+      <c r="C164" s="2" t="inlineStr">
+        <is>
+          <t>data.hasNext</t>
+        </is>
+      </c>
+      <c r="D164" s="2" t="inlineStr">
+        <is>
+          <t>Boolean</t>
+        </is>
+      </c>
+      <c r="E164" s="2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="F164" s="2" t="inlineStr">
+        <is>
+          <t>다음 묶음 존재 여부</t>
+        </is>
+      </c>
+      <c r="G164" s="2" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" s="2" t="inlineStr">
+        <is>
+          <t>I-04</t>
+        </is>
+      </c>
+      <c r="B165" s="2" t="inlineStr">
+        <is>
           <t>에러</t>
         </is>
       </c>
-      <c r="C164" s="2" t="inlineStr">
+      <c r="C165" s="2" t="inlineStr">
         <is>
           <t>AUTH_INVALID</t>
         </is>
       </c>
-      <c r="D164" s="2" t="inlineStr"/>
-      <c r="E164" s="2" t="inlineStr"/>
-      <c r="F164" s="2" t="inlineStr">
+      <c r="D165" s="2" t="inlineStr"/>
+      <c r="E165" s="2" t="inlineStr"/>
+      <c r="F165" s="2" t="inlineStr">
         <is>
           <t>JWT 없음·만료·위조, 로그인 실패</t>
         </is>
       </c>
-      <c r="G164" s="2" t="inlineStr"/>
+      <c r="G165" s="2" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G164"/>
+  <autoFilter ref="A1:G165"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
chore(chat): compose·.env.example에 OpenAI·AI 주소 추가, NFR-024 제한 값 명시 (#23)
</commit_message>
<xml_diff>
--- a/docs/smart-spec.xlsx
+++ b/docs/smart-spec.xlsx
@@ -2383,7 +2383,7 @@
       </c>
       <c r="E52" s="2" t="inlineStr">
         <is>
-          <t>Spring에서 사용자별 제한. MVP는 메모리 카운터, 제한 값 미정. 초과 시 HTTP 429 RATE_LIMITED</t>
+          <t>Spring에서 사용자별 제한. MVP는 메모리 카운터, 사용자당 분당 10회. 초과 시 HTTP 429 RATE_LIMITED</t>
         </is>
       </c>
       <c r="F52" s="2" t="inlineStr">
@@ -3436,11 +3436,7 @@
       <c r="B23" s="2" t="n">
         <v>429</v>
       </c>
-      <c r="C23" s="2" t="inlineStr">
-        <is>
-          <t>사용자별 채팅 호출 제한 초과</t>
-        </is>
-      </c>
+      <c r="C23" s="9" t="n"/>
       <c r="D23" s="9" t="n"/>
       <c r="E23" s="9" t="n"/>
       <c r="F23" s="9" t="n"/>
@@ -3555,7 +3551,6 @@
       <c r="G29" s="9" t="n"/>
       <c r="H29" s="10" t="n"/>
     </row>
-    <row r="30"/>
     <row r="31">
       <c r="A31" s="1" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
docs(spec): 명세 xlsx의 RATE_LIMITED 설명 복구, NFR-024만 수정 (#23)
</commit_message>
<xml_diff>
--- a/docs/smart-spec.xlsx
+++ b/docs/smart-spec.xlsx
@@ -3436,7 +3436,11 @@
       <c r="B23" s="2" t="n">
         <v>429</v>
       </c>
-      <c r="C23" s="9" t="n"/>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>사용자별 채팅 호출 제한 초과</t>
+        </is>
+      </c>
       <c r="D23" s="9" t="n"/>
       <c r="E23" s="9" t="n"/>
       <c r="F23" s="9" t="n"/>
@@ -3551,6 +3555,7 @@
       <c r="G29" s="9" t="n"/>
       <c r="H29" s="10" t="n"/>
     </row>
+    <row r="30"/>
     <row r="31">
       <c r="A31" s="1" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
docs(spec): 로드맵에서 gRPC 제외 — Spring ↔ FastAPI는 WebClient까지
- 개요 2절: 3단계 gRPC 삭제, MCP를 3단계로 당기고 "gRPC는 도입하지 않는다" 명시
- 개요 6절·NFR-033: 로드맵 비교를 RestClient → WebClient 두 단계로
- NFR-041(3단계 gRPC) 삭제, NFR-042를 3단계 MCP로
</commit_message>
<xml_diff>
--- a/docs/smart-spec.xlsx
+++ b/docs/smart-spec.xlsx
@@ -573,7 +573,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G71"/>
+  <dimension ref="A1:G70"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -2684,7 +2684,7 @@
       </c>
       <c r="E61" s="2" t="inlineStr">
         <is>
-          <t>채팅 메시지: REST → 비동기 → gRPC 단계별 처리량·스레드 비교, 가짜 LLM</t>
+          <t>채팅 메시지: REST(RestClient) → 비동기(WebClient) 단계별 처리량·스레드 비교, 가짜 LLM</t>
         </is>
       </c>
       <c r="F61" s="2" t="inlineStr">
@@ -2928,7 +2928,7 @@
     <row r="69">
       <c r="A69" s="3" t="inlineStr">
         <is>
-          <t>NFR-041</t>
+          <t>NFR-042</t>
         </is>
       </c>
       <c r="B69" s="3" t="inlineStr">
@@ -2943,12 +2943,12 @@
       </c>
       <c r="D69" s="3" t="inlineStr">
         <is>
-          <t>3단계 gRPC</t>
+          <t>3단계 MCP</t>
         </is>
       </c>
       <c r="E69" s="3" t="inlineStr">
         <is>
-          <t>Spring ↔ FastAPI 구간만. HTTP/2 동시 접속 대응(트래픽 추정 기준 동시 사용자 약 992명, 버퍼 약 4,960명), REST 대비 부하 테스트 수치</t>
+          <t>송금·계좌 도구(조회·요청 생성까지, 실행 권한 없음), DART 검색 도구</t>
         </is>
       </c>
       <c r="F69" s="3" t="inlineStr">
@@ -2959,77 +2959,44 @@
       <c r="G69" s="3" t="inlineStr"/>
     </row>
     <row r="70">
-      <c r="A70" s="3" t="inlineStr">
-        <is>
-          <t>NFR-042</t>
-        </is>
-      </c>
-      <c r="B70" s="3" t="inlineStr">
+      <c r="A70" s="2" t="inlineStr">
+        <is>
+          <t>NFR-043</t>
+        </is>
+      </c>
+      <c r="B70" s="2" t="inlineStr">
         <is>
           <t>비기능</t>
         </is>
       </c>
-      <c r="C70" s="3" t="inlineStr">
-        <is>
-          <t>로드맵</t>
-        </is>
-      </c>
-      <c r="D70" s="3" t="inlineStr">
-        <is>
-          <t>4단계 MCP</t>
-        </is>
-      </c>
-      <c r="E70" s="3" t="inlineStr">
-        <is>
-          <t>송금·계좌 도구(조회·요청 생성까지, 실행 권한 없음), DART 검색 도구</t>
-        </is>
-      </c>
-      <c r="F70" s="3" t="inlineStr">
-        <is>
-          <t>추후</t>
-        </is>
-      </c>
-      <c r="G70" s="3" t="inlineStr"/>
-    </row>
-    <row r="71">
-      <c r="A71" s="2" t="inlineStr">
-        <is>
-          <t>NFR-043</t>
-        </is>
-      </c>
-      <c r="B71" s="2" t="inlineStr">
-        <is>
-          <t>비기능</t>
-        </is>
-      </c>
-      <c r="C71" s="2" t="inlineStr">
+      <c r="C70" s="2" t="inlineStr">
         <is>
           <t>테스트</t>
         </is>
       </c>
-      <c r="D71" s="2" t="inlineStr">
+      <c r="D70" s="2" t="inlineStr">
         <is>
           <t>계좌 동시성 정합성</t>
         </is>
       </c>
-      <c r="E71" s="2" t="inlineStr">
+      <c r="E70" s="2" t="inlineStr">
         <is>
           <t>동시 계좌 개설(같은/다른 Idempotency-Key), 동시 대표 계좌 변경 후 확인: 대표 계좌 항상 1개, 멱등키 재사용 시 신규 계좌 미생성. 실제 PostgreSQL(Testcontainers)로 검증(목·가짜 DB 사용 안 함)</t>
         </is>
       </c>
-      <c r="F71" s="2" t="inlineStr">
+      <c r="F70" s="2" t="inlineStr">
         <is>
           <t>MVP</t>
         </is>
       </c>
-      <c r="G71" s="2" t="inlineStr">
+      <c r="G70" s="2" t="inlineStr">
         <is>
           <t>E-03, E-05</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G71"/>
+  <autoFilter ref="A1:G70"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
docs(spec): 송금 완료 알림·nginx(도메인 HTTPS)를 MVP로 — 알림 목록·스트림 API(E-14·15), NFR-053
</commit_message>
<xml_diff>
--- a/docs/smart-spec.xlsx
+++ b/docs/smart-spec.xlsx
@@ -13,9 +13,9 @@
     <sheet name="트래픽 추정" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'요구사항'!$A$1:$G$81</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'API 목록'!$A$32:$H$49</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'API 상세'!$A$1:$G$168</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'요구사항'!$A$1:$G$82</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'API 목록'!$A$32:$H$51</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'API 상세'!$A$1:$G$184</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -573,7 +573,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G81"/>
+  <dimension ref="A1:G82"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1454,37 +1454,41 @@
       <c r="G24" s="3" t="inlineStr"/>
     </row>
     <row r="25">
-      <c r="A25" s="3" t="inlineStr">
+      <c r="A25" s="2" t="inlineStr">
         <is>
           <t>FR-024</t>
         </is>
       </c>
-      <c r="B25" s="3" t="inlineStr">
+      <c r="B25" s="2" t="inlineStr">
         <is>
           <t>기능</t>
         </is>
       </c>
-      <c r="C25" s="3" t="inlineStr">
+      <c r="C25" s="2" t="inlineStr">
         <is>
           <t>알림</t>
         </is>
       </c>
-      <c r="D25" s="3" t="inlineStr">
+      <c r="D25" s="2" t="inlineStr">
         <is>
           <t>송금 완료 알림</t>
         </is>
       </c>
-      <c r="E25" s="3" t="inlineStr">
-        <is>
-          <t>송금 확정 후 보낸 사람(출금)·받은 사람(입금) 모두에게 알림. 확정 트랜잭션에 알림 행을 함께 쓰고(outbox) 발송은 비동기라 확정 응답을 늦추지 않음. 접속 중이면 SSE로 바로, 아니면 알림 목록에 남김. (송금 ID, 받는 사람) 유일 키로 한 번만 표시</t>
-        </is>
-      </c>
-      <c r="F25" s="3" t="inlineStr">
-        <is>
-          <t>추후</t>
-        </is>
-      </c>
-      <c r="G25" s="3" t="inlineStr"/>
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t>송금 확정 시 보낸 사람(출금)·받은 사람(입금)에게 알림. 알림 행은 확정 트랜잭션에 함께 저장((송금 ID, 받는 사람) 유일 키 — 커밋되면 반드시 남음), 커밋 뒤 접속 중인 사람에게 SSE로 보냄(확정 응답은 기다리지 않음). 놓친 알림은 목록으로. 화면은 Authorization 헤더를 붙이려고 EventSource 대신 fetch 스트림으로 받음(토큰을 URL에 넣지 않음). 서버 1대 기준이고 대량 전달은 NFR-045</t>
+        </is>
+      </c>
+      <c r="F25" s="2" t="inlineStr">
+        <is>
+          <t>MVP</t>
+        </is>
+      </c>
+      <c r="G25" s="2" t="inlineStr">
+        <is>
+          <t>E-12, E-14, E-15</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="3" t="inlineStr">
@@ -3253,7 +3257,7 @@
       </c>
       <c r="E78" s="3" t="inlineStr">
         <is>
-          <t>1대 한계(15 TPS, 피크 30분 약 4,800명)를 넘으면 순서대로: ① 입장 제어(사용자·API 키별 한도, 동시 처리 상한, 넘치면 429 + Retry-After, 송금 확정 우선, 쓰기 도구 멱등 키) ② 무상태화(대화 상태 PostgreSQL, 호출 제한·캐시 Redis) ③ nginx 뒤 FastAPI·Spring 여러 대(FastAPI부터), DB 커넥션 풀러 ④ LLM 토큰 예산. 1 → 2 → 4대에서 같은 stress.sh로 한계 TPS 비교</t>
+          <t>1대 한계(15 TPS, 피크 30분 약 4,800명)를 넘으면 순서대로: ① 입장 제어(사용자·API 키별 한도, 동시 처리 상한, 넘치면 429 + Retry-After, 송금 확정 우선, 쓰기 도구 멱등 키) ② 무상태화(대화 상태 PostgreSQL, 호출 제한·캐시 Redis, 알림 SSE는 연결이 다른 서버에 있어도 닿게 Redis pub/sub) ③ nginx(NFR-053) 뒤 FastAPI·Spring 여러 대(FastAPI부터), DB 커넥션 풀러 ④ LLM 토큰 예산. 1 → 2 → 4대에서 같은 stress.sh로 한계 TPS 비교</t>
         </is>
       </c>
       <c r="F78" s="3" t="inlineStr">
@@ -3286,7 +3290,7 @@
       </c>
       <c r="E79" s="3" t="inlineStr">
         <is>
-          <t>Docker 네트워크를 앞단(터널 커넥터 ↔ Spring)·내부(Spring·FastAPI·DB)·외부 호출(터널 커넥터·FastAPI·collector만 인터넷으로)로 분리 — Spring·DB는 인터넷으로 못 나감. 들어오는 포트 0(터널로 웹 공개), 관리(SSH·Grafana·DB)와 배포는 VPN(사람·기기 단위 허용)으로만. 호스트 방화벽 기본 차단, Docker 포트는 127.0.0.1에만. 앱별 DB 계정(최소 권한)</t>
+          <t>Docker 네트워크를 앞단(터널 커넥터 ↔ nginx ↔ Spring)·내부(Spring·FastAPI·DB)·외부 호출(터널 커넥터·FastAPI·collector만 인터넷으로)로 분리 — Spring·DB는 인터넷으로 못 나감. 들어오는 포트 0(터널로 웹 공개 — NFR-053의 80·443 포트포워딩을 대체), 관리(SSH·Grafana·DB)와 배포는 VPN(사람·기기 단위 허용)으로만. 호스트 방화벽 기본 차단, Docker 포트는 127.0.0.1에만. 앱별 DB 계정(최소 권한)</t>
         </is>
       </c>
       <c r="F79" s="3" t="inlineStr">
@@ -3366,8 +3370,45 @@
         </is>
       </c>
     </row>
+    <row r="82">
+      <c r="A82" s="2" t="inlineStr">
+        <is>
+          <t>NFR-053</t>
+        </is>
+      </c>
+      <c r="B82" s="2" t="inlineStr">
+        <is>
+          <t>비기능</t>
+        </is>
+      </c>
+      <c r="C82" s="2" t="inlineStr">
+        <is>
+          <t>운영</t>
+        </is>
+      </c>
+      <c r="D82" s="2" t="inlineStr">
+        <is>
+          <t>리버스 프록시·HTTPS(nginx)</t>
+        </is>
+      </c>
+      <c r="E82" s="2" t="inlineStr">
+        <is>
+          <t>도메인을 붙이고 nginx를 유일한 입구로: TLS 종료(Let's Encrypt, 자동 갱신), 80은 443으로 넘김, Spring으로 프록시(X-Forwarded-For·Proto 전달). 공유기는 80·443만 nginx로 넘기고 Spring 8080은 공개 중단(127.0.0.1에만). 타임아웃은 nginx &gt; Spring 읽기 제한(채팅 10초·상세 30초), 알림 스트림(E-15)은 버퍼링 끄고 하트비트 간격보다 길게. 로그인·가입은 IP별 요청 제한(limit_req). 부하 측정 환경은 지금처럼 Spring 직접(기준선 유지)</t>
+        </is>
+      </c>
+      <c r="F82" s="2" t="inlineStr">
+        <is>
+          <t>MVP</t>
+        </is>
+      </c>
+      <c r="G82" s="2" t="inlineStr">
+        <is>
+          <t>E-01, E-02, E-15</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:G81"/>
+  <autoFilter ref="A1:G82"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -3378,7 +3419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H49"/>
+  <dimension ref="A1:H51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -4419,12 +4460,12 @@
       </c>
       <c r="G44" s="2" t="inlineStr">
         <is>
-          <t>FR-010, NFR-001, NFR-009, NFR-010</t>
+          <t>FR-010, FR-024, NFR-001, NFR-009, NFR-010</t>
         </is>
       </c>
       <c r="H44" s="2" t="inlineStr">
         <is>
-          <t>AI 경로를 거치지 않음. 계좌 비밀번호도 여기서만 받음</t>
+          <t>AI 경로를 거치지 않음. 계좌 비밀번호도 여기서만 받음. 확정 트랜잭션에 알림 행 저장(FR-024)</t>
         </is>
       </c>
     </row>
@@ -4473,54 +4514,54 @@
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>I-01</t>
+          <t>E-14</t>
         </is>
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>내부 Spring→FastAPI</t>
+          <t>외부</t>
         </is>
       </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t>POST</t>
+          <t>GET</t>
         </is>
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>/internal/chat</t>
+          <t>/api/v1/notifications?cursor&amp;size</t>
         </is>
       </c>
       <c r="E46" s="2" t="inlineStr">
         <is>
-          <t>채팅 처리(LangGraph 구동)</t>
+          <t>알림 목록</t>
         </is>
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
-          <t>Bearer(사용자 JWT 전달)</t>
+          <t>Bearer</t>
         </is>
       </c>
       <c r="G46" s="2" t="inlineStr">
         <is>
-          <t>FR-014, FR-015, NFR-005, NFR-006</t>
+          <t>FR-024</t>
         </is>
       </c>
       <c r="H46" s="2" t="inlineStr">
         <is>
-          <t>FastAPI 쪽 API</t>
+          <t>최신순 커서(E-09와 같은 규칙). 스트림이 끊긴 사이 놓친 알림을 채움</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>I-02</t>
+          <t>E-15</t>
         </is>
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
-          <t>내부 Spring→FastAPI</t>
+          <t>외부</t>
         </is>
       </c>
       <c r="C47" s="2" t="inlineStr">
@@ -4530,39 +4571,39 @@
       </c>
       <c r="D47" s="2" t="inlineStr">
         <is>
-          <t>/internal/details/{detailId}</t>
+          <t>/api/v1/notifications/stream</t>
         </is>
       </c>
       <c r="E47" s="2" t="inlineStr">
         <is>
-          <t>상세 보고서 생성</t>
+          <t>알림 스트림(SSE)</t>
         </is>
       </c>
       <c r="F47" s="2" t="inlineStr">
         <is>
-          <t>Bearer(사용자 JWT 전달)</t>
+          <t>Bearer</t>
         </is>
       </c>
       <c r="G47" s="2" t="inlineStr">
         <is>
-          <t>FR-016, NFR-005, NFR-006</t>
+          <t>FR-024, NFR-053</t>
         </is>
       </c>
       <c r="H47" s="2" t="inlineStr">
         <is>
-          <t>FastAPI 쪽 API</t>
+          <t>text/event-stream이라 응답 형식 공통 규칙의 예외. 화면은 fetch 스트림으로 받음(EventSource는 헤더를 못 붙임). 서버는 하트비트로 연결 유지</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>I-03</t>
+          <t>I-01</t>
         </is>
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>내부 FastAPI→Spring</t>
+          <t>내부 Spring→FastAPI</t>
         </is>
       </c>
       <c r="C48" s="2" t="inlineStr">
@@ -4572,12 +4613,12 @@
       </c>
       <c r="D48" s="2" t="inlineStr">
         <is>
-          <t>/internal/transfer-requests</t>
+          <t>/internal/chat</t>
         </is>
       </c>
       <c r="E48" s="2" t="inlineStr">
         <is>
-          <t>송금 요청 생성(확인 카드용)</t>
+          <t>채팅 처리(LangGraph 구동)</t>
         </is>
       </c>
       <c r="F48" s="2" t="inlineStr">
@@ -4587,59 +4628,143 @@
       </c>
       <c r="G48" s="2" t="inlineStr">
         <is>
-          <t>FR-009, NFR-001, NFR-005, NFR-006</t>
+          <t>FR-014, FR-015, NFR-005, NFR-006</t>
         </is>
       </c>
       <c r="H48" s="2" t="inlineStr">
         <is>
-          <t>LangGraph 도구. 실행은 하지 않음</t>
+          <t>FastAPI 쪽 API</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
         <is>
+          <t>I-02</t>
+        </is>
+      </c>
+      <c r="B49" s="2" t="inlineStr">
+        <is>
+          <t>내부 Spring→FastAPI</t>
+        </is>
+      </c>
+      <c r="C49" s="2" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="D49" s="2" t="inlineStr">
+        <is>
+          <t>/internal/details/{detailId}</t>
+        </is>
+      </c>
+      <c r="E49" s="2" t="inlineStr">
+        <is>
+          <t>상세 보고서 생성</t>
+        </is>
+      </c>
+      <c r="F49" s="2" t="inlineStr">
+        <is>
+          <t>Bearer(사용자 JWT 전달)</t>
+        </is>
+      </c>
+      <c r="G49" s="2" t="inlineStr">
+        <is>
+          <t>FR-016, NFR-005, NFR-006</t>
+        </is>
+      </c>
+      <c r="H49" s="2" t="inlineStr">
+        <is>
+          <t>FastAPI 쪽 API</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="inlineStr">
+        <is>
+          <t>I-03</t>
+        </is>
+      </c>
+      <c r="B50" s="2" t="inlineStr">
+        <is>
+          <t>내부 FastAPI→Spring</t>
+        </is>
+      </c>
+      <c r="C50" s="2" t="inlineStr">
+        <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="D50" s="2" t="inlineStr">
+        <is>
+          <t>/internal/transfer-requests</t>
+        </is>
+      </c>
+      <c r="E50" s="2" t="inlineStr">
+        <is>
+          <t>송금 요청 생성(확인 카드용)</t>
+        </is>
+      </c>
+      <c r="F50" s="2" t="inlineStr">
+        <is>
+          <t>Bearer(사용자 JWT 전달)</t>
+        </is>
+      </c>
+      <c r="G50" s="2" t="inlineStr">
+        <is>
+          <t>FR-009, NFR-001, NFR-005, NFR-006</t>
+        </is>
+      </c>
+      <c r="H50" s="2" t="inlineStr">
+        <is>
+          <t>LangGraph 도구. 실행은 하지 않음</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="2" t="inlineStr">
+        <is>
           <t>I-04</t>
         </is>
       </c>
-      <c r="B49" s="2" t="inlineStr">
+      <c r="B51" s="2" t="inlineStr">
         <is>
           <t>내부 FastAPI→Spring</t>
         </is>
       </c>
-      <c r="C49" s="2" t="inlineStr">
+      <c r="C51" s="2" t="inlineStr">
         <is>
           <t>GET</t>
         </is>
       </c>
-      <c r="D49" s="2" t="inlineStr">
+      <c r="D51" s="2" t="inlineStr">
         <is>
           <t>/internal/transfers?from&amp;to&amp;cursor&amp;size</t>
         </is>
       </c>
-      <c r="E49" s="2" t="inlineStr">
+      <c r="E51" s="2" t="inlineStr">
         <is>
           <t>송금 내역·합계 조회</t>
         </is>
       </c>
-      <c r="F49" s="2" t="inlineStr">
+      <c r="F51" s="2" t="inlineStr">
         <is>
           <t>Bearer(사용자 JWT 전달)</t>
         </is>
       </c>
-      <c r="G49" s="2" t="inlineStr">
+      <c r="G51" s="2" t="inlineStr">
         <is>
           <t>FR-012, NFR-002, NFR-005, NFR-006</t>
         </is>
       </c>
-      <c r="H49" s="2" t="inlineStr">
+      <c r="H51" s="2" t="inlineStr">
         <is>
           <t>LangGraph 도구. 합계는 Spring 계산</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A32:H49"/>
+  <autoFilter ref="A32:H51"/>
   <mergeCells count="30">
     <mergeCell ref="C10:H10"/>
     <mergeCell ref="C16:H16"/>
@@ -4682,7 +4807,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G168"/>
+  <dimension ref="A1:G184"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -8555,7 +8680,7 @@
     <row r="115">
       <c r="A115" s="2" t="inlineStr">
         <is>
-          <t>I-01</t>
+          <t>E-14</t>
         </is>
       </c>
       <c r="B115" s="2" t="inlineStr">
@@ -8592,7 +8717,7 @@
     <row r="116">
       <c r="A116" s="2" t="inlineStr">
         <is>
-          <t>I-01</t>
+          <t>E-14</t>
         </is>
       </c>
       <c r="B116" s="2" t="inlineStr">
@@ -8602,34 +8727,34 @@
       </c>
       <c r="C116" s="2" t="inlineStr">
         <is>
-          <t>threadId</t>
+          <t>Query cursor</t>
         </is>
       </c>
       <c r="D116" s="2" t="inlineStr">
         <is>
-          <t>String</t>
+          <t>Long</t>
         </is>
       </c>
       <c r="E116" s="2" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="F116" s="2" t="inlineStr">
         <is>
-          <t>대화 ID(체크포인터 키)</t>
+          <t>이전 응답의 nextCursor. 없으면 최신부터</t>
         </is>
       </c>
       <c r="G116" s="2" t="inlineStr">
         <is>
-          <t>th_5b21...</t>
+          <t>502</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" s="2" t="inlineStr">
         <is>
-          <t>I-01</t>
+          <t>E-14</t>
         </is>
       </c>
       <c r="B117" s="2" t="inlineStr">
@@ -8639,34 +8764,34 @@
       </c>
       <c r="C117" s="2" t="inlineStr">
         <is>
-          <t>message</t>
+          <t>Query size</t>
         </is>
       </c>
       <c r="D117" s="2" t="inlineStr">
         <is>
-          <t>String</t>
+          <t>Integer</t>
         </is>
       </c>
       <c r="E117" s="2" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="F117" s="2" t="inlineStr">
         <is>
-          <t>사용자 메시지</t>
+          <t>묶음 크기(기본 20)</t>
         </is>
       </c>
       <c r="G117" s="2" t="inlineStr">
         <is>
-          <t>엄마한테 1만원 보내줘</t>
+          <t>20</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" s="2" t="inlineStr">
         <is>
-          <t>I-01</t>
+          <t>E-14</t>
         </is>
       </c>
       <c r="B118" s="2" t="inlineStr">
@@ -8676,12 +8801,12 @@
       </c>
       <c r="C118" s="2" t="inlineStr">
         <is>
-          <t>data.reply</t>
+          <t>data.items[].notificationId</t>
         </is>
       </c>
       <c r="D118" s="2" t="inlineStr">
         <is>
-          <t>String</t>
+          <t>Long</t>
         </is>
       </c>
       <c r="E118" s="2" t="inlineStr">
@@ -8691,19 +8816,19 @@
       </c>
       <c r="F118" s="2" t="inlineStr">
         <is>
-          <t>요약 답변. 가드에 걸리면 고정 문장</t>
+          <t>알림 ID. 화면은 마지막으로 본 ID를 기억해 새 알림을 표시(서버에 읽음 상태 없음)</t>
         </is>
       </c>
       <c r="G118" s="2" t="inlineStr">
         <is>
-          <t>삼성전자 2분기 영업이익은 ...</t>
+          <t>503</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" s="2" t="inlineStr">
         <is>
-          <t>I-01</t>
+          <t>E-14</t>
         </is>
       </c>
       <c r="B119" s="2" t="inlineStr">
@@ -8713,7 +8838,7 @@
       </c>
       <c r="C119" s="2" t="inlineStr">
         <is>
-          <t>data.guard</t>
+          <t>data.items[].direction</t>
         </is>
       </c>
       <c r="D119" s="2" t="inlineStr">
@@ -8728,19 +8853,19 @@
       </c>
       <c r="F119" s="2" t="inlineStr">
         <is>
-          <t>판정 코드: PASS / INJECTION / NUMBER_UNVERIFIED / ADVICE / PROMPT_LEAK</t>
+          <t>SENT(출금) / RECEIVED(입금)</t>
         </is>
       </c>
       <c r="G119" s="2" t="inlineStr">
         <is>
-          <t>PASS</t>
+          <t>RECEIVED</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" s="2" t="inlineStr">
         <is>
-          <t>I-01</t>
+          <t>E-14</t>
         </is>
       </c>
       <c r="B120" s="2" t="inlineStr">
@@ -8750,34 +8875,34 @@
       </c>
       <c r="C120" s="2" t="inlineStr">
         <is>
-          <t>data.transferCard.requestId</t>
+          <t>data.items[].transferId</t>
         </is>
       </c>
       <c r="D120" s="2" t="inlineStr">
         <is>
-          <t>String</t>
+          <t>Long</t>
         </is>
       </c>
       <c r="E120" s="2" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="F120" s="2" t="inlineStr">
         <is>
-          <t>송금 요청ID(1회용)</t>
+          <t>송금 ID</t>
         </is>
       </c>
       <c r="G120" s="2" t="inlineStr">
         <is>
-          <t>tr_7f3a...</t>
+          <t>1026</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" s="2" t="inlineStr">
         <is>
-          <t>I-01</t>
+          <t>E-14</t>
         </is>
       </c>
       <c r="B121" s="2" t="inlineStr">
@@ -8787,7 +8912,7 @@
       </c>
       <c r="C121" s="2" t="inlineStr">
         <is>
-          <t>data.transferCard.recipientName</t>
+          <t>data.items[].counterpartName</t>
         </is>
       </c>
       <c r="D121" s="2" t="inlineStr">
@@ -8797,24 +8922,24 @@
       </c>
       <c r="E121" s="2" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="F121" s="2" t="inlineStr">
         <is>
-          <t>수취인 이름</t>
+          <t>상대 이름</t>
         </is>
       </c>
       <c r="G121" s="2" t="inlineStr">
         <is>
-          <t>김영희</t>
+          <t>홍길동</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" s="2" t="inlineStr">
         <is>
-          <t>I-01</t>
+          <t>E-14</t>
         </is>
       </c>
       <c r="B122" s="2" t="inlineStr">
@@ -8824,34 +8949,34 @@
       </c>
       <c r="C122" s="2" t="inlineStr">
         <is>
-          <t>data.transferCard.recipientAccountNumber</t>
+          <t>data.items[].amount</t>
         </is>
       </c>
       <c r="D122" s="2" t="inlineStr">
         <is>
-          <t>String</t>
+          <t>Long</t>
         </is>
       </c>
       <c r="E122" s="2" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="F122" s="2" t="inlineStr">
         <is>
-          <t>수취인 계좌</t>
+          <t>금액(원)</t>
         </is>
       </c>
       <c r="G122" s="2" t="inlineStr">
         <is>
-          <t>123456789012</t>
+          <t>10000</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" s="2" t="inlineStr">
         <is>
-          <t>I-01</t>
+          <t>E-14</t>
         </is>
       </c>
       <c r="B123" s="2" t="inlineStr">
@@ -8861,7 +8986,7 @@
       </c>
       <c r="C123" s="2" t="inlineStr">
         <is>
-          <t>data.transferCard.fromAccountNumber</t>
+          <t>data.items[].createdAt</t>
         </is>
       </c>
       <c r="D123" s="2" t="inlineStr">
@@ -8871,24 +8996,24 @@
       </c>
       <c r="E123" s="2" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="F123" s="2" t="inlineStr">
         <is>
-          <t>출금 계좌(대표 계좌)</t>
+          <t>확정 시각(ISO-8601)</t>
         </is>
       </c>
       <c r="G123" s="2" t="inlineStr">
         <is>
-          <t>987654321098</t>
+          <t>2026-10-22T10:01:00+09:00</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" s="2" t="inlineStr">
         <is>
-          <t>I-01</t>
+          <t>E-14</t>
         </is>
       </c>
       <c r="B124" s="2" t="inlineStr">
@@ -8898,7 +9023,7 @@
       </c>
       <c r="C124" s="2" t="inlineStr">
         <is>
-          <t>data.transferCard.amount</t>
+          <t>data.nextCursor</t>
         </is>
       </c>
       <c r="D124" s="2" t="inlineStr">
@@ -8913,19 +9038,19 @@
       </c>
       <c r="F124" s="2" t="inlineStr">
         <is>
-          <t>금액(원)</t>
+          <t>다음 요청의 cursor(마지막 notificationId). 없으면 null</t>
         </is>
       </c>
       <c r="G124" s="2" t="inlineStr">
         <is>
-          <t>10000</t>
+          <t>484</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" s="2" t="inlineStr">
         <is>
-          <t>I-01</t>
+          <t>E-14</t>
         </is>
       </c>
       <c r="B125" s="2" t="inlineStr">
@@ -8935,108 +9060,96 @@
       </c>
       <c r="C125" s="2" t="inlineStr">
         <is>
-          <t>data.transferCard.expiresAt</t>
+          <t>data.hasNext</t>
         </is>
       </c>
       <c r="D125" s="2" t="inlineStr">
         <is>
-          <t>String</t>
+          <t>Boolean</t>
         </is>
       </c>
       <c r="E125" s="2" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="F125" s="2" t="inlineStr">
         <is>
-          <t>만료 시각(생성 + 5분, ISO-8601)</t>
+          <t>다음 묶음 존재 여부</t>
         </is>
       </c>
       <c r="G125" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T10:05:00+09:00</t>
+          <t>true</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="A126" s="2" t="inlineStr">
         <is>
-          <t>I-01</t>
+          <t>E-14</t>
         </is>
       </c>
       <c r="B126" s="2" t="inlineStr">
         <is>
-          <t>응답</t>
+          <t>에러</t>
         </is>
       </c>
       <c r="C126" s="2" t="inlineStr">
         <is>
-          <t>data.table.columns</t>
-        </is>
-      </c>
-      <c r="D126" s="2" t="inlineStr">
-        <is>
-          <t>String[]</t>
-        </is>
-      </c>
-      <c r="E126" s="2" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
+          <t>AUTH_INVALID</t>
+        </is>
+      </c>
+      <c r="D126" s="2" t="inlineStr"/>
+      <c r="E126" s="2" t="inlineStr"/>
       <c r="F126" s="2" t="inlineStr">
         <is>
-          <t>표 머리글</t>
-        </is>
-      </c>
-      <c r="G126" s="2" t="inlineStr">
-        <is>
-          <t>["항목","삼성전자","SK하이닉스"]</t>
-        </is>
-      </c>
+          <t>JWT 없음·만료·위조, 로그인 실패</t>
+        </is>
+      </c>
+      <c r="G126" s="2" t="inlineStr"/>
     </row>
     <row r="127">
       <c r="A127" s="2" t="inlineStr">
         <is>
-          <t>I-01</t>
+          <t>E-15</t>
         </is>
       </c>
       <c r="B127" s="2" t="inlineStr">
         <is>
-          <t>응답</t>
+          <t>요청</t>
         </is>
       </c>
       <c r="C127" s="2" t="inlineStr">
         <is>
-          <t>data.table.rows</t>
+          <t>Header Authorization</t>
         </is>
       </c>
       <c r="D127" s="2" t="inlineStr">
         <is>
-          <t>String[][]</t>
+          <t>String</t>
         </is>
       </c>
       <c r="E127" s="2" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="F127" s="2" t="inlineStr">
         <is>
-          <t>표 행</t>
+          <t>Bearer {JWT}. fetch 스트림으로 보냄(EventSource는 헤더를 못 붙이고, 토큰을 URL에 넣지 않음)</t>
         </is>
       </c>
       <c r="G127" s="2" t="inlineStr">
         <is>
-          <t>[["영업이익","...","..."]]</t>
+          <t>Bearer eyJ...</t>
         </is>
       </c>
     </row>
     <row r="128">
       <c r="A128" s="2" t="inlineStr">
         <is>
-          <t>I-01</t>
+          <t>E-15</t>
         </is>
       </c>
       <c r="B128" s="2" t="inlineStr">
@@ -9046,34 +9159,34 @@
       </c>
       <c r="C128" s="2" t="inlineStr">
         <is>
-          <t>data.table.note</t>
+          <t>event: notification</t>
         </is>
       </c>
       <c r="D128" s="2" t="inlineStr">
         <is>
-          <t>String</t>
+          <t>JSON</t>
         </is>
       </c>
       <c r="E128" s="2" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="F128" s="2" t="inlineStr">
         <is>
-          <t>재무제표 기준(연결/별도)·미공시 표시</t>
+          <t>알림 한 건. data는 E-14 items[] 한 개와 같은 모양</t>
         </is>
       </c>
       <c r="G128" s="2" t="inlineStr">
         <is>
-          <t>연결 기준</t>
+          <t>{"notificationId":503,"direction":"RECEIVED",...}</t>
         </is>
       </c>
     </row>
     <row r="129">
       <c r="A129" s="2" t="inlineStr">
         <is>
-          <t>I-01</t>
+          <t>E-15</t>
         </is>
       </c>
       <c r="B129" s="2" t="inlineStr">
@@ -9083,7 +9196,7 @@
       </c>
       <c r="C129" s="2" t="inlineStr">
         <is>
-          <t>data.detailId</t>
+          <t>: ping</t>
         </is>
       </c>
       <c r="D129" s="2" t="inlineStr">
@@ -9093,24 +9206,24 @@
       </c>
       <c r="E129" s="2" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="F129" s="2" t="inlineStr">
         <is>
-          <t>상세 보기 ID(분석 답변일 때)</t>
+          <t>하트비트 주석 줄. nginx 읽기 제한보다 짧은 간격으로 보내 연결 유지</t>
         </is>
       </c>
       <c r="G129" s="2" t="inlineStr">
         <is>
-          <t>dt_91c2...</t>
+          <t>: ping</t>
         </is>
       </c>
     </row>
     <row r="130">
       <c r="A130" s="2" t="inlineStr">
         <is>
-          <t>I-01</t>
+          <t>E-15</t>
         </is>
       </c>
       <c r="B130" s="2" t="inlineStr">
@@ -9127,7 +9240,7 @@
       <c r="E130" s="2" t="inlineStr"/>
       <c r="F130" s="2" t="inlineStr">
         <is>
-          <t>JWT 없음·만료·위조, 로그인 실패</t>
+          <t>JWT 없음·만료·위조 — 스트림을 열기 전에 401</t>
         </is>
       </c>
       <c r="G130" s="2" t="inlineStr"/>
@@ -9135,7 +9248,7 @@
     <row r="131">
       <c r="A131" s="2" t="inlineStr">
         <is>
-          <t>I-02</t>
+          <t>I-01</t>
         </is>
       </c>
       <c r="B131" s="2" t="inlineStr">
@@ -9172,7 +9285,7 @@
     <row r="132">
       <c r="A132" s="2" t="inlineStr">
         <is>
-          <t>I-02</t>
+          <t>I-01</t>
         </is>
       </c>
       <c r="B132" s="2" t="inlineStr">
@@ -9182,7 +9295,7 @@
       </c>
       <c r="C132" s="2" t="inlineStr">
         <is>
-          <t>Path detailId</t>
+          <t>threadId</t>
         </is>
       </c>
       <c r="D132" s="2" t="inlineStr">
@@ -9197,29 +9310,29 @@
       </c>
       <c r="F132" s="2" t="inlineStr">
         <is>
-          <t>상세 보기 ID</t>
+          <t>대화 ID(체크포인터 키)</t>
         </is>
       </c>
       <c r="G132" s="2" t="inlineStr">
         <is>
-          <t>dt_91c2...</t>
+          <t>th_5b21...</t>
         </is>
       </c>
     </row>
     <row r="133">
       <c r="A133" s="2" t="inlineStr">
         <is>
-          <t>I-02</t>
+          <t>I-01</t>
         </is>
       </c>
       <c r="B133" s="2" t="inlineStr">
         <is>
-          <t>응답</t>
+          <t>요청</t>
         </is>
       </c>
       <c r="C133" s="2" t="inlineStr">
         <is>
-          <t>data.report</t>
+          <t>message</t>
         </is>
       </c>
       <c r="D133" s="2" t="inlineStr">
@@ -9234,19 +9347,19 @@
       </c>
       <c r="F133" s="2" t="inlineStr">
         <is>
-          <t>상세 보고서 본문</t>
+          <t>사용자 메시지</t>
         </is>
       </c>
       <c r="G133" s="2" t="inlineStr">
         <is>
-          <t>...</t>
+          <t>엄마한테 1만원 보내줘</t>
         </is>
       </c>
     </row>
     <row r="134">
       <c r="A134" s="2" t="inlineStr">
         <is>
-          <t>I-02</t>
+          <t>I-01</t>
         </is>
       </c>
       <c r="B134" s="2" t="inlineStr">
@@ -9256,34 +9369,34 @@
       </c>
       <c r="C134" s="2" t="inlineStr">
         <is>
-          <t>data.table.columns</t>
+          <t>data.reply</t>
         </is>
       </c>
       <c r="D134" s="2" t="inlineStr">
         <is>
-          <t>String[]</t>
+          <t>String</t>
         </is>
       </c>
       <c r="E134" s="2" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="F134" s="2" t="inlineStr">
         <is>
-          <t>표 머리글</t>
+          <t>요약 답변. 가드에 걸리면 고정 문장</t>
         </is>
       </c>
       <c r="G134" s="2" t="inlineStr">
         <is>
-          <t>["항목", ...]</t>
+          <t>삼성전자 2분기 영업이익은 ...</t>
         </is>
       </c>
     </row>
     <row r="135">
       <c r="A135" s="2" t="inlineStr">
         <is>
-          <t>I-02</t>
+          <t>I-01</t>
         </is>
       </c>
       <c r="B135" s="2" t="inlineStr">
@@ -9293,34 +9406,34 @@
       </c>
       <c r="C135" s="2" t="inlineStr">
         <is>
-          <t>data.table.rows</t>
+          <t>data.guard</t>
         </is>
       </c>
       <c r="D135" s="2" t="inlineStr">
         <is>
-          <t>String[][]</t>
+          <t>String</t>
         </is>
       </c>
       <c r="E135" s="2" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="F135" s="2" t="inlineStr">
         <is>
-          <t>표 행</t>
+          <t>판정 코드: PASS / INJECTION / NUMBER_UNVERIFIED / ADVICE / PROMPT_LEAK</t>
         </is>
       </c>
       <c r="G135" s="2" t="inlineStr">
         <is>
-          <t>[[...]]</t>
+          <t>PASS</t>
         </is>
       </c>
     </row>
     <row r="136">
       <c r="A136" s="2" t="inlineStr">
         <is>
-          <t>I-02</t>
+          <t>I-01</t>
         </is>
       </c>
       <c r="B136" s="2" t="inlineStr">
@@ -9330,7 +9443,7 @@
       </c>
       <c r="C136" s="2" t="inlineStr">
         <is>
-          <t>data.table.note</t>
+          <t>data.transferCard.requestId</t>
         </is>
       </c>
       <c r="D136" s="2" t="inlineStr">
@@ -9345,79 +9458,103 @@
       </c>
       <c r="F136" s="2" t="inlineStr">
         <is>
-          <t>재무제표 기준·미공시 표시</t>
+          <t>송금 요청ID(1회용)</t>
         </is>
       </c>
       <c r="G136" s="2" t="inlineStr">
         <is>
-          <t>연결 기준</t>
+          <t>tr_7f3a...</t>
         </is>
       </c>
     </row>
     <row r="137">
       <c r="A137" s="2" t="inlineStr">
         <is>
-          <t>I-02</t>
+          <t>I-01</t>
         </is>
       </c>
       <c r="B137" s="2" t="inlineStr">
         <is>
-          <t>에러</t>
+          <t>응답</t>
         </is>
       </c>
       <c r="C137" s="2" t="inlineStr">
         <is>
-          <t>AUTH_INVALID</t>
-        </is>
-      </c>
-      <c r="D137" s="2" t="inlineStr"/>
-      <c r="E137" s="2" t="inlineStr"/>
+          <t>data.transferCard.recipientName</t>
+        </is>
+      </c>
+      <c r="D137" s="2" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="E137" s="2" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="F137" s="2" t="inlineStr">
         <is>
-          <t>JWT 없음·만료·위조, 로그인 실패</t>
-        </is>
-      </c>
-      <c r="G137" s="2" t="inlineStr"/>
+          <t>수취인 이름</t>
+        </is>
+      </c>
+      <c r="G137" s="2" t="inlineStr">
+        <is>
+          <t>김영희</t>
+        </is>
+      </c>
     </row>
     <row r="138">
       <c r="A138" s="2" t="inlineStr">
         <is>
-          <t>I-02</t>
+          <t>I-01</t>
         </is>
       </c>
       <c r="B138" s="2" t="inlineStr">
         <is>
-          <t>에러</t>
+          <t>응답</t>
         </is>
       </c>
       <c r="C138" s="2" t="inlineStr">
         <is>
-          <t>DETAIL_NOT_FOUND</t>
-        </is>
-      </c>
-      <c r="D138" s="2" t="inlineStr"/>
-      <c r="E138" s="2" t="inlineStr"/>
+          <t>data.transferCard.recipientAccountNumber</t>
+        </is>
+      </c>
+      <c r="D138" s="2" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="E138" s="2" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="F138" s="2" t="inlineStr">
         <is>
-          <t>상세 보기 대상 없음(또는 남의 것)</t>
-        </is>
-      </c>
-      <c r="G138" s="2" t="inlineStr"/>
+          <t>수취인 계좌</t>
+        </is>
+      </c>
+      <c r="G138" s="2" t="inlineStr">
+        <is>
+          <t>123456789012</t>
+        </is>
+      </c>
     </row>
     <row r="139">
       <c r="A139" s="2" t="inlineStr">
         <is>
-          <t>I-03</t>
+          <t>I-01</t>
         </is>
       </c>
       <c r="B139" s="2" t="inlineStr">
         <is>
-          <t>요청</t>
+          <t>응답</t>
         </is>
       </c>
       <c r="C139" s="2" t="inlineStr">
         <is>
-          <t>Header Authorization</t>
+          <t>data.transferCard.fromAccountNumber</t>
         </is>
       </c>
       <c r="D139" s="2" t="inlineStr">
@@ -9427,39 +9564,39 @@
       </c>
       <c r="E139" s="2" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="F139" s="2" t="inlineStr">
         <is>
-          <t>Bearer {JWT}</t>
+          <t>출금 계좌(대표 계좌)</t>
         </is>
       </c>
       <c r="G139" s="2" t="inlineStr">
         <is>
-          <t>Bearer eyJ...</t>
+          <t>987654321098</t>
         </is>
       </c>
     </row>
     <row r="140">
       <c r="A140" s="2" t="inlineStr">
         <is>
-          <t>I-03</t>
+          <t>I-01</t>
         </is>
       </c>
       <c r="B140" s="2" t="inlineStr">
         <is>
-          <t>요청</t>
+          <t>응답</t>
         </is>
       </c>
       <c r="C140" s="2" t="inlineStr">
         <is>
-          <t>recipientAccountNumber</t>
+          <t>data.transferCard.amount</t>
         </is>
       </c>
       <c r="D140" s="2" t="inlineStr">
         <is>
-          <t>String</t>
+          <t>Long</t>
         </is>
       </c>
       <c r="E140" s="2" t="inlineStr">
@@ -9469,29 +9606,29 @@
       </c>
       <c r="F140" s="2" t="inlineStr">
         <is>
-          <t>수취인 계좌번호(alias와 둘 중 하나)</t>
+          <t>금액(원)</t>
         </is>
       </c>
       <c r="G140" s="2" t="inlineStr">
         <is>
-          <t>123456789012</t>
+          <t>10000</t>
         </is>
       </c>
     </row>
     <row r="141">
       <c r="A141" s="2" t="inlineStr">
         <is>
-          <t>I-03</t>
+          <t>I-01</t>
         </is>
       </c>
       <c r="B141" s="2" t="inlineStr">
         <is>
-          <t>요청</t>
+          <t>응답</t>
         </is>
       </c>
       <c r="C141" s="2" t="inlineStr">
         <is>
-          <t>alias</t>
+          <t>data.transferCard.expiresAt</t>
         </is>
       </c>
       <c r="D141" s="2" t="inlineStr">
@@ -9506,56 +9643,56 @@
       </c>
       <c r="F141" s="2" t="inlineStr">
         <is>
-          <t>별칭(recipientAccountNumber와 둘 중 하나)</t>
+          <t>만료 시각(생성 + 5분, ISO-8601)</t>
         </is>
       </c>
       <c r="G141" s="2" t="inlineStr">
         <is>
-          <t>엄마</t>
+          <t>2026-09-27T10:05:00+09:00</t>
         </is>
       </c>
     </row>
     <row r="142">
       <c r="A142" s="2" t="inlineStr">
         <is>
-          <t>I-03</t>
+          <t>I-01</t>
         </is>
       </c>
       <c r="B142" s="2" t="inlineStr">
         <is>
-          <t>요청</t>
+          <t>응답</t>
         </is>
       </c>
       <c r="C142" s="2" t="inlineStr">
         <is>
-          <t>amount</t>
+          <t>data.table.columns</t>
         </is>
       </c>
       <c r="D142" s="2" t="inlineStr">
         <is>
-          <t>Long</t>
+          <t>String[]</t>
         </is>
       </c>
       <c r="E142" s="2" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="F142" s="2" t="inlineStr">
         <is>
-          <t>금액(원)</t>
+          <t>표 머리글</t>
         </is>
       </c>
       <c r="G142" s="2" t="inlineStr">
         <is>
-          <t>10000</t>
+          <t>["항목","삼성전자","SK하이닉스"]</t>
         </is>
       </c>
     </row>
     <row r="143">
       <c r="A143" s="2" t="inlineStr">
         <is>
-          <t>I-03</t>
+          <t>I-01</t>
         </is>
       </c>
       <c r="B143" s="2" t="inlineStr">
@@ -9565,34 +9702,34 @@
       </c>
       <c r="C143" s="2" t="inlineStr">
         <is>
-          <t>data.requestId</t>
+          <t>data.table.rows</t>
         </is>
       </c>
       <c r="D143" s="2" t="inlineStr">
         <is>
-          <t>String</t>
+          <t>String[][]</t>
         </is>
       </c>
       <c r="E143" s="2" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="F143" s="2" t="inlineStr">
         <is>
-          <t>송금 요청ID(1회용)</t>
+          <t>표 행</t>
         </is>
       </c>
       <c r="G143" s="2" t="inlineStr">
         <is>
-          <t>tr_7f3a...</t>
+          <t>[["영업이익","...","..."]]</t>
         </is>
       </c>
     </row>
     <row r="144">
       <c r="A144" s="2" t="inlineStr">
         <is>
-          <t>I-03</t>
+          <t>I-01</t>
         </is>
       </c>
       <c r="B144" s="2" t="inlineStr">
@@ -9602,7 +9739,7 @@
       </c>
       <c r="C144" s="2" t="inlineStr">
         <is>
-          <t>data.recipientName</t>
+          <t>data.table.note</t>
         </is>
       </c>
       <c r="D144" s="2" t="inlineStr">
@@ -9612,24 +9749,24 @@
       </c>
       <c r="E144" s="2" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="F144" s="2" t="inlineStr">
         <is>
-          <t>수취인 이름</t>
+          <t>재무제표 기준(연결/별도)·미공시 표시</t>
         </is>
       </c>
       <c r="G144" s="2" t="inlineStr">
         <is>
-          <t>김영희</t>
+          <t>연결 기준</t>
         </is>
       </c>
     </row>
     <row r="145">
       <c r="A145" s="2" t="inlineStr">
         <is>
-          <t>I-03</t>
+          <t>I-01</t>
         </is>
       </c>
       <c r="B145" s="2" t="inlineStr">
@@ -9639,7 +9776,7 @@
       </c>
       <c r="C145" s="2" t="inlineStr">
         <is>
-          <t>data.recipientAccountNumber</t>
+          <t>data.detailId</t>
         </is>
       </c>
       <c r="D145" s="2" t="inlineStr">
@@ -9649,76 +9786,64 @@
       </c>
       <c r="E145" s="2" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="F145" s="2" t="inlineStr">
         <is>
-          <t>수취인 계좌</t>
+          <t>상세 보기 ID(분석 답변일 때)</t>
         </is>
       </c>
       <c r="G145" s="2" t="inlineStr">
         <is>
-          <t>123456789012</t>
+          <t>dt_91c2...</t>
         </is>
       </c>
     </row>
     <row r="146">
       <c r="A146" s="2" t="inlineStr">
         <is>
-          <t>I-03</t>
+          <t>I-01</t>
         </is>
       </c>
       <c r="B146" s="2" t="inlineStr">
         <is>
-          <t>응답</t>
+          <t>에러</t>
         </is>
       </c>
       <c r="C146" s="2" t="inlineStr">
         <is>
-          <t>data.fromAccountNumber</t>
-        </is>
-      </c>
-      <c r="D146" s="2" t="inlineStr">
-        <is>
-          <t>String</t>
-        </is>
-      </c>
-      <c r="E146" s="2" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+          <t>AUTH_INVALID</t>
+        </is>
+      </c>
+      <c r="D146" s="2" t="inlineStr"/>
+      <c r="E146" s="2" t="inlineStr"/>
       <c r="F146" s="2" t="inlineStr">
         <is>
-          <t>출금 계좌(대표 계좌)</t>
-        </is>
-      </c>
-      <c r="G146" s="2" t="inlineStr">
-        <is>
-          <t>987654321098</t>
-        </is>
-      </c>
+          <t>JWT 없음·만료·위조, 로그인 실패</t>
+        </is>
+      </c>
+      <c r="G146" s="2" t="inlineStr"/>
     </row>
     <row r="147">
       <c r="A147" s="2" t="inlineStr">
         <is>
-          <t>I-03</t>
+          <t>I-02</t>
         </is>
       </c>
       <c r="B147" s="2" t="inlineStr">
         <is>
-          <t>응답</t>
+          <t>요청</t>
         </is>
       </c>
       <c r="C147" s="2" t="inlineStr">
         <is>
-          <t>data.amount</t>
+          <t>Header Authorization</t>
         </is>
       </c>
       <c r="D147" s="2" t="inlineStr">
         <is>
-          <t>Long</t>
+          <t>String</t>
         </is>
       </c>
       <c r="E147" s="2" t="inlineStr">
@@ -9728,29 +9853,29 @@
       </c>
       <c r="F147" s="2" t="inlineStr">
         <is>
-          <t>금액(원)</t>
+          <t>Bearer {JWT}</t>
         </is>
       </c>
       <c r="G147" s="2" t="inlineStr">
         <is>
-          <t>10000</t>
+          <t>Bearer eyJ...</t>
         </is>
       </c>
     </row>
     <row r="148">
       <c r="A148" s="2" t="inlineStr">
         <is>
-          <t>I-03</t>
+          <t>I-02</t>
         </is>
       </c>
       <c r="B148" s="2" t="inlineStr">
         <is>
-          <t>응답</t>
+          <t>요청</t>
         </is>
       </c>
       <c r="C148" s="2" t="inlineStr">
         <is>
-          <t>data.expiresAt</t>
+          <t>Path detailId</t>
         </is>
       </c>
       <c r="D148" s="2" t="inlineStr">
@@ -9765,104 +9890,140 @@
       </c>
       <c r="F148" s="2" t="inlineStr">
         <is>
-          <t>만료 시각(생성 + 5분, ISO-8601)</t>
+          <t>상세 보기 ID</t>
         </is>
       </c>
       <c r="G148" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T10:05:00+09:00</t>
+          <t>dt_91c2...</t>
         </is>
       </c>
     </row>
     <row r="149">
       <c r="A149" s="2" t="inlineStr">
         <is>
-          <t>I-03</t>
+          <t>I-02</t>
         </is>
       </c>
       <c r="B149" s="2" t="inlineStr">
         <is>
-          <t>에러</t>
+          <t>응답</t>
         </is>
       </c>
       <c r="C149" s="2" t="inlineStr">
         <is>
-          <t>AUTH_INVALID</t>
-        </is>
-      </c>
-      <c r="D149" s="2" t="inlineStr"/>
-      <c r="E149" s="2" t="inlineStr"/>
+          <t>data.report</t>
+        </is>
+      </c>
+      <c r="D149" s="2" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="E149" s="2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="F149" s="2" t="inlineStr">
         <is>
-          <t>JWT 없음·만료·위조, 로그인 실패</t>
-        </is>
-      </c>
-      <c r="G149" s="2" t="inlineStr"/>
+          <t>상세 보고서 본문</t>
+        </is>
+      </c>
+      <c r="G149" s="2" t="inlineStr">
+        <is>
+          <t>...</t>
+        </is>
+      </c>
     </row>
     <row r="150">
       <c r="A150" s="2" t="inlineStr">
         <is>
-          <t>I-03</t>
+          <t>I-02</t>
         </is>
       </c>
       <c r="B150" s="2" t="inlineStr">
         <is>
-          <t>에러</t>
+          <t>응답</t>
         </is>
       </c>
       <c r="C150" s="2" t="inlineStr">
         <is>
-          <t>ALIAS_NOT_FOUND</t>
-        </is>
-      </c>
-      <c r="D150" s="2" t="inlineStr"/>
-      <c r="E150" s="2" t="inlineStr"/>
+          <t>data.table.columns</t>
+        </is>
+      </c>
+      <c r="D150" s="2" t="inlineStr">
+        <is>
+          <t>String[]</t>
+        </is>
+      </c>
+      <c r="E150" s="2" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="F150" s="2" t="inlineStr">
         <is>
-          <t>등록되지 않은 별칭</t>
-        </is>
-      </c>
-      <c r="G150" s="2" t="inlineStr"/>
+          <t>표 머리글</t>
+        </is>
+      </c>
+      <c r="G150" s="2" t="inlineStr">
+        <is>
+          <t>["항목", ...]</t>
+        </is>
+      </c>
     </row>
     <row r="151">
       <c r="A151" s="2" t="inlineStr">
         <is>
-          <t>I-03</t>
+          <t>I-02</t>
         </is>
       </c>
       <c r="B151" s="2" t="inlineStr">
         <is>
-          <t>에러</t>
+          <t>응답</t>
         </is>
       </c>
       <c r="C151" s="2" t="inlineStr">
         <is>
-          <t>ACCOUNT_NOT_FOUND</t>
-        </is>
-      </c>
-      <c r="D151" s="2" t="inlineStr"/>
-      <c r="E151" s="2" t="inlineStr"/>
+          <t>data.table.rows</t>
+        </is>
+      </c>
+      <c r="D151" s="2" t="inlineStr">
+        <is>
+          <t>String[][]</t>
+        </is>
+      </c>
+      <c r="E151" s="2" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="F151" s="2" t="inlineStr">
         <is>
-          <t>계좌 없음</t>
-        </is>
-      </c>
-      <c r="G151" s="2" t="inlineStr"/>
+          <t>표 행</t>
+        </is>
+      </c>
+      <c r="G151" s="2" t="inlineStr">
+        <is>
+          <t>[[...]]</t>
+        </is>
+      </c>
     </row>
     <row r="152">
       <c r="A152" s="2" t="inlineStr">
         <is>
-          <t>I-04</t>
+          <t>I-02</t>
         </is>
       </c>
       <c r="B152" s="2" t="inlineStr">
         <is>
-          <t>요청</t>
+          <t>응답</t>
         </is>
       </c>
       <c r="C152" s="2" t="inlineStr">
         <is>
-          <t>Header Authorization</t>
+          <t>data.table.note</t>
         </is>
       </c>
       <c r="D152" s="2" t="inlineStr">
@@ -9872,98 +10033,74 @@
       </c>
       <c r="E152" s="2" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="F152" s="2" t="inlineStr">
         <is>
-          <t>Bearer {JWT}</t>
+          <t>재무제표 기준·미공시 표시</t>
         </is>
       </c>
       <c r="G152" s="2" t="inlineStr">
         <is>
-          <t>Bearer eyJ...</t>
+          <t>연결 기준</t>
         </is>
       </c>
     </row>
     <row r="153">
       <c r="A153" s="2" t="inlineStr">
         <is>
-          <t>I-04</t>
+          <t>I-02</t>
         </is>
       </c>
       <c r="B153" s="2" t="inlineStr">
         <is>
-          <t>요청</t>
+          <t>에러</t>
         </is>
       </c>
       <c r="C153" s="2" t="inlineStr">
         <is>
-          <t>Query from</t>
-        </is>
-      </c>
-      <c r="D153" s="2" t="inlineStr">
-        <is>
-          <t>String</t>
-        </is>
-      </c>
-      <c r="E153" s="2" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+          <t>AUTH_INVALID</t>
+        </is>
+      </c>
+      <c r="D153" s="2" t="inlineStr"/>
+      <c r="E153" s="2" t="inlineStr"/>
       <c r="F153" s="2" t="inlineStr">
         <is>
-          <t>시작일(yyyy-MM-dd)</t>
-        </is>
-      </c>
-      <c r="G153" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-01</t>
-        </is>
-      </c>
+          <t>JWT 없음·만료·위조, 로그인 실패</t>
+        </is>
+      </c>
+      <c r="G153" s="2" t="inlineStr"/>
     </row>
     <row r="154">
       <c r="A154" s="2" t="inlineStr">
         <is>
-          <t>I-04</t>
+          <t>I-02</t>
         </is>
       </c>
       <c r="B154" s="2" t="inlineStr">
         <is>
-          <t>요청</t>
+          <t>에러</t>
         </is>
       </c>
       <c r="C154" s="2" t="inlineStr">
         <is>
-          <t>Query to</t>
-        </is>
-      </c>
-      <c r="D154" s="2" t="inlineStr">
-        <is>
-          <t>String</t>
-        </is>
-      </c>
-      <c r="E154" s="2" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+          <t>DETAIL_NOT_FOUND</t>
+        </is>
+      </c>
+      <c r="D154" s="2" t="inlineStr"/>
+      <c r="E154" s="2" t="inlineStr"/>
       <c r="F154" s="2" t="inlineStr">
         <is>
-          <t>종료일(yyyy-MM-dd)</t>
-        </is>
-      </c>
-      <c r="G154" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-30</t>
-        </is>
-      </c>
+          <t>상세 보기 대상 없음(또는 남의 것)</t>
+        </is>
+      </c>
+      <c r="G154" s="2" t="inlineStr"/>
     </row>
     <row r="155">
       <c r="A155" s="2" t="inlineStr">
         <is>
-          <t>I-04</t>
+          <t>I-03</t>
         </is>
       </c>
       <c r="B155" s="2" t="inlineStr">
@@ -9973,30 +10110,34 @@
       </c>
       <c r="C155" s="2" t="inlineStr">
         <is>
-          <t>Query cursor</t>
+          <t>Header Authorization</t>
         </is>
       </c>
       <c r="D155" s="2" t="inlineStr">
         <is>
-          <t>Long</t>
+          <t>String</t>
         </is>
       </c>
       <c r="E155" s="2" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="F155" s="2" t="inlineStr">
         <is>
-          <t>E-09와 같은 커서 규칙</t>
-        </is>
-      </c>
-      <c r="G155" s="2" t="inlineStr"/>
+          <t>Bearer {JWT}</t>
+        </is>
+      </c>
+      <c r="G155" s="2" t="inlineStr">
+        <is>
+          <t>Bearer eyJ...</t>
+        </is>
+      </c>
     </row>
     <row r="156">
       <c r="A156" s="2" t="inlineStr">
         <is>
-          <t>I-04</t>
+          <t>I-03</t>
         </is>
       </c>
       <c r="B156" s="2" t="inlineStr">
@@ -10006,12 +10147,12 @@
       </c>
       <c r="C156" s="2" t="inlineStr">
         <is>
-          <t>Query size</t>
+          <t>recipientAccountNumber</t>
         </is>
       </c>
       <c r="D156" s="2" t="inlineStr">
         <is>
-          <t>Integer</t>
+          <t>String</t>
         </is>
       </c>
       <c r="E156" s="2" t="inlineStr">
@@ -10021,66 +10162,66 @@
       </c>
       <c r="F156" s="2" t="inlineStr">
         <is>
-          <t>기본 20</t>
+          <t>수취인 계좌번호(alias와 둘 중 하나)</t>
         </is>
       </c>
       <c r="G156" s="2" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>123456789012</t>
         </is>
       </c>
     </row>
     <row r="157">
       <c r="A157" s="2" t="inlineStr">
         <is>
-          <t>I-04</t>
+          <t>I-03</t>
         </is>
       </c>
       <c r="B157" s="2" t="inlineStr">
         <is>
-          <t>응답</t>
+          <t>요청</t>
         </is>
       </c>
       <c r="C157" s="2" t="inlineStr">
         <is>
-          <t>data.sentTotal</t>
+          <t>alias</t>
         </is>
       </c>
       <c r="D157" s="2" t="inlineStr">
         <is>
-          <t>Long</t>
+          <t>String</t>
         </is>
       </c>
       <c r="E157" s="2" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="F157" s="2" t="inlineStr">
         <is>
-          <t>기간 내 보낸 합계(원, Spring 계산)</t>
+          <t>별칭(recipientAccountNumber와 둘 중 하나)</t>
         </is>
       </c>
       <c r="G157" s="2" t="inlineStr">
         <is>
-          <t>230000</t>
+          <t>엄마</t>
         </is>
       </c>
     </row>
     <row r="158">
       <c r="A158" s="2" t="inlineStr">
         <is>
-          <t>I-04</t>
+          <t>I-03</t>
         </is>
       </c>
       <c r="B158" s="2" t="inlineStr">
         <is>
-          <t>응답</t>
+          <t>요청</t>
         </is>
       </c>
       <c r="C158" s="2" t="inlineStr">
         <is>
-          <t>data.receivedTotal</t>
+          <t>amount</t>
         </is>
       </c>
       <c r="D158" s="2" t="inlineStr">
@@ -10095,19 +10236,19 @@
       </c>
       <c r="F158" s="2" t="inlineStr">
         <is>
-          <t>기간 내 받은 합계(원, Spring 계산)</t>
+          <t>금액(원)</t>
         </is>
       </c>
       <c r="G158" s="2" t="inlineStr">
         <is>
-          <t>50000</t>
+          <t>10000</t>
         </is>
       </c>
     </row>
     <row r="159">
       <c r="A159" s="2" t="inlineStr">
         <is>
-          <t>I-04</t>
+          <t>I-03</t>
         </is>
       </c>
       <c r="B159" s="2" t="inlineStr">
@@ -10117,12 +10258,12 @@
       </c>
       <c r="C159" s="2" t="inlineStr">
         <is>
-          <t>data.count</t>
+          <t>data.requestId</t>
         </is>
       </c>
       <c r="D159" s="2" t="inlineStr">
         <is>
-          <t>Integer</t>
+          <t>String</t>
         </is>
       </c>
       <c r="E159" s="2" t="inlineStr">
@@ -10132,19 +10273,19 @@
       </c>
       <c r="F159" s="2" t="inlineStr">
         <is>
-          <t>기간 내 건수</t>
+          <t>송금 요청ID(1회용)</t>
         </is>
       </c>
       <c r="G159" s="2" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>tr_7f3a...</t>
         </is>
       </c>
     </row>
     <row r="160">
       <c r="A160" s="2" t="inlineStr">
         <is>
-          <t>I-04</t>
+          <t>I-03</t>
         </is>
       </c>
       <c r="B160" s="2" t="inlineStr">
@@ -10154,12 +10295,12 @@
       </c>
       <c r="C160" s="2" t="inlineStr">
         <is>
-          <t>data.items[].transferId</t>
+          <t>data.recipientName</t>
         </is>
       </c>
       <c r="D160" s="2" t="inlineStr">
         <is>
-          <t>Long</t>
+          <t>String</t>
         </is>
       </c>
       <c r="E160" s="2" t="inlineStr">
@@ -10169,19 +10310,19 @@
       </c>
       <c r="F160" s="2" t="inlineStr">
         <is>
-          <t>송금 ID</t>
+          <t>수취인 이름</t>
         </is>
       </c>
       <c r="G160" s="2" t="inlineStr">
         <is>
-          <t>1024</t>
+          <t>김영희</t>
         </is>
       </c>
     </row>
     <row r="161">
       <c r="A161" s="2" t="inlineStr">
         <is>
-          <t>I-04</t>
+          <t>I-03</t>
         </is>
       </c>
       <c r="B161" s="2" t="inlineStr">
@@ -10191,7 +10332,7 @@
       </c>
       <c r="C161" s="2" t="inlineStr">
         <is>
-          <t>data.items[].direction</t>
+          <t>data.recipientAccountNumber</t>
         </is>
       </c>
       <c r="D161" s="2" t="inlineStr">
@@ -10206,19 +10347,19 @@
       </c>
       <c r="F161" s="2" t="inlineStr">
         <is>
-          <t>SENT / RECEIVED</t>
+          <t>수취인 계좌</t>
         </is>
       </c>
       <c r="G161" s="2" t="inlineStr">
         <is>
-          <t>SENT</t>
+          <t>123456789012</t>
         </is>
       </c>
     </row>
     <row r="162">
       <c r="A162" s="2" t="inlineStr">
         <is>
-          <t>I-04</t>
+          <t>I-03</t>
         </is>
       </c>
       <c r="B162" s="2" t="inlineStr">
@@ -10228,7 +10369,7 @@
       </c>
       <c r="C162" s="2" t="inlineStr">
         <is>
-          <t>data.items[].counterpartName</t>
+          <t>data.fromAccountNumber</t>
         </is>
       </c>
       <c r="D162" s="2" t="inlineStr">
@@ -10243,19 +10384,19 @@
       </c>
       <c r="F162" s="2" t="inlineStr">
         <is>
-          <t>상대 이름</t>
+          <t>출금 계좌(대표 계좌)</t>
         </is>
       </c>
       <c r="G162" s="2" t="inlineStr">
         <is>
-          <t>김영희</t>
+          <t>987654321098</t>
         </is>
       </c>
     </row>
     <row r="163">
       <c r="A163" s="2" t="inlineStr">
         <is>
-          <t>I-04</t>
+          <t>I-03</t>
         </is>
       </c>
       <c r="B163" s="2" t="inlineStr">
@@ -10265,12 +10406,12 @@
       </c>
       <c r="C163" s="2" t="inlineStr">
         <is>
-          <t>data.items[].counterpartAccountNumber</t>
+          <t>data.amount</t>
         </is>
       </c>
       <c r="D163" s="2" t="inlineStr">
         <is>
-          <t>String</t>
+          <t>Long</t>
         </is>
       </c>
       <c r="E163" s="2" t="inlineStr">
@@ -10280,19 +10421,19 @@
       </c>
       <c r="F163" s="2" t="inlineStr">
         <is>
-          <t>상대 계좌</t>
+          <t>금액(원)</t>
         </is>
       </c>
       <c r="G163" s="2" t="inlineStr">
         <is>
-          <t>123456789012</t>
+          <t>10000</t>
         </is>
       </c>
     </row>
     <row r="164">
       <c r="A164" s="2" t="inlineStr">
         <is>
-          <t>I-04</t>
+          <t>I-03</t>
         </is>
       </c>
       <c r="B164" s="2" t="inlineStr">
@@ -10302,12 +10443,12 @@
       </c>
       <c r="C164" s="2" t="inlineStr">
         <is>
-          <t>data.items[].amount</t>
+          <t>data.expiresAt</t>
         </is>
       </c>
       <c r="D164" s="2" t="inlineStr">
         <is>
-          <t>Long</t>
+          <t>String</t>
         </is>
       </c>
       <c r="E164" s="2" t="inlineStr">
@@ -10317,125 +10458,89 @@
       </c>
       <c r="F164" s="2" t="inlineStr">
         <is>
-          <t>금액(원)</t>
+          <t>만료 시각(생성 + 5분, ISO-8601)</t>
         </is>
       </c>
       <c r="G164" s="2" t="inlineStr">
         <is>
-          <t>10000</t>
+          <t>2026-09-27T10:05:00+09:00</t>
         </is>
       </c>
     </row>
     <row r="165">
       <c r="A165" s="2" t="inlineStr">
         <is>
-          <t>I-04</t>
+          <t>I-03</t>
         </is>
       </c>
       <c r="B165" s="2" t="inlineStr">
         <is>
-          <t>응답</t>
+          <t>에러</t>
         </is>
       </c>
       <c r="C165" s="2" t="inlineStr">
         <is>
-          <t>data.items[].createdAt</t>
-        </is>
-      </c>
-      <c r="D165" s="2" t="inlineStr">
-        <is>
-          <t>String</t>
-        </is>
-      </c>
-      <c r="E165" s="2" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+          <t>AUTH_INVALID</t>
+        </is>
+      </c>
+      <c r="D165" s="2" t="inlineStr"/>
+      <c r="E165" s="2" t="inlineStr"/>
       <c r="F165" s="2" t="inlineStr">
         <is>
-          <t>시각(ISO-8601)</t>
-        </is>
-      </c>
-      <c r="G165" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-27T10:01:00+09:00</t>
-        </is>
-      </c>
+          <t>JWT 없음·만료·위조, 로그인 실패</t>
+        </is>
+      </c>
+      <c r="G165" s="2" t="inlineStr"/>
     </row>
     <row r="166">
       <c r="A166" s="2" t="inlineStr">
         <is>
-          <t>I-04</t>
+          <t>I-03</t>
         </is>
       </c>
       <c r="B166" s="2" t="inlineStr">
         <is>
-          <t>응답</t>
+          <t>에러</t>
         </is>
       </c>
       <c r="C166" s="2" t="inlineStr">
         <is>
-          <t>data.nextCursor</t>
-        </is>
-      </c>
-      <c r="D166" s="2" t="inlineStr">
-        <is>
-          <t>Long</t>
-        </is>
-      </c>
-      <c r="E166" s="2" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
+          <t>ALIAS_NOT_FOUND</t>
+        </is>
+      </c>
+      <c r="D166" s="2" t="inlineStr"/>
+      <c r="E166" s="2" t="inlineStr"/>
       <c r="F166" s="2" t="inlineStr">
         <is>
-          <t>다음 요청의 cursor(마지막 transferId). 없으면 null</t>
-        </is>
-      </c>
-      <c r="G166" s="2" t="inlineStr">
-        <is>
-          <t>1005</t>
-        </is>
-      </c>
+          <t>등록되지 않은 별칭</t>
+        </is>
+      </c>
+      <c r="G166" s="2" t="inlineStr"/>
     </row>
     <row r="167">
       <c r="A167" s="2" t="inlineStr">
         <is>
-          <t>I-04</t>
+          <t>I-03</t>
         </is>
       </c>
       <c r="B167" s="2" t="inlineStr">
         <is>
-          <t>응답</t>
+          <t>에러</t>
         </is>
       </c>
       <c r="C167" s="2" t="inlineStr">
         <is>
-          <t>data.hasNext</t>
-        </is>
-      </c>
-      <c r="D167" s="2" t="inlineStr">
-        <is>
-          <t>Boolean</t>
-        </is>
-      </c>
-      <c r="E167" s="2" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+          <t>ACCOUNT_NOT_FOUND</t>
+        </is>
+      </c>
+      <c r="D167" s="2" t="inlineStr"/>
+      <c r="E167" s="2" t="inlineStr"/>
       <c r="F167" s="2" t="inlineStr">
         <is>
-          <t>다음 묶음 존재 여부</t>
-        </is>
-      </c>
-      <c r="G167" s="2" t="inlineStr">
-        <is>
-          <t>true</t>
-        </is>
-      </c>
+          <t>계좌 없음</t>
+        </is>
+      </c>
+      <c r="G167" s="2" t="inlineStr"/>
     </row>
     <row r="168">
       <c r="A168" s="2" t="inlineStr">
@@ -10445,25 +10550,613 @@
       </c>
       <c r="B168" s="2" t="inlineStr">
         <is>
+          <t>요청</t>
+        </is>
+      </c>
+      <c r="C168" s="2" t="inlineStr">
+        <is>
+          <t>Header Authorization</t>
+        </is>
+      </c>
+      <c r="D168" s="2" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="E168" s="2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="F168" s="2" t="inlineStr">
+        <is>
+          <t>Bearer {JWT}</t>
+        </is>
+      </c>
+      <c r="G168" s="2" t="inlineStr">
+        <is>
+          <t>Bearer eyJ...</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" s="2" t="inlineStr">
+        <is>
+          <t>I-04</t>
+        </is>
+      </c>
+      <c r="B169" s="2" t="inlineStr">
+        <is>
+          <t>요청</t>
+        </is>
+      </c>
+      <c r="C169" s="2" t="inlineStr">
+        <is>
+          <t>Query from</t>
+        </is>
+      </c>
+      <c r="D169" s="2" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="E169" s="2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="F169" s="2" t="inlineStr">
+        <is>
+          <t>시작일(yyyy-MM-dd)</t>
+        </is>
+      </c>
+      <c r="G169" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" s="2" t="inlineStr">
+        <is>
+          <t>I-04</t>
+        </is>
+      </c>
+      <c r="B170" s="2" t="inlineStr">
+        <is>
+          <t>요청</t>
+        </is>
+      </c>
+      <c r="C170" s="2" t="inlineStr">
+        <is>
+          <t>Query to</t>
+        </is>
+      </c>
+      <c r="D170" s="2" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="E170" s="2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="F170" s="2" t="inlineStr">
+        <is>
+          <t>종료일(yyyy-MM-dd)</t>
+        </is>
+      </c>
+      <c r="G170" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" s="2" t="inlineStr">
+        <is>
+          <t>I-04</t>
+        </is>
+      </c>
+      <c r="B171" s="2" t="inlineStr">
+        <is>
+          <t>요청</t>
+        </is>
+      </c>
+      <c r="C171" s="2" t="inlineStr">
+        <is>
+          <t>Query cursor</t>
+        </is>
+      </c>
+      <c r="D171" s="2" t="inlineStr">
+        <is>
+          <t>Long</t>
+        </is>
+      </c>
+      <c r="E171" s="2" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="F171" s="2" t="inlineStr">
+        <is>
+          <t>E-09와 같은 커서 규칙</t>
+        </is>
+      </c>
+      <c r="G171" s="2" t="inlineStr"/>
+    </row>
+    <row r="172">
+      <c r="A172" s="2" t="inlineStr">
+        <is>
+          <t>I-04</t>
+        </is>
+      </c>
+      <c r="B172" s="2" t="inlineStr">
+        <is>
+          <t>요청</t>
+        </is>
+      </c>
+      <c r="C172" s="2" t="inlineStr">
+        <is>
+          <t>Query size</t>
+        </is>
+      </c>
+      <c r="D172" s="2" t="inlineStr">
+        <is>
+          <t>Integer</t>
+        </is>
+      </c>
+      <c r="E172" s="2" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="F172" s="2" t="inlineStr">
+        <is>
+          <t>기본 20</t>
+        </is>
+      </c>
+      <c r="G172" s="2" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" s="2" t="inlineStr">
+        <is>
+          <t>I-04</t>
+        </is>
+      </c>
+      <c r="B173" s="2" t="inlineStr">
+        <is>
+          <t>응답</t>
+        </is>
+      </c>
+      <c r="C173" s="2" t="inlineStr">
+        <is>
+          <t>data.sentTotal</t>
+        </is>
+      </c>
+      <c r="D173" s="2" t="inlineStr">
+        <is>
+          <t>Long</t>
+        </is>
+      </c>
+      <c r="E173" s="2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="F173" s="2" t="inlineStr">
+        <is>
+          <t>기간 내 보낸 합계(원, Spring 계산)</t>
+        </is>
+      </c>
+      <c r="G173" s="2" t="inlineStr">
+        <is>
+          <t>230000</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" s="2" t="inlineStr">
+        <is>
+          <t>I-04</t>
+        </is>
+      </c>
+      <c r="B174" s="2" t="inlineStr">
+        <is>
+          <t>응답</t>
+        </is>
+      </c>
+      <c r="C174" s="2" t="inlineStr">
+        <is>
+          <t>data.receivedTotal</t>
+        </is>
+      </c>
+      <c r="D174" s="2" t="inlineStr">
+        <is>
+          <t>Long</t>
+        </is>
+      </c>
+      <c r="E174" s="2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="F174" s="2" t="inlineStr">
+        <is>
+          <t>기간 내 받은 합계(원, Spring 계산)</t>
+        </is>
+      </c>
+      <c r="G174" s="2" t="inlineStr">
+        <is>
+          <t>50000</t>
+        </is>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" s="2" t="inlineStr">
+        <is>
+          <t>I-04</t>
+        </is>
+      </c>
+      <c r="B175" s="2" t="inlineStr">
+        <is>
+          <t>응답</t>
+        </is>
+      </c>
+      <c r="C175" s="2" t="inlineStr">
+        <is>
+          <t>data.count</t>
+        </is>
+      </c>
+      <c r="D175" s="2" t="inlineStr">
+        <is>
+          <t>Integer</t>
+        </is>
+      </c>
+      <c r="E175" s="2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="F175" s="2" t="inlineStr">
+        <is>
+          <t>기간 내 건수</t>
+        </is>
+      </c>
+      <c r="G175" s="2" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" s="2" t="inlineStr">
+        <is>
+          <t>I-04</t>
+        </is>
+      </c>
+      <c r="B176" s="2" t="inlineStr">
+        <is>
+          <t>응답</t>
+        </is>
+      </c>
+      <c r="C176" s="2" t="inlineStr">
+        <is>
+          <t>data.items[].transferId</t>
+        </is>
+      </c>
+      <c r="D176" s="2" t="inlineStr">
+        <is>
+          <t>Long</t>
+        </is>
+      </c>
+      <c r="E176" s="2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="F176" s="2" t="inlineStr">
+        <is>
+          <t>송금 ID</t>
+        </is>
+      </c>
+      <c r="G176" s="2" t="inlineStr">
+        <is>
+          <t>1024</t>
+        </is>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" s="2" t="inlineStr">
+        <is>
+          <t>I-04</t>
+        </is>
+      </c>
+      <c r="B177" s="2" t="inlineStr">
+        <is>
+          <t>응답</t>
+        </is>
+      </c>
+      <c r="C177" s="2" t="inlineStr">
+        <is>
+          <t>data.items[].direction</t>
+        </is>
+      </c>
+      <c r="D177" s="2" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="E177" s="2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="F177" s="2" t="inlineStr">
+        <is>
+          <t>SENT / RECEIVED</t>
+        </is>
+      </c>
+      <c r="G177" s="2" t="inlineStr">
+        <is>
+          <t>SENT</t>
+        </is>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" s="2" t="inlineStr">
+        <is>
+          <t>I-04</t>
+        </is>
+      </c>
+      <c r="B178" s="2" t="inlineStr">
+        <is>
+          <t>응답</t>
+        </is>
+      </c>
+      <c r="C178" s="2" t="inlineStr">
+        <is>
+          <t>data.items[].counterpartName</t>
+        </is>
+      </c>
+      <c r="D178" s="2" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="E178" s="2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="F178" s="2" t="inlineStr">
+        <is>
+          <t>상대 이름</t>
+        </is>
+      </c>
+      <c r="G178" s="2" t="inlineStr">
+        <is>
+          <t>김영희</t>
+        </is>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" s="2" t="inlineStr">
+        <is>
+          <t>I-04</t>
+        </is>
+      </c>
+      <c r="B179" s="2" t="inlineStr">
+        <is>
+          <t>응답</t>
+        </is>
+      </c>
+      <c r="C179" s="2" t="inlineStr">
+        <is>
+          <t>data.items[].counterpartAccountNumber</t>
+        </is>
+      </c>
+      <c r="D179" s="2" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="E179" s="2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="F179" s="2" t="inlineStr">
+        <is>
+          <t>상대 계좌</t>
+        </is>
+      </c>
+      <c r="G179" s="2" t="inlineStr">
+        <is>
+          <t>123456789012</t>
+        </is>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" s="2" t="inlineStr">
+        <is>
+          <t>I-04</t>
+        </is>
+      </c>
+      <c r="B180" s="2" t="inlineStr">
+        <is>
+          <t>응답</t>
+        </is>
+      </c>
+      <c r="C180" s="2" t="inlineStr">
+        <is>
+          <t>data.items[].amount</t>
+        </is>
+      </c>
+      <c r="D180" s="2" t="inlineStr">
+        <is>
+          <t>Long</t>
+        </is>
+      </c>
+      <c r="E180" s="2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="F180" s="2" t="inlineStr">
+        <is>
+          <t>금액(원)</t>
+        </is>
+      </c>
+      <c r="G180" s="2" t="inlineStr">
+        <is>
+          <t>10000</t>
+        </is>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" s="2" t="inlineStr">
+        <is>
+          <t>I-04</t>
+        </is>
+      </c>
+      <c r="B181" s="2" t="inlineStr">
+        <is>
+          <t>응답</t>
+        </is>
+      </c>
+      <c r="C181" s="2" t="inlineStr">
+        <is>
+          <t>data.items[].createdAt</t>
+        </is>
+      </c>
+      <c r="D181" s="2" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="E181" s="2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="F181" s="2" t="inlineStr">
+        <is>
+          <t>시각(ISO-8601)</t>
+        </is>
+      </c>
+      <c r="G181" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-27T10:01:00+09:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" s="2" t="inlineStr">
+        <is>
+          <t>I-04</t>
+        </is>
+      </c>
+      <c r="B182" s="2" t="inlineStr">
+        <is>
+          <t>응답</t>
+        </is>
+      </c>
+      <c r="C182" s="2" t="inlineStr">
+        <is>
+          <t>data.nextCursor</t>
+        </is>
+      </c>
+      <c r="D182" s="2" t="inlineStr">
+        <is>
+          <t>Long</t>
+        </is>
+      </c>
+      <c r="E182" s="2" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="F182" s="2" t="inlineStr">
+        <is>
+          <t>다음 요청의 cursor(마지막 transferId). 없으면 null</t>
+        </is>
+      </c>
+      <c r="G182" s="2" t="inlineStr">
+        <is>
+          <t>1005</t>
+        </is>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" s="2" t="inlineStr">
+        <is>
+          <t>I-04</t>
+        </is>
+      </c>
+      <c r="B183" s="2" t="inlineStr">
+        <is>
+          <t>응답</t>
+        </is>
+      </c>
+      <c r="C183" s="2" t="inlineStr">
+        <is>
+          <t>data.hasNext</t>
+        </is>
+      </c>
+      <c r="D183" s="2" t="inlineStr">
+        <is>
+          <t>Boolean</t>
+        </is>
+      </c>
+      <c r="E183" s="2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="F183" s="2" t="inlineStr">
+        <is>
+          <t>다음 묶음 존재 여부</t>
+        </is>
+      </c>
+      <c r="G183" s="2" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" s="2" t="inlineStr">
+        <is>
+          <t>I-04</t>
+        </is>
+      </c>
+      <c r="B184" s="2" t="inlineStr">
+        <is>
           <t>에러</t>
         </is>
       </c>
-      <c r="C168" s="2" t="inlineStr">
+      <c r="C184" s="2" t="inlineStr">
         <is>
           <t>AUTH_INVALID</t>
         </is>
       </c>
-      <c r="D168" s="2" t="inlineStr"/>
-      <c r="E168" s="2" t="inlineStr"/>
-      <c r="F168" s="2" t="inlineStr">
+      <c r="D184" s="2" t="inlineStr"/>
+      <c r="E184" s="2" t="inlineStr"/>
+      <c r="F184" s="2" t="inlineStr">
         <is>
           <t>JWT 없음·만료·위조, 로그인 실패</t>
         </is>
       </c>
-      <c r="G168" s="2" t="inlineStr"/>
+      <c r="G184" s="2" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G168"/>
+  <autoFilter ref="A1:G184"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
docs: 도메인·HTTPS(nginx) 구현·검증·한계, 명세(RATE_LIMITED 설명·E-01/E-02 요청 제한·NFR-053 내부 경로 404) (#87)
</commit_message>
<xml_diff>
--- a/docs/smart-spec.xlsx
+++ b/docs/smart-spec.xlsx
@@ -3467,7 +3467,7 @@
       </c>
       <c r="E84" s="2" t="inlineStr">
         <is>
-          <t>도메인을 붙이고 nginx를 유일한 입구로: TLS 종료(Let's Encrypt, 자동 갱신), 80은 443으로 넘김, Spring으로 프록시(X-Forwarded-For·Proto 전달). 공유기는 80·443만 nginx로 넘기고 Spring 8080은 공개 중단(127.0.0.1에만). 타임아웃은 nginx &gt; Spring 읽기 제한(채팅 10초·상세 30초), 알림 스트림(E-15)은 버퍼링 끄고 하트비트 간격보다 길게. 로그인·가입은 IP별 요청 제한(limit_req). 부하 측정 환경은 지금처럼 Spring 직접(기준선 유지)</t>
+          <t>도메인을 붙이고 nginx를 유일한 입구로: TLS 종료(Let's Encrypt, 자동 갱신), 80은 443으로 넘김, Spring으로 프록시(X-Forwarded-For·Proto 전달). 공유기는 80·443만 nginx로 넘기고 Spring 8080은 공개 중단(127.0.0.1에만). 타임아웃은 nginx &gt; Spring 읽기 제한(채팅 10초·상세 30초), 알림 스트림(E-15)은 버퍼링 끄고 하트비트 간격보다 길게. 로그인·가입은 IP별 요청 제한(limit_req). 내부 경로(/internal/**·/actuator/**)는 입구에서 404. 부하 측정 환경은 지금처럼 Spring 직접(기준선 유지)</t>
         </is>
       </c>
       <c r="F84" s="2" t="inlineStr">
@@ -4055,7 +4055,7 @@
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>사용자별 채팅 호출 제한 초과</t>
+          <t>호출 제한 초과 — 채팅은 사용자별(분당 10회), 로그인·가입은 IP별(nginx)</t>
         </is>
       </c>
       <c r="D24" s="9" t="n"/>
@@ -4331,7 +4331,11 @@
           <t>FR-001</t>
         </is>
       </c>
-      <c r="H37" s="2" t="inlineStr"/>
+      <c r="H37" s="2" t="inlineStr">
+        <is>
+          <t>입구(nginx)가 IP별로 제한한다(분당 10회, 연속 5회까지). 넘으면 429 RATE_LIMITED</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -4369,7 +4373,11 @@
           <t>FR-002</t>
         </is>
       </c>
-      <c r="H38" s="2" t="inlineStr"/>
+      <c r="H38" s="2" t="inlineStr">
+        <is>
+          <t>입구(nginx)가 IP별로 제한한다(분당 10회, 연속 5회까지). 넘으면 429 RATE_LIMITED</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">

</xml_diff>